<commit_message>
feat: reporte ventas julio 2026 - SUMIF por vendedor
</commit_message>
<xml_diff>
--- a/EXCEL/Presupuesto Personal.xlsx
+++ b/EXCEL/Presupuesto Personal.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/1d86eecf8daf4f0d/Documents/SQL Server Management Studio 22/Tienda-sqlserver/EXCEL/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="1" documentId="8_{EE053816-48E3-4E91-A6AD-611A9303676C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{EB2B45EC-DFFD-4117-A825-63EE03B4F0B7}"/>
+  <xr:revisionPtr revIDLastSave="2" documentId="8_{EE053816-48E3-4E91-A6AD-611A9303676C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{71C0AE0A-1937-4A33-91DE-38CE252A77EB}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="624" windowWidth="11268" windowHeight="9840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="588" yWindow="336" windowWidth="11760" windowHeight="12240" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Personal-Budget_2026" sheetId="2" r:id="rId1"/>
@@ -32,7 +32,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="201" uniqueCount="152">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="221" uniqueCount="172">
   <si>
     <t xml:space="preserve">Cantidad </t>
   </si>
@@ -424,24 +424,6 @@
     <t>Silla de escritorio</t>
   </si>
   <si>
-    <t>Total</t>
-  </si>
-  <si>
-    <t>SUMA</t>
-  </si>
-  <si>
-    <t xml:space="preserve">AVEGARE </t>
-  </si>
-  <si>
-    <t>COUNT</t>
-  </si>
-  <si>
-    <t xml:space="preserve">MIN </t>
-  </si>
-  <si>
-    <t>MAX</t>
-  </si>
-  <si>
     <t>Cursos + Claude</t>
   </si>
   <si>
@@ -488,20 +470,111 @@
   </si>
   <si>
     <t>Completo</t>
+  </si>
+  <si>
+    <t>A</t>
+  </si>
+  <si>
+    <t>B</t>
+  </si>
+  <si>
+    <t>C</t>
+  </si>
+  <si>
+    <t>D</t>
+  </si>
+  <si>
+    <t>E</t>
+  </si>
+  <si>
+    <t>F</t>
+  </si>
+  <si>
+    <t>Articulo</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Categoria </t>
+  </si>
+  <si>
+    <t>Fecha Compra</t>
+  </si>
+  <si>
+    <t>Precio</t>
+  </si>
+  <si>
+    <t>Proximo Mantenimiento</t>
+  </si>
+  <si>
+    <t>Garantia Hasta</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Estado </t>
+  </si>
+  <si>
+    <t>Lentes</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Salud/Vision </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Lugar de Compra </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Numero de Serie </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Clove EyeWear </t>
+  </si>
+  <si>
+    <t xml:space="preserve">VS AR CLOVE 65037 C9 52 18-142 Gris </t>
+  </si>
+  <si>
+    <r>
+      <t>Registro de Activos Personales</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="14"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>.</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">Nuevo </t>
+  </si>
+  <si>
+    <t xml:space="preserve">H </t>
+  </si>
+  <si>
+    <t xml:space="preserve">I </t>
+  </si>
+  <si>
+    <t xml:space="preserve">J </t>
+  </si>
+  <si>
+    <t xml:space="preserve">K </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Comprobante/Recibo </t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="5">
+  <numFmts count="6">
     <numFmt numFmtId="43" formatCode="_-* #,##0.00_-;\-* #,##0.00_-;_-* &quot;-&quot;??_-;_-@_-"/>
     <numFmt numFmtId="164" formatCode="_-[$$-409]* #,##0.00_ ;_-[$$-409]* \-#,##0.00\ ;_-[$$-409]* &quot;-&quot;??_ ;_-@_ "/>
     <numFmt numFmtId="165" formatCode="_-[$$-409]* #,##0.000_ ;_-[$$-409]* \-#,##0.000\ ;_-[$$-409]* &quot;-&quot;??_ ;_-@_ "/>
     <numFmt numFmtId="166" formatCode="_-* #,##0.0_-;\-* #,##0.0_-;_-* &quot;-&quot;??_-;_-@_-"/>
     <numFmt numFmtId="167" formatCode="_-[$$-2C0A]\ * #,##0.00_-;\-[$$-2C0A]\ * #,##0.00_-;_-[$$-2C0A]\ * &quot;-&quot;??_-;_-@_-"/>
+    <numFmt numFmtId="173" formatCode="dd/mm/yyyy;@"/>
   </numFmts>
-  <fonts count="12" x14ac:knownFonts="1">
+  <fonts count="14" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -586,8 +659,23 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FFFF0000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="14"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="16">
+  <fills count="17">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -678,6 +766,12 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="3" tint="0.59999389629810485"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="2">
     <border>
@@ -710,7 +804,7 @@
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="59">
+  <cellXfs count="67">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -831,6 +925,24 @@
     <xf numFmtId="167" fontId="0" fillId="14" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="9" fillId="12" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="17" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="17" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="17" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="17" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="9" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -864,29 +976,35 @@
     <xf numFmtId="0" fontId="8" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="17" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="173" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="173" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="43" fontId="0" fillId="0" borderId="1" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="16" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="16" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="17" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="17" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="16" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="16" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="17" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="17" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1">
-      <alignment vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="3">
@@ -2153,6 +2271,111 @@
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
+      <xdr:col>14</xdr:col>
+      <xdr:colOff>179456</xdr:colOff>
+      <xdr:row>75</xdr:row>
+      <xdr:rowOff>132522</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>23</xdr:col>
+      <xdr:colOff>563216</xdr:colOff>
+      <xdr:row>110</xdr:row>
+      <xdr:rowOff>176694</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="5" name="Picture 4">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{F8F8EA6A-1C31-3033-B60C-A1B29F5CF09C}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1">
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="10891630" y="18453652"/>
+          <a:ext cx="6468716" cy="8624955"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>8</xdr:col>
+      <xdr:colOff>179454</xdr:colOff>
+      <xdr:row>80</xdr:row>
+      <xdr:rowOff>198781</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>8</xdr:col>
+      <xdr:colOff>1391478</xdr:colOff>
+      <xdr:row>80</xdr:row>
+      <xdr:rowOff>1814814</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="9" name="Picture 8">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{88F8AC32-6FD9-6023-D01B-83CE1583688D}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId2" cstate="print">
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="7192063" y="19679477"/>
+          <a:ext cx="1212024" cy="1616033"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
       <xdr:col>2</xdr:col>
       <xdr:colOff>906600</xdr:colOff>
       <xdr:row>11</xdr:row>
@@ -2584,52 +2807,59 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E523AC75-1258-4F5B-8926-C1F345A2AD27}">
-  <dimension ref="A2:O82"/>
+  <dimension ref="A2:R81"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="11.109375" customWidth="1"/>
     <col min="2" max="2" width="14.5546875" customWidth="1"/>
-    <col min="3" max="5" width="11.5546875" customWidth="1"/>
-    <col min="6" max="6" width="10.88671875" customWidth="1"/>
-    <col min="7" max="7" width="15.33203125" customWidth="1"/>
-    <col min="8" max="8" width="9" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="11.77734375" customWidth="1"/>
+    <col min="3" max="3" width="11.5546875" customWidth="1"/>
+    <col min="4" max="4" width="13.88671875" bestFit="1" customWidth="1"/>
+    <col min="5" max="6" width="11.5546875" customWidth="1"/>
+    <col min="7" max="7" width="14.77734375" customWidth="1"/>
+    <col min="8" max="8" width="13.21875" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="21.44140625" customWidth="1"/>
+    <col min="10" max="10" width="15.33203125" customWidth="1"/>
     <col min="11" max="11" width="9" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="10.77734375" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="12.33203125" customWidth="1"/>
-    <col min="15" max="15" width="12.33203125" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="11.77734375" customWidth="1"/>
+    <col min="14" max="14" width="9" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="10.77734375" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="12.33203125" customWidth="1"/>
+    <col min="18" max="18" width="12.33203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="1:15" ht="31.2" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:18" ht="31.2" x14ac:dyDescent="0.3">
       <c r="A2" s="15" t="s">
         <v>44</v>
       </c>
     </row>
-    <row r="4" spans="1:15" ht="23.4" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:18" ht="23.4" x14ac:dyDescent="0.3">
       <c r="A4" s="16" t="s">
         <v>45</v>
       </c>
     </row>
-    <row r="6" spans="1:15" ht="31.2" x14ac:dyDescent="0.3">
-      <c r="A6" s="41" t="s">
+    <row r="6" spans="1:18" ht="31.2" x14ac:dyDescent="0.3">
+      <c r="A6" s="47" t="s">
         <v>46</v>
       </c>
-      <c r="B6" s="41"/>
-      <c r="C6" s="41"/>
-      <c r="D6" s="41"/>
-      <c r="E6" s="41"/>
-      <c r="F6" s="41"/>
-      <c r="G6" s="41"/>
-      <c r="H6" s="41"/>
-      <c r="I6" s="41"/>
-      <c r="J6" s="41"/>
-      <c r="K6" s="41"/>
-      <c r="L6" s="41"/>
-      <c r="M6" s="41"/>
-      <c r="N6" s="41"/>
-      <c r="O6" s="41"/>
-    </row>
-    <row r="8" spans="1:15" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="B6" s="47"/>
+      <c r="C6" s="47"/>
+      <c r="D6" s="47"/>
+      <c r="E6" s="47"/>
+      <c r="F6" s="47"/>
+      <c r="G6" s="47"/>
+      <c r="H6" s="47"/>
+      <c r="I6" s="47"/>
+      <c r="J6" s="47"/>
+      <c r="K6" s="47"/>
+      <c r="L6" s="47"/>
+      <c r="M6" s="47"/>
+      <c r="N6" s="47"/>
+      <c r="O6" s="47"/>
+      <c r="P6" s="47"/>
+      <c r="Q6" s="47"/>
+      <c r="R6" s="47"/>
+    </row>
+    <row r="8" spans="1:18" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A8" s="34" t="s">
         <v>47</v>
       </c>
@@ -2641,38 +2871,41 @@
       </c>
       <c r="D8" s="34"/>
       <c r="E8" s="34"/>
-      <c r="F8" s="34" t="s">
+      <c r="F8" s="34"/>
+      <c r="G8" s="34"/>
+      <c r="H8" s="34" t="s">
         <v>50</v>
       </c>
-      <c r="G8" s="34" t="s">
+      <c r="I8" s="34"/>
+      <c r="J8" s="34" t="s">
         <v>51</v>
       </c>
-      <c r="H8" s="34" t="s">
+      <c r="K8" s="34" t="s">
         <v>52</v>
       </c>
-      <c r="I8" s="34" t="s">
+      <c r="L8" s="34" t="s">
         <v>53</v>
       </c>
-      <c r="J8" s="34" t="s">
+      <c r="M8" s="34" t="s">
         <v>77</v>
       </c>
-      <c r="K8" s="34" t="s">
+      <c r="N8" s="34" t="s">
         <v>54</v>
       </c>
-      <c r="L8" s="34" t="s">
+      <c r="O8" s="34" t="s">
         <v>55</v>
       </c>
-      <c r="M8" s="34" t="s">
+      <c r="P8" s="34" t="s">
         <v>56</v>
       </c>
-      <c r="N8" s="34" t="s">
+      <c r="Q8" s="34" t="s">
         <v>57</v>
       </c>
-      <c r="O8" s="34" t="s">
+      <c r="R8" s="34" t="s">
         <v>58</v>
       </c>
     </row>
-    <row r="9" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A9" s="26">
         <v>1</v>
       </c>
@@ -2684,36 +2917,39 @@
       </c>
       <c r="D9" s="27"/>
       <c r="E9" s="27"/>
-      <c r="F9" s="27" t="s">
+      <c r="F9" s="27"/>
+      <c r="G9" s="27"/>
+      <c r="H9" s="27" t="s">
         <v>61</v>
       </c>
-      <c r="G9" s="27" t="s">
+      <c r="I9" s="27"/>
+      <c r="J9" s="27" t="s">
         <v>62</v>
       </c>
-      <c r="H9" s="28">
+      <c r="K9" s="28">
         <v>900</v>
       </c>
-      <c r="I9" s="28">
+      <c r="L9" s="28">
         <v>1200</v>
       </c>
-      <c r="J9" s="28"/>
-      <c r="K9" s="27">
+      <c r="M9" s="28"/>
+      <c r="N9" s="27">
         <v>1</v>
       </c>
-      <c r="L9" s="29">
+      <c r="O9" s="29">
         <v>46244</v>
       </c>
-      <c r="M9" s="27" t="s">
+      <c r="P9" s="27" t="s">
         <v>63</v>
       </c>
-      <c r="N9" s="27" t="s">
+      <c r="Q9" s="27" t="s">
         <v>64</v>
       </c>
-      <c r="O9" s="30" t="s">
+      <c r="R9" s="30" t="s">
         <v>65</v>
       </c>
     </row>
-    <row r="10" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A10" s="26">
         <v>2</v>
       </c>
@@ -2725,36 +2961,39 @@
       </c>
       <c r="D10" s="27"/>
       <c r="E10" s="27"/>
-      <c r="F10" s="27" t="s">
+      <c r="F10" s="27"/>
+      <c r="G10" s="27"/>
+      <c r="H10" s="27" t="s">
         <v>68</v>
       </c>
-      <c r="G10" s="27" t="s">
+      <c r="I10" s="27"/>
+      <c r="J10" s="27" t="s">
         <v>69</v>
       </c>
-      <c r="H10" s="28">
+      <c r="K10" s="28">
         <v>150</v>
       </c>
-      <c r="I10" s="28">
+      <c r="L10" s="28">
         <v>250</v>
       </c>
-      <c r="J10" s="28"/>
-      <c r="K10" s="27">
+      <c r="M10" s="28"/>
+      <c r="N10" s="27">
         <v>1</v>
       </c>
-      <c r="L10" s="29">
+      <c r="O10" s="29">
         <v>46249</v>
       </c>
-      <c r="M10" s="27" t="s">
+      <c r="P10" s="27" t="s">
         <v>63</v>
       </c>
-      <c r="N10" s="27" t="s">
+      <c r="Q10" s="27" t="s">
         <v>70</v>
       </c>
-      <c r="O10" s="30" t="s">
+      <c r="R10" s="30" t="s">
         <v>71</v>
       </c>
     </row>
-    <row r="11" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A11" s="26">
         <v>3</v>
       </c>
@@ -2766,36 +3005,39 @@
       </c>
       <c r="D11" s="27"/>
       <c r="E11" s="27"/>
-      <c r="F11" s="27" t="s">
+      <c r="F11" s="27"/>
+      <c r="G11" s="27"/>
+      <c r="H11" s="27" t="s">
         <v>61</v>
       </c>
-      <c r="G11" s="27" t="s">
+      <c r="I11" s="27"/>
+      <c r="J11" s="27" t="s">
         <v>62</v>
       </c>
-      <c r="H11" s="28">
+      <c r="K11" s="28">
         <v>250</v>
       </c>
-      <c r="I11" s="28">
+      <c r="L11" s="28">
         <v>275</v>
       </c>
-      <c r="J11" s="28"/>
-      <c r="K11" s="27">
+      <c r="M11" s="28"/>
+      <c r="N11" s="27">
         <v>1</v>
       </c>
-      <c r="L11" s="31">
+      <c r="O11" s="31">
         <v>46254</v>
       </c>
-      <c r="M11" s="27" t="s">
+      <c r="P11" s="27" t="s">
         <v>63</v>
       </c>
-      <c r="N11" s="32" t="s">
+      <c r="Q11" s="32" t="s">
         <v>64</v>
       </c>
-      <c r="O11" s="33" t="s">
+      <c r="R11" s="33" t="s">
         <v>73</v>
       </c>
     </row>
-    <row r="12" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A12" s="26">
         <v>4</v>
       </c>
@@ -2807,64 +3049,70 @@
       </c>
       <c r="D12" s="27"/>
       <c r="E12" s="27"/>
-      <c r="F12" s="27" t="s">
+      <c r="F12" s="27"/>
+      <c r="G12" s="27"/>
+      <c r="H12" s="27" t="s">
         <v>61</v>
       </c>
-      <c r="G12" s="27" t="s">
+      <c r="I12" s="27"/>
+      <c r="J12" s="27" t="s">
         <v>69</v>
       </c>
-      <c r="H12" s="28">
+      <c r="K12" s="28">
         <v>1500</v>
       </c>
-      <c r="I12" s="28">
+      <c r="L12" s="28">
         <v>1575</v>
       </c>
-      <c r="J12" s="28">
+      <c r="M12" s="28">
         <v>75</v>
       </c>
-      <c r="K12" s="27">
+      <c r="N12" s="27">
         <v>1</v>
       </c>
-      <c r="L12" s="31">
+      <c r="O12" s="31">
         <v>46175</v>
       </c>
-      <c r="M12" s="27" t="s">
+      <c r="P12" s="27" t="s">
         <v>76</v>
       </c>
-      <c r="N12" s="32" t="s">
+      <c r="Q12" s="32" t="s">
         <v>64</v>
       </c>
-      <c r="O12" s="32" t="s">
+      <c r="R12" s="32" t="s">
         <v>71</v>
       </c>
     </row>
-    <row r="16" spans="1:15" ht="31.2" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:18" ht="31.2" x14ac:dyDescent="0.3">
       <c r="A16" s="15" t="s">
         <v>78</v>
       </c>
     </row>
-    <row r="18" spans="1:11" ht="23.4" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:14" ht="23.4" x14ac:dyDescent="0.3">
       <c r="A18" s="16" t="s">
         <v>45</v>
       </c>
     </row>
-    <row r="20" spans="1:11" ht="31.2" x14ac:dyDescent="0.3">
-      <c r="A20" s="42" t="s">
+    <row r="20" spans="1:14" ht="31.2" x14ac:dyDescent="0.3">
+      <c r="A20" s="48" t="s">
         <v>79</v>
       </c>
-      <c r="B20" s="42"/>
-      <c r="C20" s="42"/>
-      <c r="D20" s="42"/>
-      <c r="E20" s="42"/>
-      <c r="F20" s="42"/>
-      <c r="G20" s="42"/>
-      <c r="H20" s="42"/>
-      <c r="I20" s="42"/>
-      <c r="K20" s="16" t="s">
+      <c r="B20" s="48"/>
+      <c r="C20" s="48"/>
+      <c r="D20" s="48"/>
+      <c r="E20" s="48"/>
+      <c r="F20" s="48"/>
+      <c r="G20" s="48"/>
+      <c r="H20" s="48"/>
+      <c r="I20" s="48"/>
+      <c r="J20" s="48"/>
+      <c r="K20" s="48"/>
+      <c r="L20" s="48"/>
+      <c r="N20" s="16" t="s">
         <v>90</v>
       </c>
     </row>
-    <row r="21" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A21" s="2"/>
       <c r="B21" s="2"/>
       <c r="C21" s="2"/>
@@ -2874,8 +3122,11 @@
       <c r="G21" s="2"/>
       <c r="H21" s="2"/>
       <c r="I21" s="2"/>
-    </row>
-    <row r="22" spans="1:11" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="J21" s="2"/>
+      <c r="K21" s="2"/>
+      <c r="L21" s="2"/>
+    </row>
+    <row r="22" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A22" s="19" t="s">
         <v>80</v>
       </c>
@@ -2887,23 +3138,26 @@
       </c>
       <c r="D22" s="19"/>
       <c r="E22" s="19"/>
-      <c r="F22" s="19" t="s">
+      <c r="F22" s="19"/>
+      <c r="G22" s="19"/>
+      <c r="H22" s="19" t="s">
         <v>83</v>
       </c>
-      <c r="G22" s="19" t="s">
+      <c r="I22" s="19"/>
+      <c r="J22" s="19" t="s">
         <v>84</v>
       </c>
-      <c r="H22" s="19" t="s">
+      <c r="K22" s="19" t="s">
         <v>85</v>
       </c>
-      <c r="I22" s="19" t="s">
+      <c r="L22" s="19" t="s">
         <v>86</v>
       </c>
-      <c r="K22" t="s">
+      <c r="N22" t="s">
         <v>91</v>
       </c>
     </row>
-    <row r="23" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A23" s="24" t="s">
         <v>87</v>
       </c>
@@ -2915,21 +3169,24 @@
       </c>
       <c r="D23" s="24"/>
       <c r="E23" s="24"/>
-      <c r="F23" s="24">
-        <v>0</v>
-      </c>
-      <c r="G23" s="24">
-        <v>0</v>
-      </c>
+      <c r="F23" s="24"/>
+      <c r="G23" s="24"/>
       <c r="H23" s="24">
         <v>0</v>
       </c>
-      <c r="I23" s="24">
+      <c r="I23" s="24"/>
+      <c r="J23" s="24">
         <v>0</v>
       </c>
-      <c r="K23" s="20"/>
-    </row>
-    <row r="24" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="K23" s="24">
+        <v>0</v>
+      </c>
+      <c r="L23" s="24">
+        <v>0</v>
+      </c>
+      <c r="N23" s="20"/>
+    </row>
+    <row r="24" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A24" s="24" t="s">
         <v>88</v>
       </c>
@@ -2941,23 +3198,26 @@
       </c>
       <c r="D24" s="24"/>
       <c r="E24" s="24"/>
-      <c r="F24" s="24">
-        <v>0</v>
-      </c>
-      <c r="G24" s="24">
-        <v>0</v>
-      </c>
+      <c r="F24" s="24"/>
+      <c r="G24" s="24"/>
       <c r="H24" s="24">
         <v>0</v>
       </c>
-      <c r="I24" s="24">
+      <c r="I24" s="24"/>
+      <c r="J24" s="24">
         <v>0</v>
       </c>
-      <c r="K24" s="20" t="s">
+      <c r="K24" s="24">
+        <v>0</v>
+      </c>
+      <c r="L24" s="24">
+        <v>0</v>
+      </c>
+      <c r="N24" s="20" t="s">
         <v>92</v>
       </c>
     </row>
-    <row r="25" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A25" s="24" t="s">
         <v>89</v>
       </c>
@@ -2969,79 +3229,88 @@
       </c>
       <c r="D25" s="24"/>
       <c r="E25" s="24"/>
-      <c r="F25" s="24">
-        <v>0</v>
-      </c>
-      <c r="G25" s="24">
-        <v>0</v>
-      </c>
+      <c r="F25" s="24"/>
+      <c r="G25" s="24"/>
       <c r="H25" s="24">
         <v>0</v>
       </c>
-      <c r="I25" s="24">
+      <c r="I25" s="24"/>
+      <c r="J25" s="24">
         <v>0</v>
       </c>
-      <c r="K25" s="20" t="s">
+      <c r="K25" s="24">
+        <v>0</v>
+      </c>
+      <c r="L25" s="24">
+        <v>0</v>
+      </c>
+      <c r="N25" s="20" t="s">
         <v>93</v>
       </c>
     </row>
-    <row r="26" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="K26" s="20" t="s">
+    <row r="26" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="N26" s="20" t="s">
         <v>94</v>
       </c>
     </row>
-    <row r="27" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="K27" s="20" t="s">
+    <row r="27" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="N27" s="20" t="s">
         <v>95</v>
       </c>
     </row>
-    <row r="28" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="K28" s="20" t="s">
+    <row r="28" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="N28" s="20" t="s">
         <v>96</v>
       </c>
     </row>
-    <row r="29" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="K29" s="20" t="s">
+    <row r="29" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="N29" s="20" t="s">
         <v>97</v>
       </c>
     </row>
-    <row r="30" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="K30" s="20" t="s">
+    <row r="30" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="N30" s="20" t="s">
         <v>71</v>
       </c>
     </row>
-    <row r="33" spans="1:9" ht="31.2" x14ac:dyDescent="0.3">
-      <c r="A33" s="43" t="s">
+    <row r="33" spans="1:12" ht="31.2" x14ac:dyDescent="0.3">
+      <c r="A33" s="49" t="s">
         <v>107</v>
       </c>
-      <c r="B33" s="43"/>
-      <c r="C33" s="43"/>
-      <c r="D33" s="43"/>
-      <c r="E33" s="43"/>
-      <c r="F33" s="43"/>
-      <c r="G33" s="43"/>
-      <c r="H33" s="43"/>
-      <c r="I33" s="43"/>
-    </row>
-    <row r="35" spans="1:9" ht="23.4" x14ac:dyDescent="0.3">
+      <c r="B33" s="49"/>
+      <c r="C33" s="49"/>
+      <c r="D33" s="49"/>
+      <c r="E33" s="49"/>
+      <c r="F33" s="49"/>
+      <c r="G33" s="49"/>
+      <c r="H33" s="49"/>
+      <c r="I33" s="49"/>
+      <c r="J33" s="49"/>
+      <c r="K33" s="49"/>
+      <c r="L33" s="49"/>
+    </row>
+    <row r="35" spans="1:12" ht="23.4" x14ac:dyDescent="0.3">
       <c r="A35" s="16" t="s">
         <v>45</v>
       </c>
     </row>
-    <row r="37" spans="1:9" ht="31.2" x14ac:dyDescent="0.3">
-      <c r="A37" s="44" t="s">
+    <row r="37" spans="1:12" ht="31.2" x14ac:dyDescent="0.3">
+      <c r="A37" s="50" t="s">
         <v>98</v>
       </c>
-      <c r="B37" s="44"/>
-      <c r="C37" s="44"/>
-      <c r="D37" s="44"/>
-      <c r="E37" s="44"/>
-      <c r="F37" s="44"/>
-      <c r="G37" s="44"/>
-      <c r="H37" s="44"/>
-      <c r="I37" s="44"/>
-    </row>
-    <row r="39" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="B37" s="50"/>
+      <c r="C37" s="50"/>
+      <c r="D37" s="50"/>
+      <c r="E37" s="50"/>
+      <c r="F37" s="50"/>
+      <c r="G37" s="50"/>
+      <c r="H37" s="50"/>
+      <c r="I37" s="50"/>
+      <c r="J37" s="50"/>
+      <c r="K37" s="50"/>
+      <c r="L37" s="50"/>
+    </row>
+    <row r="39" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A39" s="35" t="s">
         <v>99</v>
       </c>
@@ -3051,20 +3320,23 @@
       <c r="C39" s="35" t="s">
         <v>101</v>
       </c>
-      <c r="D39" s="35" t="s">
+      <c r="D39" s="35"/>
+      <c r="E39" s="35"/>
+      <c r="F39" s="35" t="s">
         <v>50</v>
       </c>
-      <c r="E39" s="35" t="s">
+      <c r="G39" s="35" t="s">
         <v>56</v>
       </c>
-      <c r="F39" s="35" t="s">
+      <c r="H39" s="35" t="s">
         <v>102</v>
       </c>
-      <c r="G39" s="35" t="s">
+      <c r="I39" s="35"/>
+      <c r="J39" s="35" t="s">
         <v>103</v>
       </c>
     </row>
-    <row r="40" spans="1:9" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:12" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A40" s="18" t="s">
         <v>129</v>
       </c>
@@ -3074,20 +3346,23 @@
       <c r="C40" s="21">
         <v>46357</v>
       </c>
-      <c r="D40" s="18" t="s">
+      <c r="D40" s="21"/>
+      <c r="E40" s="21"/>
+      <c r="F40" s="18" t="s">
         <v>61</v>
       </c>
-      <c r="E40" s="18" t="s">
+      <c r="G40" s="18" t="s">
         <v>104</v>
       </c>
-      <c r="F40" s="36">
+      <c r="H40" s="36">
         <v>100</v>
       </c>
-      <c r="G40" s="36">
+      <c r="I40" s="36"/>
+      <c r="J40" s="36">
         <v>50</v>
       </c>
     </row>
-    <row r="41" spans="1:9" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:12" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A41" s="18" t="s">
         <v>105</v>
       </c>
@@ -3097,20 +3372,23 @@
       <c r="C41" s="21">
         <v>46296</v>
       </c>
-      <c r="D41" s="18" t="s">
+      <c r="D41" s="21"/>
+      <c r="E41" s="21"/>
+      <c r="F41" s="18" t="s">
         <v>61</v>
       </c>
-      <c r="E41" s="18" t="s">
+      <c r="G41" s="18" t="s">
         <v>63</v>
       </c>
-      <c r="F41" s="18">
+      <c r="H41" s="18">
         <v>0</v>
       </c>
-      <c r="G41" s="18">
+      <c r="I41" s="18"/>
+      <c r="J41" s="18">
         <v>1250</v>
       </c>
     </row>
-    <row r="42" spans="1:9" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:12" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A42" s="18" t="s">
         <v>106</v>
       </c>
@@ -3120,40 +3398,46 @@
       <c r="C42" s="21">
         <v>46388</v>
       </c>
-      <c r="D42" s="18" t="s">
+      <c r="D42" s="21"/>
+      <c r="E42" s="21"/>
+      <c r="F42" s="18" t="s">
         <v>68</v>
       </c>
-      <c r="E42" s="18" t="s">
+      <c r="G42" s="18" t="s">
         <v>63</v>
       </c>
-      <c r="F42" s="2">
+      <c r="H42" s="2">
         <v>50</v>
       </c>
-      <c r="G42" s="18">
+      <c r="I42" s="2"/>
+      <c r="J42" s="18">
         <v>450</v>
       </c>
     </row>
-    <row r="47" spans="1:9" ht="31.2" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:12" ht="31.2" x14ac:dyDescent="0.3">
       <c r="A47" s="15" t="s">
         <v>108</v>
       </c>
     </row>
-    <row r="49" spans="1:6" ht="23.4" x14ac:dyDescent="0.3">
+    <row r="49" spans="1:9" ht="23.4" x14ac:dyDescent="0.3">
       <c r="A49" s="16" t="s">
         <v>45</v>
       </c>
     </row>
-    <row r="51" spans="1:6" ht="31.2" x14ac:dyDescent="0.3">
-      <c r="A51" s="45" t="s">
+    <row r="51" spans="1:9" ht="31.2" x14ac:dyDescent="0.3">
+      <c r="A51" s="51" t="s">
         <v>109</v>
       </c>
-      <c r="B51" s="45"/>
-      <c r="C51" s="45"/>
-      <c r="D51" s="45"/>
-      <c r="E51" s="45"/>
-      <c r="F51" s="45"/>
-    </row>
-    <row r="53" spans="1:6" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="B51" s="51"/>
+      <c r="C51" s="51"/>
+      <c r="D51" s="51"/>
+      <c r="E51" s="51"/>
+      <c r="F51" s="51"/>
+      <c r="G51" s="51"/>
+      <c r="H51" s="51"/>
+      <c r="I51" s="40"/>
+    </row>
+    <row r="53" spans="1:9" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A53" s="22" t="s">
         <v>110</v>
       </c>
@@ -3163,11 +3447,13 @@
       <c r="C53" s="22" t="s">
         <v>112</v>
       </c>
-      <c r="D53" s="22" t="s">
+      <c r="D53" s="22"/>
+      <c r="E53" s="22"/>
+      <c r="F53" s="22" t="s">
         <v>113</v>
       </c>
     </row>
-    <row r="54" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="54" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A54" s="25">
         <v>46174</v>
       </c>
@@ -3177,11 +3463,13 @@
       <c r="C54" s="24" t="s">
         <v>66</v>
       </c>
-      <c r="D54" s="39">
+      <c r="D54" s="24"/>
+      <c r="E54" s="24"/>
+      <c r="F54" s="39">
         <v>300</v>
       </c>
     </row>
-    <row r="55" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="55" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A55" s="25">
         <v>46387</v>
       </c>
@@ -3191,35 +3479,40 @@
       <c r="C55" s="24" t="s">
         <v>114</v>
       </c>
-      <c r="D55" s="38">
+      <c r="D55" s="24"/>
+      <c r="E55" s="24"/>
+      <c r="F55" s="38">
         <v>50</v>
       </c>
     </row>
-    <row r="60" spans="1:6" ht="31.2" x14ac:dyDescent="0.3">
+    <row r="60" spans="1:9" ht="31.2" x14ac:dyDescent="0.3">
       <c r="A60" s="15" t="s">
         <v>115</v>
       </c>
     </row>
-    <row r="62" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="62" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A62" t="s">
         <v>116</v>
       </c>
     </row>
-    <row r="64" spans="1:6" ht="23.4" x14ac:dyDescent="0.3">
+    <row r="64" spans="1:9" ht="23.4" x14ac:dyDescent="0.3">
       <c r="A64" s="16" t="s">
         <v>45</v>
       </c>
     </row>
     <row r="66" spans="1:10" ht="31.2" x14ac:dyDescent="0.3">
-      <c r="A66" s="40" t="s">
+      <c r="A66" s="46" t="s">
         <v>117</v>
       </c>
-      <c r="B66" s="40"/>
-      <c r="C66" s="40"/>
-      <c r="D66" s="40"/>
-      <c r="E66" s="40"/>
-      <c r="F66" s="40"/>
-      <c r="G66" s="40"/>
+      <c r="B66" s="46"/>
+      <c r="C66" s="46"/>
+      <c r="D66" s="46"/>
+      <c r="E66" s="46"/>
+      <c r="F66" s="46"/>
+      <c r="G66" s="46"/>
+      <c r="H66" s="46"/>
+      <c r="I66" s="46"/>
+      <c r="J66" s="46"/>
     </row>
     <row r="68" spans="1:10" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A68" s="23" t="s">
@@ -3231,16 +3524,19 @@
       <c r="C68" s="23" t="s">
         <v>119</v>
       </c>
-      <c r="D68" s="23" t="s">
+      <c r="D68" s="23"/>
+      <c r="E68" s="23"/>
+      <c r="F68" s="23" t="s">
+        <v>134</v>
+      </c>
+      <c r="G68" s="23" t="s">
+        <v>120</v>
+      </c>
+      <c r="H68" s="23" t="s">
         <v>140</v>
       </c>
-      <c r="E68" s="23" t="s">
-        <v>120</v>
-      </c>
-      <c r="F68" s="23" t="s">
-        <v>146</v>
-      </c>
-      <c r="G68" s="23" t="s">
+      <c r="I68" s="23"/>
+      <c r="J68" s="23" t="s">
         <v>121</v>
       </c>
     </row>
@@ -3252,19 +3548,22 @@
         <v>104</v>
       </c>
       <c r="C69" s="17" t="s">
-        <v>139</v>
-      </c>
-      <c r="D69" s="53" t="s">
-        <v>142</v>
-      </c>
-      <c r="E69" s="53" t="s">
-        <v>144</v>
-      </c>
-      <c r="F69" s="21" t="s">
-        <v>147</v>
-      </c>
-      <c r="G69" s="18" t="s">
+        <v>133</v>
+      </c>
+      <c r="D69" s="17"/>
+      <c r="E69" s="17"/>
+      <c r="F69" s="43" t="s">
         <v>136</v>
+      </c>
+      <c r="G69" s="43" t="s">
+        <v>138</v>
+      </c>
+      <c r="H69" s="21" t="s">
+        <v>141</v>
+      </c>
+      <c r="I69" s="21"/>
+      <c r="J69" s="17" t="s">
+        <v>130</v>
       </c>
     </row>
     <row r="70" spans="1:10" ht="28.8" x14ac:dyDescent="0.3">
@@ -3277,17 +3576,20 @@
       <c r="C70" s="18" t="s">
         <v>123</v>
       </c>
-      <c r="D70" s="53" t="s">
-        <v>143</v>
-      </c>
-      <c r="E70" s="53" t="s">
-        <v>145</v>
-      </c>
-      <c r="F70" s="21">
+      <c r="D70" s="18"/>
+      <c r="E70" s="18"/>
+      <c r="F70" s="43" t="s">
+        <v>137</v>
+      </c>
+      <c r="G70" s="43" t="s">
+        <v>139</v>
+      </c>
+      <c r="H70" s="21">
         <v>46266</v>
       </c>
-      <c r="G70" s="18" t="s">
-        <v>137</v>
+      <c r="I70" s="21"/>
+      <c r="J70" s="17" t="s">
+        <v>131</v>
       </c>
     </row>
     <row r="71" spans="1:10" x14ac:dyDescent="0.3">
@@ -3300,17 +3602,20 @@
       <c r="C71" s="18" t="s">
         <v>123</v>
       </c>
-      <c r="D71" s="53" t="s">
-        <v>143</v>
-      </c>
-      <c r="E71" s="21">
+      <c r="D71" s="18"/>
+      <c r="E71" s="18"/>
+      <c r="F71" s="43" t="s">
+        <v>137</v>
+      </c>
+      <c r="G71" s="21">
         <v>47696</v>
       </c>
-      <c r="F71" s="21">
+      <c r="H71" s="21">
         <v>46327</v>
       </c>
-      <c r="G71" s="18" t="s">
-        <v>138</v>
+      <c r="I71" s="21"/>
+      <c r="J71" s="17" t="s">
+        <v>132</v>
       </c>
     </row>
     <row r="72" spans="1:10" x14ac:dyDescent="0.3">
@@ -3323,14 +3628,17 @@
       <c r="C72" s="18" t="s">
         <v>126</v>
       </c>
-      <c r="D72" s="51">
+      <c r="D72" s="18"/>
+      <c r="E72" s="18"/>
+      <c r="F72" s="41">
         <v>46296</v>
       </c>
-      <c r="E72" s="17"/>
-      <c r="F72" s="51">
+      <c r="G72" s="17"/>
+      <c r="H72" s="41">
         <v>46388</v>
       </c>
-      <c r="G72" s="18" t="s">
+      <c r="I72" s="41"/>
+      <c r="J72" s="17" t="s">
         <v>127</v>
       </c>
     </row>
@@ -3344,133 +3652,163 @@
       <c r="C73" s="18" t="s">
         <v>126</v>
       </c>
-      <c r="D73" s="51">
+      <c r="D73" s="18"/>
+      <c r="E73" s="18"/>
+      <c r="F73" s="41">
         <v>46388</v>
       </c>
-      <c r="E73" s="51">
+      <c r="G73" s="43">
         <v>46447</v>
       </c>
-      <c r="F73" s="54">
+      <c r="H73" s="44">
         <v>46539</v>
       </c>
-      <c r="G73" s="52" t="s">
+      <c r="I73" s="44"/>
+      <c r="J73" s="42" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="74" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A74" s="18" t="s">
+        <v>143</v>
+      </c>
+      <c r="B74" s="18" t="s">
+        <v>144</v>
+      </c>
+      <c r="C74" s="18" t="s">
+        <v>145</v>
+      </c>
+      <c r="D74" s="18"/>
+      <c r="E74" s="18"/>
+      <c r="F74" s="41" t="s">
+        <v>135</v>
+      </c>
+      <c r="G74" s="17" t="s">
+        <v>135</v>
+      </c>
+      <c r="H74" s="45">
+        <v>46539</v>
+      </c>
+      <c r="I74" s="45"/>
+      <c r="J74" s="17" t="s">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="77" spans="1:10" ht="18" x14ac:dyDescent="0.3">
+      <c r="A77" s="58" t="s">
+        <v>165</v>
+      </c>
+      <c r="B77" s="58"/>
+      <c r="C77" s="58"/>
+      <c r="D77" s="57"/>
+      <c r="E77" s="57"/>
+    </row>
+    <row r="79" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A79" s="59" t="s">
+        <v>146</v>
+      </c>
+      <c r="B79" s="59" t="s">
+        <v>147</v>
+      </c>
+      <c r="C79" s="59" t="s">
         <v>148</v>
       </c>
-    </row>
-    <row r="74" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A74" s="55" t="s">
+      <c r="D79" s="59" t="s">
         <v>149</v>
       </c>
-      <c r="B74" s="55" t="s">
+      <c r="E79" s="59" t="s">
         <v>150</v>
       </c>
-      <c r="C74" s="55" t="s">
+      <c r="F79" s="59" t="s">
         <v>151</v>
       </c>
-      <c r="D74" s="56" t="s">
-        <v>141</v>
-      </c>
-      <c r="E74" s="57" t="s">
-        <v>141</v>
-      </c>
-      <c r="F74" s="58">
-        <v>46539</v>
-      </c>
-      <c r="G74" s="57" t="s">
-        <v>141</v>
-      </c>
-    </row>
-    <row r="76" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="H76" t="s">
-        <v>134</v>
-      </c>
-      <c r="I76" t="s">
-        <v>135</v>
-      </c>
-    </row>
-    <row r="77" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="H77" t="s">
-        <v>131</v>
-      </c>
-      <c r="I77" t="s">
-        <v>132</v>
-      </c>
-      <c r="J77" t="s">
-        <v>133</v>
-      </c>
-    </row>
-    <row r="78" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="H78">
-        <v>8</v>
-      </c>
-      <c r="I78">
-        <v>2</v>
-      </c>
-      <c r="J78">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="79" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="H79">
-        <v>5</v>
-      </c>
-      <c r="I79">
-        <v>2</v>
-      </c>
-      <c r="J79">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="80" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="H80">
-        <v>3</v>
-      </c>
-      <c r="I80">
-        <v>8</v>
-      </c>
-      <c r="J80">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="81" spans="8:11" x14ac:dyDescent="0.3">
-      <c r="H81">
-        <v>4</v>
-      </c>
-      <c r="I81">
-        <v>2</v>
-      </c>
-      <c r="J81">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="82" spans="8:11" x14ac:dyDescent="0.3">
-      <c r="H82">
-        <f>MIN(H78:H81)</f>
-        <v>3</v>
-      </c>
-      <c r="I82">
-        <f>MAX(I78:I81)</f>
-        <v>8</v>
-      </c>
-      <c r="J82">
-        <f>AVERAGE(J78:J81)</f>
-        <v>5</v>
-      </c>
-      <c r="K82" t="s">
-        <v>130</v>
+      <c r="G79" s="59" t="s">
+        <v>167</v>
+      </c>
+      <c r="H79" s="59" t="s">
+        <v>168</v>
+      </c>
+      <c r="I79" s="59" t="s">
+        <v>169</v>
+      </c>
+      <c r="J79" s="59" t="s">
+        <v>170</v>
+      </c>
+    </row>
+    <row r="80" spans="1:10" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A80" s="63" t="s">
+        <v>152</v>
+      </c>
+      <c r="B80" s="63" t="s">
+        <v>153</v>
+      </c>
+      <c r="C80" s="64" t="s">
+        <v>154</v>
+      </c>
+      <c r="D80" s="64" t="s">
+        <v>161</v>
+      </c>
+      <c r="E80" s="64" t="s">
+        <v>162</v>
+      </c>
+      <c r="F80" s="63" t="s">
+        <v>155</v>
+      </c>
+      <c r="G80" s="64" t="s">
+        <v>156</v>
+      </c>
+      <c r="H80" s="65" t="s">
+        <v>157</v>
+      </c>
+      <c r="I80" s="66" t="s">
+        <v>171</v>
+      </c>
+      <c r="J80" s="64" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="81" spans="1:10" ht="156" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A81" s="2" t="s">
+        <v>159</v>
+      </c>
+      <c r="B81" s="2" t="s">
+        <v>160</v>
+      </c>
+      <c r="C81" s="60">
+        <v>46181</v>
+      </c>
+      <c r="D81" s="60" t="s">
+        <v>163</v>
+      </c>
+      <c r="E81" s="61" t="s">
+        <v>164</v>
+      </c>
+      <c r="F81" s="62">
+        <v>3800</v>
+      </c>
+      <c r="G81" s="2"/>
+      <c r="H81" s="60">
+        <v>46184</v>
+      </c>
+      <c r="I81" s="60"/>
+      <c r="J81" s="2" t="s">
+        <v>166</v>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="6">
-    <mergeCell ref="A66:G66"/>
-    <mergeCell ref="A6:O6"/>
-    <mergeCell ref="A20:I20"/>
-    <mergeCell ref="A33:I33"/>
-    <mergeCell ref="A37:I37"/>
-    <mergeCell ref="A51:F51"/>
+  <mergeCells count="7">
+    <mergeCell ref="A77:C77"/>
+    <mergeCell ref="A66:J66"/>
+    <mergeCell ref="A6:R6"/>
+    <mergeCell ref="A20:L20"/>
+    <mergeCell ref="A33:L33"/>
+    <mergeCell ref="A37:L37"/>
+    <mergeCell ref="A51:H51"/>
   </mergeCells>
   <phoneticPr fontId="11" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
+  <drawing r:id="rId2"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{05C60535-1F16-4fd2-B633-F4F36F0B64E0}">
       <x14:sparklineGroups xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
@@ -3485,12 +3823,16 @@
           <x14:colorLow rgb="FFD00000"/>
           <x14:sparklines>
             <x14:sparkline>
-              <xm:f>'Personal-Budget_2026'!F:F</xm:f>
-              <xm:sqref>F68</xm:sqref>
+              <xm:f>'Personal-Budget_2026'!G:G</xm:f>
+              <xm:sqref>G68</xm:sqref>
             </x14:sparkline>
             <x14:sparkline>
-              <xm:f>'Personal-Budget_2026'!E:E</xm:f>
-              <xm:sqref>E68</xm:sqref>
+              <xm:f>'Personal-Budget_2026'!H:H</xm:f>
+              <xm:sqref>H68</xm:sqref>
+            </x14:sparkline>
+            <x14:sparkline>
+              <xm:f>'Personal-Budget_2026'!I:I</xm:f>
+              <xm:sqref>I68</xm:sqref>
             </x14:sparkline>
           </x14:sparklines>
         </x14:sparklineGroup>
@@ -3514,11 +3856,11 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:4" ht="18" x14ac:dyDescent="0.3">
-      <c r="A1" s="46" t="s">
+      <c r="A1" s="52" t="s">
         <v>4</v>
       </c>
-      <c r="B1" s="47"/>
-      <c r="C1" s="47"/>
+      <c r="B1" s="53"/>
+      <c r="C1" s="53"/>
     </row>
     <row r="2" spans="1:4" ht="15" x14ac:dyDescent="0.3">
       <c r="B2" s="1"/>
@@ -3659,11 +4001,11 @@
       <c r="C16" s="8"/>
     </row>
     <row r="17" spans="1:4" ht="21" x14ac:dyDescent="0.3">
-      <c r="A17" s="48" t="s">
+      <c r="A17" s="54" t="s">
         <v>13</v>
       </c>
-      <c r="B17" s="48"/>
-      <c r="C17" s="48"/>
+      <c r="B17" s="54"/>
+      <c r="C17" s="54"/>
     </row>
     <row r="19" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A19" s="12" t="s">
@@ -3815,11 +4157,11 @@
       </c>
     </row>
     <row r="31" spans="1:4" ht="21" x14ac:dyDescent="0.3">
-      <c r="A31" s="48" t="s">
+      <c r="A31" s="54" t="s">
         <v>13</v>
       </c>
-      <c r="B31" s="48"/>
-      <c r="C31" s="48"/>
+      <c r="B31" s="54"/>
+      <c r="C31" s="54"/>
     </row>
     <row r="33" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A33" s="12" t="s">
@@ -3971,26 +4313,26 @@
       </c>
     </row>
     <row r="46" spans="1:7" ht="25.8" x14ac:dyDescent="0.3">
-      <c r="A46" s="49" t="s">
+      <c r="A46" s="55" t="s">
         <v>27</v>
       </c>
-      <c r="B46" s="49"/>
-      <c r="C46" s="49"/>
-      <c r="D46" s="49"/>
-      <c r="E46" s="49"/>
-      <c r="F46" s="49"/>
-      <c r="G46" s="49"/>
+      <c r="B46" s="55"/>
+      <c r="C46" s="55"/>
+      <c r="D46" s="55"/>
+      <c r="E46" s="55"/>
+      <c r="F46" s="55"/>
+      <c r="G46" s="55"/>
     </row>
     <row r="48" spans="1:7" ht="18" x14ac:dyDescent="0.3">
-      <c r="A48" s="50" t="s">
+      <c r="A48" s="56" t="s">
         <v>28</v>
       </c>
-      <c r="B48" s="50"/>
-      <c r="C48" s="50"/>
-      <c r="D48" s="50"/>
-      <c r="E48" s="50"/>
-      <c r="F48" s="50"/>
-      <c r="G48" s="50"/>
+      <c r="B48" s="56"/>
+      <c r="C48" s="56"/>
+      <c r="D48" s="56"/>
+      <c r="E48" s="56"/>
+      <c r="F48" s="56"/>
+      <c r="G48" s="56"/>
     </row>
     <row r="50" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A50" s="13" t="s">

</xml_diff>

<commit_message>
feat: validacion de datos - registro empleados, conditional formatting, antiguedad, correos
</commit_message>
<xml_diff>
--- a/EXCEL/Presupuesto Personal.xlsx
+++ b/EXCEL/Presupuesto Personal.xlsx
@@ -8,13 +8,15 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/1d86eecf8daf4f0d/Documents/SQL Server Management Studio 22/Tienda-sqlserver/EXCEL/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="2" documentId="8_{EE053816-48E3-4E91-A6AD-611A9303676C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{71C0AE0A-1937-4A33-91DE-38CE252A77EB}"/>
+  <xr:revisionPtr revIDLastSave="4" documentId="8_{EE053816-48E3-4E91-A6AD-611A9303676C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{2933B2D6-B1F1-4430-BB71-35C809E9BCE4}"/>
   <bookViews>
-    <workbookView xWindow="588" yWindow="336" windowWidth="11760" windowHeight="12240" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="1" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Personal-Budget_2026" sheetId="2" r:id="rId1"/>
-    <sheet name="Sheet1" sheetId="1" r:id="rId2"/>
+    <sheet name="Junio-2026" sheetId="1" r:id="rId2"/>
+    <sheet name="Resumen" sheetId="3" r:id="rId3"/>
+    <sheet name="Libros " sheetId="4" r:id="rId4"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -32,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="221" uniqueCount="172">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="321" uniqueCount="221">
   <si>
     <t xml:space="preserve">Cantidad </t>
   </si>
@@ -561,20 +563,169 @@
   <si>
     <t xml:space="preserve">Comprobante/Recibo </t>
   </si>
+  <si>
+    <t xml:space="preserve">Gastos </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Fecha </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Descripcion </t>
+  </si>
+  <si>
+    <t>Monto RD$</t>
+  </si>
+  <si>
+    <t>JUN 12, 2026</t>
+  </si>
+  <si>
+    <t>JUN 15, 2026</t>
+  </si>
+  <si>
+    <t>Salud</t>
+  </si>
+  <si>
+    <t>Temu</t>
+  </si>
+  <si>
+    <t>Dentista</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Compras online </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Comida </t>
+  </si>
+  <si>
+    <t>Almuerzo</t>
+  </si>
+  <si>
+    <t>JUN , 2026</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Transporte </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Salidas </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Gasto Normal Controlado </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sin Registro Aun </t>
+  </si>
+  <si>
+    <t>Gasto Mas Elevado, !Cuidad!</t>
+  </si>
+  <si>
+    <t>Total RD$</t>
+  </si>
+  <si>
+    <t>Comida</t>
+  </si>
+  <si>
+    <t>Transporte</t>
+  </si>
+  <si>
+    <t>Otros</t>
+  </si>
+  <si>
+    <t>Compras online</t>
+  </si>
+  <si>
+    <t>Salidas</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Diligencia </t>
+  </si>
+  <si>
+    <t>Fiestas</t>
+  </si>
+  <si>
+    <t>JUN 8, 2027</t>
+  </si>
+  <si>
+    <t>Vision</t>
+  </si>
+  <si>
+    <t>Resumen</t>
+  </si>
+  <si>
+    <t>Registro de Lectura 2026</t>
+  </si>
+  <si>
+    <t>Libro</t>
+  </si>
+  <si>
+    <t>Autor</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Fecha inicio </t>
+  </si>
+  <si>
+    <t>Fecha Fin</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Dias Invertidos </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Leccion Principal </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Calificacion ⭐  </t>
+  </si>
+  <si>
+    <t>#</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Padre Rico, Padre Pobre </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Habitos Atomicos </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Deja de Ser Tu </t>
+  </si>
+  <si>
+    <t>La Psicologia del Dinero</t>
+  </si>
+  <si>
+    <t>Robert Kiyosaki</t>
+  </si>
+  <si>
+    <t xml:space="preserve">James Clear </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Joe Dispenza </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Morgan Housel </t>
+  </si>
+  <si>
+    <t>04/15/2026</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Done </t>
+  </si>
+  <si>
+    <t>Leyendo</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="6">
+  <numFmts count="8">
+    <numFmt numFmtId="44" formatCode="_-&quot;XDR&quot;* #,##0.00_-;\-&quot;XDR&quot;* #,##0.00_-;_-&quot;XDR&quot;* &quot;-&quot;??_-;_-@_-"/>
     <numFmt numFmtId="43" formatCode="_-* #,##0.00_-;\-* #,##0.00_-;_-* &quot;-&quot;??_-;_-@_-"/>
     <numFmt numFmtId="164" formatCode="_-[$$-409]* #,##0.00_ ;_-[$$-409]* \-#,##0.00\ ;_-[$$-409]* &quot;-&quot;??_ ;_-@_ "/>
     <numFmt numFmtId="165" formatCode="_-[$$-409]* #,##0.000_ ;_-[$$-409]* \-#,##0.000\ ;_-[$$-409]* &quot;-&quot;??_ ;_-@_ "/>
     <numFmt numFmtId="166" formatCode="_-* #,##0.0_-;\-* #,##0.0_-;_-* &quot;-&quot;??_-;_-@_-"/>
     <numFmt numFmtId="167" formatCode="_-[$$-2C0A]\ * #,##0.00_-;\-[$$-2C0A]\ * #,##0.00_-;_-[$$-2C0A]\ * &quot;-&quot;??_-;_-@_-"/>
-    <numFmt numFmtId="173" formatCode="dd/mm/yyyy;@"/>
+    <numFmt numFmtId="168" formatCode="dd/mm/yyyy;@"/>
+    <numFmt numFmtId="170" formatCode="mm/dd/yyyy;@"/>
   </numFmts>
-  <fonts count="14" x14ac:knownFonts="1">
+  <fonts count="20" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -674,8 +825,51 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="5"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="7"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="7"/>
+      <name val="Stencil"/>
+      <family val="5"/>
+    </font>
   </fonts>
-  <fills count="17">
+  <fills count="20">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -772,8 +966,26 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.79998168889431442"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="3"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF002060"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="2">
+  <borders count="4">
     <border>
       <left/>
       <right/>
@@ -796,15 +1008,36 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
-  <cellStyleXfs count="3">
+  <cellStyleXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="44" fontId="14" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="67">
+  <cellXfs count="107">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -943,6 +1176,96 @@
     <xf numFmtId="17" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="168" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="168" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="43" fontId="0" fillId="0" borderId="1" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="16" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="16" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="16" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="16" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="167" fontId="13" fillId="0" borderId="1" xfId="3" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="12" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="167" fontId="15" fillId="0" borderId="1" xfId="3" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="12" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="167" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="12" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="167" fontId="15" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="17" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="167" fontId="15" fillId="14" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="167" fontId="16" fillId="14" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="9" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -961,6 +1284,12 @@
     <xf numFmtId="0" fontId="9" fillId="12" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -976,43 +1305,187 @@
     <xf numFmtId="0" fontId="8" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="170" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="168" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="170" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="168" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="170" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="173" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1">
+    <xf numFmtId="170" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="173" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="43" fontId="0" fillId="0" borderId="1" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="14" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="16" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="19" fillId="18" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="19" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="19" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="16" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="170" fontId="18" fillId="19" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="16" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="16" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
+    <xf numFmtId="14" fontId="18" fillId="19" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
-  <cellStyles count="3">
+  <cellStyles count="4">
     <cellStyle name="Comma" xfId="2" builtinId="3"/>
+    <cellStyle name="Currency" xfId="3" builtinId="4"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
     <cellStyle name="Percent" xfId="1" builtinId="5"/>
   </cellStyles>
-  <dxfs count="0"/>
+  <dxfs count="16">
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF0000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF0000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFFF00"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF00B050"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFFF00"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF00B050"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF0000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF0000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF0000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFFF00"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF00B050"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFFF00"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF00B050"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF0000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+  </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
@@ -1137,7 +1610,7 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Sheet1!$D$20:$D$28</c:f>
+              <c:f>'Junio-2026'!$D$20:$D$28</c:f>
               <c:numCache>
                 <c:formatCode>_-[$$-409]* #,##0.00_ ;_-[$$-409]* \-#,##0.00\ ;_-[$$-409]* "-"??_ ;_-@_ </c:formatCode>
                 <c:ptCount val="9"/>
@@ -1182,7 +1655,7 @@
           <c:order val="1"/>
           <c:tx>
             <c:strRef>
-              <c:f>Sheet1!$A$34:$A$42</c:f>
+              <c:f>'Junio-2026'!$A$34:$A$42</c:f>
               <c:strCache>
                 <c:ptCount val="9"/>
                 <c:pt idx="0">
@@ -1310,7 +1783,7 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Sheet1!$D$34:$D$42</c:f>
+              <c:f>'Junio-2026'!$D$34:$D$42</c:f>
               <c:numCache>
                 <c:formatCode>_-[$$-409]* #,##0.00_ ;_-[$$-409]* \-#,##0.00\ ;_-[$$-409]* "-"??_ ;_-@_ </c:formatCode>
                 <c:ptCount val="9"/>
@@ -1355,7 +1828,7 @@
           <c:order val="3"/>
           <c:tx>
             <c:strRef>
-              <c:f>Sheet1!$A$20:$A$28</c:f>
+              <c:f>'Junio-2026'!$A$20:$A$28</c:f>
               <c:strCache>
                 <c:ptCount val="9"/>
                 <c:pt idx="0">
@@ -2838,26 +3311,26 @@
       </c>
     </row>
     <row r="6" spans="1:18" ht="31.2" x14ac:dyDescent="0.3">
-      <c r="A6" s="47" t="s">
+      <c r="A6" s="77" t="s">
         <v>46</v>
       </c>
-      <c r="B6" s="47"/>
-      <c r="C6" s="47"/>
-      <c r="D6" s="47"/>
-      <c r="E6" s="47"/>
-      <c r="F6" s="47"/>
-      <c r="G6" s="47"/>
-      <c r="H6" s="47"/>
-      <c r="I6" s="47"/>
-      <c r="J6" s="47"/>
-      <c r="K6" s="47"/>
-      <c r="L6" s="47"/>
-      <c r="M6" s="47"/>
-      <c r="N6" s="47"/>
-      <c r="O6" s="47"/>
-      <c r="P6" s="47"/>
-      <c r="Q6" s="47"/>
-      <c r="R6" s="47"/>
+      <c r="B6" s="77"/>
+      <c r="C6" s="77"/>
+      <c r="D6" s="77"/>
+      <c r="E6" s="77"/>
+      <c r="F6" s="77"/>
+      <c r="G6" s="77"/>
+      <c r="H6" s="77"/>
+      <c r="I6" s="77"/>
+      <c r="J6" s="77"/>
+      <c r="K6" s="77"/>
+      <c r="L6" s="77"/>
+      <c r="M6" s="77"/>
+      <c r="N6" s="77"/>
+      <c r="O6" s="77"/>
+      <c r="P6" s="77"/>
+      <c r="Q6" s="77"/>
+      <c r="R6" s="77"/>
     </row>
     <row r="8" spans="1:18" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A8" s="34" t="s">
@@ -3094,20 +3567,20 @@
       </c>
     </row>
     <row r="20" spans="1:14" ht="31.2" x14ac:dyDescent="0.3">
-      <c r="A20" s="48" t="s">
+      <c r="A20" s="78" t="s">
         <v>79</v>
       </c>
-      <c r="B20" s="48"/>
-      <c r="C20" s="48"/>
-      <c r="D20" s="48"/>
-      <c r="E20" s="48"/>
-      <c r="F20" s="48"/>
-      <c r="G20" s="48"/>
-      <c r="H20" s="48"/>
-      <c r="I20" s="48"/>
-      <c r="J20" s="48"/>
-      <c r="K20" s="48"/>
-      <c r="L20" s="48"/>
+      <c r="B20" s="78"/>
+      <c r="C20" s="78"/>
+      <c r="D20" s="78"/>
+      <c r="E20" s="78"/>
+      <c r="F20" s="78"/>
+      <c r="G20" s="78"/>
+      <c r="H20" s="78"/>
+      <c r="I20" s="78"/>
+      <c r="J20" s="78"/>
+      <c r="K20" s="78"/>
+      <c r="L20" s="78"/>
       <c r="N20" s="16" t="s">
         <v>90</v>
       </c>
@@ -3274,20 +3747,20 @@
       </c>
     </row>
     <row r="33" spans="1:12" ht="31.2" x14ac:dyDescent="0.3">
-      <c r="A33" s="49" t="s">
+      <c r="A33" s="79" t="s">
         <v>107</v>
       </c>
-      <c r="B33" s="49"/>
-      <c r="C33" s="49"/>
-      <c r="D33" s="49"/>
-      <c r="E33" s="49"/>
-      <c r="F33" s="49"/>
-      <c r="G33" s="49"/>
-      <c r="H33" s="49"/>
-      <c r="I33" s="49"/>
-      <c r="J33" s="49"/>
-      <c r="K33" s="49"/>
-      <c r="L33" s="49"/>
+      <c r="B33" s="79"/>
+      <c r="C33" s="79"/>
+      <c r="D33" s="79"/>
+      <c r="E33" s="79"/>
+      <c r="F33" s="79"/>
+      <c r="G33" s="79"/>
+      <c r="H33" s="79"/>
+      <c r="I33" s="79"/>
+      <c r="J33" s="79"/>
+      <c r="K33" s="79"/>
+      <c r="L33" s="79"/>
     </row>
     <row r="35" spans="1:12" ht="23.4" x14ac:dyDescent="0.3">
       <c r="A35" s="16" t="s">
@@ -3295,20 +3768,20 @@
       </c>
     </row>
     <row r="37" spans="1:12" ht="31.2" x14ac:dyDescent="0.3">
-      <c r="A37" s="50" t="s">
+      <c r="A37" s="80" t="s">
         <v>98</v>
       </c>
-      <c r="B37" s="50"/>
-      <c r="C37" s="50"/>
-      <c r="D37" s="50"/>
-      <c r="E37" s="50"/>
-      <c r="F37" s="50"/>
-      <c r="G37" s="50"/>
-      <c r="H37" s="50"/>
-      <c r="I37" s="50"/>
-      <c r="J37" s="50"/>
-      <c r="K37" s="50"/>
-      <c r="L37" s="50"/>
+      <c r="B37" s="80"/>
+      <c r="C37" s="80"/>
+      <c r="D37" s="80"/>
+      <c r="E37" s="80"/>
+      <c r="F37" s="80"/>
+      <c r="G37" s="80"/>
+      <c r="H37" s="80"/>
+      <c r="I37" s="80"/>
+      <c r="J37" s="80"/>
+      <c r="K37" s="80"/>
+      <c r="L37" s="80"/>
     </row>
     <row r="39" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A39" s="35" t="s">
@@ -3425,16 +3898,16 @@
       </c>
     </row>
     <row r="51" spans="1:9" ht="31.2" x14ac:dyDescent="0.3">
-      <c r="A51" s="51" t="s">
+      <c r="A51" s="81" t="s">
         <v>109</v>
       </c>
-      <c r="B51" s="51"/>
-      <c r="C51" s="51"/>
-      <c r="D51" s="51"/>
-      <c r="E51" s="51"/>
-      <c r="F51" s="51"/>
-      <c r="G51" s="51"/>
-      <c r="H51" s="51"/>
+      <c r="B51" s="81"/>
+      <c r="C51" s="81"/>
+      <c r="D51" s="81"/>
+      <c r="E51" s="81"/>
+      <c r="F51" s="81"/>
+      <c r="G51" s="81"/>
+      <c r="H51" s="81"/>
       <c r="I51" s="40"/>
     </row>
     <row r="53" spans="1:9" ht="28.8" x14ac:dyDescent="0.3">
@@ -3501,18 +3974,18 @@
       </c>
     </row>
     <row r="66" spans="1:10" ht="31.2" x14ac:dyDescent="0.3">
-      <c r="A66" s="46" t="s">
+      <c r="A66" s="76" t="s">
         <v>117</v>
       </c>
-      <c r="B66" s="46"/>
-      <c r="C66" s="46"/>
-      <c r="D66" s="46"/>
-      <c r="E66" s="46"/>
-      <c r="F66" s="46"/>
-      <c r="G66" s="46"/>
-      <c r="H66" s="46"/>
-      <c r="I66" s="46"/>
-      <c r="J66" s="46"/>
+      <c r="B66" s="76"/>
+      <c r="C66" s="76"/>
+      <c r="D66" s="76"/>
+      <c r="E66" s="76"/>
+      <c r="F66" s="76"/>
+      <c r="G66" s="76"/>
+      <c r="H66" s="76"/>
+      <c r="I66" s="76"/>
+      <c r="J66" s="76"/>
     </row>
     <row r="68" spans="1:10" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A68" s="23" t="s">
@@ -3695,75 +4168,75 @@
       </c>
     </row>
     <row r="77" spans="1:10" ht="18" x14ac:dyDescent="0.3">
-      <c r="A77" s="58" t="s">
+      <c r="A77" s="75" t="s">
         <v>165</v>
       </c>
-      <c r="B77" s="58"/>
-      <c r="C77" s="58"/>
-      <c r="D77" s="57"/>
-      <c r="E77" s="57"/>
+      <c r="B77" s="75"/>
+      <c r="C77" s="75"/>
+      <c r="D77" s="46"/>
+      <c r="E77" s="46"/>
     </row>
     <row r="79" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A79" s="59" t="s">
+      <c r="A79" s="47" t="s">
         <v>146</v>
       </c>
-      <c r="B79" s="59" t="s">
+      <c r="B79" s="47" t="s">
         <v>147</v>
       </c>
-      <c r="C79" s="59" t="s">
+      <c r="C79" s="47" t="s">
         <v>148</v>
       </c>
-      <c r="D79" s="59" t="s">
+      <c r="D79" s="47" t="s">
         <v>149</v>
       </c>
-      <c r="E79" s="59" t="s">
+      <c r="E79" s="47" t="s">
         <v>150</v>
       </c>
-      <c r="F79" s="59" t="s">
+      <c r="F79" s="47" t="s">
         <v>151</v>
       </c>
-      <c r="G79" s="59" t="s">
+      <c r="G79" s="47" t="s">
         <v>167</v>
       </c>
-      <c r="H79" s="59" t="s">
+      <c r="H79" s="47" t="s">
         <v>168</v>
       </c>
-      <c r="I79" s="59" t="s">
+      <c r="I79" s="47" t="s">
         <v>169</v>
       </c>
-      <c r="J79" s="59" t="s">
+      <c r="J79" s="47" t="s">
         <v>170</v>
       </c>
     </row>
     <row r="80" spans="1:10" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A80" s="63" t="s">
+      <c r="A80" s="51" t="s">
         <v>152</v>
       </c>
-      <c r="B80" s="63" t="s">
+      <c r="B80" s="51" t="s">
         <v>153</v>
       </c>
-      <c r="C80" s="64" t="s">
+      <c r="C80" s="52" t="s">
         <v>154</v>
       </c>
-      <c r="D80" s="64" t="s">
+      <c r="D80" s="52" t="s">
         <v>161</v>
       </c>
-      <c r="E80" s="64" t="s">
+      <c r="E80" s="52" t="s">
         <v>162</v>
       </c>
-      <c r="F80" s="63" t="s">
+      <c r="F80" s="51" t="s">
         <v>155</v>
       </c>
-      <c r="G80" s="64" t="s">
+      <c r="G80" s="52" t="s">
         <v>156</v>
       </c>
-      <c r="H80" s="65" t="s">
+      <c r="H80" s="53" t="s">
         <v>157</v>
       </c>
-      <c r="I80" s="66" t="s">
+      <c r="I80" s="54" t="s">
         <v>171</v>
       </c>
-      <c r="J80" s="64" t="s">
+      <c r="J80" s="52" t="s">
         <v>158</v>
       </c>
     </row>
@@ -3774,23 +4247,23 @@
       <c r="B81" s="2" t="s">
         <v>160</v>
       </c>
-      <c r="C81" s="60">
+      <c r="C81" s="48">
         <v>46181</v>
       </c>
-      <c r="D81" s="60" t="s">
+      <c r="D81" s="48" t="s">
         <v>163</v>
       </c>
-      <c r="E81" s="61" t="s">
+      <c r="E81" s="49" t="s">
         <v>164</v>
       </c>
-      <c r="F81" s="62">
+      <c r="F81" s="50">
         <v>3800</v>
       </c>
       <c r="G81" s="2"/>
-      <c r="H81" s="60">
+      <c r="H81" s="48">
         <v>46184</v>
       </c>
-      <c r="I81" s="60"/>
+      <c r="I81" s="48"/>
       <c r="J81" s="2" t="s">
         <v>166</v>
       </c>
@@ -3844,7 +4317,10 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A65ADDB5-C914-4D41-B3AC-1DECB4CEAAB9}">
-  <dimension ref="A1:G54"/>
+  <sheetPr>
+    <tabColor theme="1"/>
+  </sheetPr>
+  <dimension ref="A1:G96"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="17.33203125" customWidth="1"/>
@@ -3856,11 +4332,11 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:4" ht="18" x14ac:dyDescent="0.3">
-      <c r="A1" s="52" t="s">
+      <c r="A1" s="84" t="s">
         <v>4</v>
       </c>
-      <c r="B1" s="53"/>
-      <c r="C1" s="53"/>
+      <c r="B1" s="85"/>
+      <c r="C1" s="85"/>
     </row>
     <row r="2" spans="1:4" ht="15" x14ac:dyDescent="0.3">
       <c r="B2" s="1"/>
@@ -4001,11 +4477,11 @@
       <c r="C16" s="8"/>
     </row>
     <row r="17" spans="1:4" ht="21" x14ac:dyDescent="0.3">
-      <c r="A17" s="54" t="s">
+      <c r="A17" s="86" t="s">
         <v>13</v>
       </c>
-      <c r="B17" s="54"/>
-      <c r="C17" s="54"/>
+      <c r="B17" s="86"/>
+      <c r="C17" s="86"/>
     </row>
     <row r="19" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A19" s="12" t="s">
@@ -4157,11 +4633,11 @@
       </c>
     </row>
     <row r="31" spans="1:4" ht="21" x14ac:dyDescent="0.3">
-      <c r="A31" s="54" t="s">
+      <c r="A31" s="86" t="s">
         <v>13</v>
       </c>
-      <c r="B31" s="54"/>
-      <c r="C31" s="54"/>
+      <c r="B31" s="86"/>
+      <c r="C31" s="86"/>
     </row>
     <row r="33" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A33" s="12" t="s">
@@ -4313,26 +4789,26 @@
       </c>
     </row>
     <row r="46" spans="1:7" ht="25.8" x14ac:dyDescent="0.3">
-      <c r="A46" s="55" t="s">
+      <c r="A46" s="87" t="s">
         <v>27</v>
       </c>
-      <c r="B46" s="55"/>
-      <c r="C46" s="55"/>
-      <c r="D46" s="55"/>
-      <c r="E46" s="55"/>
-      <c r="F46" s="55"/>
-      <c r="G46" s="55"/>
+      <c r="B46" s="87"/>
+      <c r="C46" s="87"/>
+      <c r="D46" s="87"/>
+      <c r="E46" s="87"/>
+      <c r="F46" s="87"/>
+      <c r="G46" s="87"/>
     </row>
     <row r="48" spans="1:7" ht="18" x14ac:dyDescent="0.3">
-      <c r="A48" s="56" t="s">
+      <c r="A48" s="88" t="s">
         <v>28</v>
       </c>
-      <c r="B48" s="56"/>
-      <c r="C48" s="56"/>
-      <c r="D48" s="56"/>
-      <c r="E48" s="56"/>
-      <c r="F48" s="56"/>
-      <c r="G48" s="56"/>
+      <c r="B48" s="88"/>
+      <c r="C48" s="88"/>
+      <c r="D48" s="88"/>
+      <c r="E48" s="88"/>
+      <c r="F48" s="88"/>
+      <c r="G48" s="88"/>
     </row>
     <row r="50" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A50" s="13" t="s">
@@ -4457,16 +4933,787 @@
         <v>REPROBADO</v>
       </c>
     </row>
+    <row r="78" spans="1:5" ht="18" x14ac:dyDescent="0.3">
+      <c r="A78" s="57" t="s">
+        <v>172</v>
+      </c>
+      <c r="B78" s="58"/>
+      <c r="C78" s="58"/>
+      <c r="D78" s="58"/>
+    </row>
+    <row r="79" spans="1:5" ht="18" x14ac:dyDescent="0.3">
+      <c r="A79" s="61" t="s">
+        <v>173</v>
+      </c>
+      <c r="B79" s="61" t="s">
+        <v>153</v>
+      </c>
+      <c r="C79" s="61" t="s">
+        <v>174</v>
+      </c>
+      <c r="D79" s="61" t="s">
+        <v>175</v>
+      </c>
+    </row>
+    <row r="80" spans="1:5" ht="18" x14ac:dyDescent="0.3">
+      <c r="A80" s="59" t="s">
+        <v>176</v>
+      </c>
+      <c r="B80" s="59" t="s">
+        <v>178</v>
+      </c>
+      <c r="C80" s="59" t="s">
+        <v>180</v>
+      </c>
+      <c r="D80" s="60">
+        <v>1000</v>
+      </c>
+      <c r="E80" s="64" t="s">
+        <v>187</v>
+      </c>
+    </row>
+    <row r="81" spans="1:7" ht="18" x14ac:dyDescent="0.3">
+      <c r="A81" s="59" t="s">
+        <v>177</v>
+      </c>
+      <c r="B81" s="59" t="s">
+        <v>181</v>
+      </c>
+      <c r="C81" s="59" t="s">
+        <v>179</v>
+      </c>
+      <c r="D81" s="60">
+        <v>1083</v>
+      </c>
+      <c r="E81" s="82" t="s">
+        <v>189</v>
+      </c>
+      <c r="F81" s="83"/>
+      <c r="G81" s="83"/>
+    </row>
+    <row r="82" spans="1:7" ht="18" x14ac:dyDescent="0.3">
+      <c r="A82" s="59" t="s">
+        <v>184</v>
+      </c>
+      <c r="B82" s="59" t="s">
+        <v>182</v>
+      </c>
+      <c r="C82" s="59" t="s">
+        <v>183</v>
+      </c>
+      <c r="D82" s="60">
+        <v>0</v>
+      </c>
+      <c r="E82" s="64" t="s">
+        <v>188</v>
+      </c>
+    </row>
+    <row r="83" spans="1:7" ht="18" x14ac:dyDescent="0.3">
+      <c r="A83" s="59" t="s">
+        <v>184</v>
+      </c>
+      <c r="B83" s="59" t="s">
+        <v>195</v>
+      </c>
+      <c r="C83" s="59" t="s">
+        <v>197</v>
+      </c>
+      <c r="D83" s="60">
+        <v>0</v>
+      </c>
+      <c r="E83" s="58"/>
+    </row>
+    <row r="84" spans="1:7" ht="18" x14ac:dyDescent="0.3">
+      <c r="A84" s="59" t="s">
+        <v>198</v>
+      </c>
+      <c r="B84" s="59" t="s">
+        <v>178</v>
+      </c>
+      <c r="C84" s="59" t="s">
+        <v>199</v>
+      </c>
+      <c r="D84" s="60">
+        <v>3800</v>
+      </c>
+      <c r="E84" s="58"/>
+    </row>
+    <row r="85" spans="1:7" ht="18" x14ac:dyDescent="0.3">
+      <c r="A85" s="59" t="s">
+        <v>184</v>
+      </c>
+      <c r="B85" s="59" t="s">
+        <v>185</v>
+      </c>
+      <c r="C85" s="59" t="s">
+        <v>196</v>
+      </c>
+      <c r="D85" s="60">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="88" spans="1:7" ht="18" x14ac:dyDescent="0.3">
+      <c r="A88" s="58" t="s">
+        <v>200</v>
+      </c>
+      <c r="C88" s="66"/>
+    </row>
+    <row r="89" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A89" s="65" t="s">
+        <v>153</v>
+      </c>
+      <c r="B89" s="65" t="s">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="90" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A90" s="2" t="s">
+        <v>191</v>
+      </c>
+      <c r="B90" s="2">
+        <f>SUMIF('Junio-2026'!C:C,"Comida",'Junio-2026'!D:D)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="91" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A91" s="2" t="s">
+        <v>192</v>
+      </c>
+      <c r="B91" s="2">
+        <f>SUMIF('Junio-2026'!C:C,"Transporte",'Junio-2026'!D:D)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="92" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A92" s="2" t="s">
+        <v>178</v>
+      </c>
+      <c r="B92" s="2"/>
+    </row>
+    <row r="93" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A93" s="2" t="s">
+        <v>194</v>
+      </c>
+      <c r="B93" s="2">
+        <f>SUMIF('Junio-2026'!B167:B172,"Compras online", 'Junio-2026'!D167:D172)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="94" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A94" s="2" t="s">
+        <v>186</v>
+      </c>
+      <c r="B94" s="2">
+        <f>SUMIF('Junio-2026'!B167:B172,"Compras online", 'Junio-2026'!D167:D172)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="95" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A95" s="2" t="s">
+        <v>178</v>
+      </c>
+      <c r="B95" s="2">
+        <f>SUMIF('Junio-2026'!B167:B172,"Salud",'Junio-2026'!D167:D172)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="96" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A96" s="2" t="s">
+        <v>193</v>
+      </c>
+      <c r="B96" s="2"/>
+    </row>
   </sheetData>
-  <mergeCells count="5">
+  <mergeCells count="6">
+    <mergeCell ref="E81:G81"/>
     <mergeCell ref="A1:C1"/>
     <mergeCell ref="A17:C17"/>
     <mergeCell ref="A31:C31"/>
     <mergeCell ref="A46:G46"/>
     <mergeCell ref="A48:G48"/>
   </mergeCells>
+  <phoneticPr fontId="11" type="noConversion"/>
+  <conditionalFormatting sqref="D80:D85">
+    <cfRule type="cellIs" dxfId="15" priority="11" operator="greaterThan">
+      <formula>1050</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="14" priority="12" operator="greaterThan">
+      <formula>500</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="13" priority="13" operator="lessThan">
+      <formula>500</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="12" priority="14" operator="lessThan">
+      <formula>500</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="11" priority="15" operator="greaterThan">
+      <formula>1050</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="10" priority="16" operator="greaterThan">
+      <formula>500</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="9" priority="17" operator="greaterThan">
+      <formula>1000</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="8" priority="18" operator="greaterThan">
+      <formula>" $ 1,100.00"</formula>
+    </cfRule>
+    <cfRule type="colorScale" priority="19">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="max"/>
+        <color rgb="FFFF7128"/>
+        <color rgb="FFFFEF9C"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
   <drawing r:id="rId2"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B76DEFF3-7E62-4F9E-9708-A59A85B67BFA}">
+  <sheetPr>
+    <tabColor rgb="FFFF0000"/>
+  </sheetPr>
+  <dimension ref="A2:G20"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="17.77734375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="17.88671875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="14.109375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="16.21875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="28.44140625" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="2" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A2" s="56" t="s">
+        <v>172</v>
+      </c>
+      <c r="B2" s="55"/>
+      <c r="C2" s="55"/>
+      <c r="D2" s="55"/>
+      <c r="E2" s="55"/>
+      <c r="F2" s="55"/>
+      <c r="G2" s="55"/>
+    </row>
+    <row r="3" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A3" s="67" t="s">
+        <v>173</v>
+      </c>
+      <c r="B3" s="67" t="s">
+        <v>153</v>
+      </c>
+      <c r="C3" s="67" t="s">
+        <v>174</v>
+      </c>
+      <c r="D3" s="67" t="s">
+        <v>175</v>
+      </c>
+      <c r="E3" s="55"/>
+      <c r="F3" s="55"/>
+      <c r="G3" s="55"/>
+    </row>
+    <row r="4" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A4" s="63" t="s">
+        <v>176</v>
+      </c>
+      <c r="B4" s="63" t="s">
+        <v>178</v>
+      </c>
+      <c r="C4" s="63" t="s">
+        <v>180</v>
+      </c>
+      <c r="D4" s="62">
+        <v>1000</v>
+      </c>
+      <c r="E4" s="68" t="s">
+        <v>187</v>
+      </c>
+      <c r="F4" s="55"/>
+      <c r="G4" s="55"/>
+    </row>
+    <row r="5" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A5" s="63" t="s">
+        <v>177</v>
+      </c>
+      <c r="B5" s="63" t="s">
+        <v>181</v>
+      </c>
+      <c r="C5" s="63" t="s">
+        <v>179</v>
+      </c>
+      <c r="D5" s="62">
+        <v>1083</v>
+      </c>
+      <c r="E5" s="73" t="s">
+        <v>189</v>
+      </c>
+      <c r="F5" s="74"/>
+      <c r="G5" s="74"/>
+    </row>
+    <row r="6" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A6" s="63" t="s">
+        <v>184</v>
+      </c>
+      <c r="B6" s="63" t="s">
+        <v>182</v>
+      </c>
+      <c r="C6" s="63" t="s">
+        <v>183</v>
+      </c>
+      <c r="D6" s="62">
+        <v>0</v>
+      </c>
+      <c r="E6" s="68" t="s">
+        <v>188</v>
+      </c>
+      <c r="F6" s="55"/>
+      <c r="G6" s="55"/>
+    </row>
+    <row r="7" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A7" s="63" t="s">
+        <v>184</v>
+      </c>
+      <c r="B7" s="63" t="s">
+        <v>195</v>
+      </c>
+      <c r="C7" s="63" t="s">
+        <v>197</v>
+      </c>
+      <c r="D7" s="62">
+        <v>0</v>
+      </c>
+      <c r="E7" s="55"/>
+      <c r="F7" s="55"/>
+      <c r="G7" s="55"/>
+    </row>
+    <row r="8" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A8" s="63" t="s">
+        <v>198</v>
+      </c>
+      <c r="B8" s="63" t="s">
+        <v>178</v>
+      </c>
+      <c r="C8" s="63" t="s">
+        <v>199</v>
+      </c>
+      <c r="D8" s="62">
+        <v>3800</v>
+      </c>
+      <c r="E8" s="55"/>
+      <c r="F8" s="55"/>
+      <c r="G8" s="55"/>
+    </row>
+    <row r="9" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A9" s="63" t="s">
+        <v>184</v>
+      </c>
+      <c r="B9" s="63" t="s">
+        <v>185</v>
+      </c>
+      <c r="C9" s="63" t="s">
+        <v>196</v>
+      </c>
+      <c r="D9" s="62">
+        <v>0</v>
+      </c>
+      <c r="E9" s="55"/>
+      <c r="F9" s="55"/>
+      <c r="G9" s="55"/>
+    </row>
+    <row r="10" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A10" s="55"/>
+      <c r="B10" s="55"/>
+      <c r="C10" s="55"/>
+      <c r="D10" s="55"/>
+      <c r="E10" s="55"/>
+      <c r="F10" s="55"/>
+      <c r="G10" s="55"/>
+    </row>
+    <row r="11" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A11" s="55"/>
+      <c r="B11" s="55"/>
+      <c r="C11" s="55"/>
+      <c r="D11" s="55"/>
+      <c r="E11" s="55"/>
+      <c r="F11" s="55"/>
+      <c r="G11" s="55"/>
+    </row>
+    <row r="12" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A12" s="55" t="s">
+        <v>200</v>
+      </c>
+      <c r="B12" s="55"/>
+      <c r="C12" s="69"/>
+      <c r="D12" s="55"/>
+      <c r="E12" s="55"/>
+      <c r="F12" s="55"/>
+      <c r="G12" s="55"/>
+    </row>
+    <row r="13" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A13" s="67" t="s">
+        <v>153</v>
+      </c>
+      <c r="B13" s="67" t="s">
+        <v>190</v>
+      </c>
+      <c r="C13" s="55"/>
+      <c r="D13" s="55"/>
+      <c r="E13" s="55"/>
+      <c r="F13" s="55"/>
+      <c r="G13" s="55"/>
+    </row>
+    <row r="14" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A14" s="70" t="s">
+        <v>181</v>
+      </c>
+      <c r="B14" s="71">
+        <f ca="1">SUMIF($B$4:$B$9, A14, $D$4:$D$8)</f>
+        <v>1083</v>
+      </c>
+      <c r="C14" s="55"/>
+      <c r="D14" s="55"/>
+      <c r="E14" s="55"/>
+      <c r="F14" s="55"/>
+      <c r="G14" s="55"/>
+    </row>
+    <row r="15" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A15" s="70" t="s">
+        <v>191</v>
+      </c>
+      <c r="B15" s="71">
+        <f t="shared" ref="B15:B18" ca="1" si="0">SUMIF($B$4:$B$9, A15, $D$4:$D$8)</f>
+        <v>0</v>
+      </c>
+      <c r="C15" s="55"/>
+      <c r="D15" s="55"/>
+      <c r="E15" s="55"/>
+      <c r="F15" s="55"/>
+      <c r="G15" s="55"/>
+    </row>
+    <row r="16" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A16" s="70" t="s">
+        <v>192</v>
+      </c>
+      <c r="B16" s="71">
+        <f t="shared" ca="1" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="C16" s="55"/>
+      <c r="D16" s="55"/>
+      <c r="E16" s="55"/>
+      <c r="F16" s="55"/>
+      <c r="G16" s="55"/>
+    </row>
+    <row r="17" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A17" s="70" t="s">
+        <v>178</v>
+      </c>
+      <c r="B17" s="71">
+        <f t="shared" ca="1" si="0"/>
+        <v>4800</v>
+      </c>
+      <c r="C17" s="55"/>
+      <c r="D17" s="55"/>
+      <c r="E17" s="55"/>
+      <c r="F17" s="55"/>
+      <c r="G17" s="55"/>
+    </row>
+    <row r="18" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A18" s="70" t="s">
+        <v>186</v>
+      </c>
+      <c r="B18" s="71">
+        <f t="shared" ca="1" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="C18" s="55"/>
+      <c r="D18" s="55"/>
+      <c r="E18" s="55"/>
+      <c r="F18" s="55"/>
+      <c r="G18" s="55"/>
+    </row>
+    <row r="19" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A19" s="70" t="s">
+        <v>193</v>
+      </c>
+      <c r="B19" s="72">
+        <f ca="1">+SUM(B14:B18)</f>
+        <v>5883</v>
+      </c>
+      <c r="C19" s="55"/>
+      <c r="D19" s="55"/>
+      <c r="E19" s="55"/>
+      <c r="F19" s="55"/>
+      <c r="G19" s="55"/>
+    </row>
+    <row r="20" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A20" s="55"/>
+      <c r="B20" s="55"/>
+      <c r="C20" s="55"/>
+      <c r="D20" s="55"/>
+      <c r="E20" s="55"/>
+      <c r="F20" s="55"/>
+      <c r="G20" s="55"/>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="E5:G5"/>
+  </mergeCells>
+  <conditionalFormatting sqref="D4:D9">
+    <cfRule type="cellIs" dxfId="7" priority="1" operator="greaterThan">
+      <formula>1050</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="6" priority="2" operator="greaterThan">
+      <formula>500</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="5" priority="3" operator="lessThan">
+      <formula>500</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="4" priority="4" operator="lessThan">
+      <formula>500</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="3" priority="5" operator="greaterThan">
+      <formula>1050</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="2" priority="6" operator="greaterThan">
+      <formula>500</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="1" priority="7" operator="greaterThan">
+      <formula>1000</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="0" priority="8" operator="greaterThan">
+      <formula>" $ 1,100.00"</formula>
+    </cfRule>
+    <cfRule type="colorScale" priority="9">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="max"/>
+        <color rgb="FFFF7128"/>
+        <color rgb="FFFFEF9C"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CFFFD5F3-00B0-4AD2-8853-B354DEE4CC20}">
+  <sheetPr>
+    <tabColor rgb="FF002060"/>
+  </sheetPr>
+  <dimension ref="A1:I20"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="2.109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="27.77734375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="13.6640625" style="89" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="10.5546875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="10.5546875" style="92" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="13.109375" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="9.109375" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="10.44140625" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="14.6640625" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:9" ht="18" x14ac:dyDescent="0.3">
+      <c r="B1" s="57" t="s">
+        <v>201</v>
+      </c>
+      <c r="D1" s="93"/>
+    </row>
+    <row r="2" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A2" s="98"/>
+      <c r="B2" s="98"/>
+      <c r="C2" s="99"/>
+      <c r="D2" s="100"/>
+      <c r="E2" s="101"/>
+      <c r="F2" s="98"/>
+      <c r="G2" s="98"/>
+      <c r="H2" s="98"/>
+      <c r="I2" s="98"/>
+    </row>
+    <row r="3" spans="1:9" s="90" customFormat="1" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A3" s="102" t="s">
+        <v>209</v>
+      </c>
+      <c r="B3" s="103" t="s">
+        <v>202</v>
+      </c>
+      <c r="C3" s="104" t="s">
+        <v>203</v>
+      </c>
+      <c r="D3" s="105" t="s">
+        <v>204</v>
+      </c>
+      <c r="E3" s="106" t="s">
+        <v>205</v>
+      </c>
+      <c r="F3" s="103" t="s">
+        <v>206</v>
+      </c>
+      <c r="G3" s="103" t="s">
+        <v>56</v>
+      </c>
+      <c r="H3" s="103" t="s">
+        <v>208</v>
+      </c>
+      <c r="I3" s="103" t="s">
+        <v>207</v>
+      </c>
+    </row>
+    <row r="4" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A4" s="42">
+        <v>1</v>
+      </c>
+      <c r="B4" s="2" t="s">
+        <v>210</v>
+      </c>
+      <c r="C4" s="18" t="s">
+        <v>214</v>
+      </c>
+      <c r="D4" s="48" t="s">
+        <v>218</v>
+      </c>
+      <c r="E4" s="48">
+        <v>46154</v>
+      </c>
+      <c r="F4" s="2"/>
+      <c r="G4" s="2" t="s">
+        <v>219</v>
+      </c>
+      <c r="H4" s="14">
+        <v>4</v>
+      </c>
+      <c r="I4" s="2"/>
+    </row>
+    <row r="5" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A5" s="42">
+        <v>2</v>
+      </c>
+      <c r="B5" s="2" t="s">
+        <v>211</v>
+      </c>
+      <c r="C5" s="18" t="s">
+        <v>215</v>
+      </c>
+      <c r="D5" s="95">
+        <v>46157</v>
+      </c>
+      <c r="E5" s="48">
+        <v>46203</v>
+      </c>
+      <c r="F5" s="2" t="s">
+        <v>135</v>
+      </c>
+      <c r="G5" s="2" t="s">
+        <v>219</v>
+      </c>
+      <c r="H5" s="14">
+        <v>5</v>
+      </c>
+      <c r="I5" s="2"/>
+    </row>
+    <row r="6" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A6" s="42">
+        <v>3</v>
+      </c>
+      <c r="B6" s="2" t="s">
+        <v>212</v>
+      </c>
+      <c r="C6" s="18" t="s">
+        <v>216</v>
+      </c>
+      <c r="D6" s="95">
+        <v>46174</v>
+      </c>
+      <c r="E6" s="96" t="s">
+        <v>135</v>
+      </c>
+      <c r="F6" s="2" t="s">
+        <v>135</v>
+      </c>
+      <c r="G6" s="2" t="s">
+        <v>220</v>
+      </c>
+      <c r="H6" s="14">
+        <v>5</v>
+      </c>
+      <c r="I6" s="2"/>
+    </row>
+    <row r="7" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A7" s="42">
+        <v>4</v>
+      </c>
+      <c r="B7" s="2" t="s">
+        <v>213</v>
+      </c>
+      <c r="C7" s="18" t="s">
+        <v>217</v>
+      </c>
+      <c r="D7" s="97" t="s">
+        <v>135</v>
+      </c>
+      <c r="E7" s="96" t="s">
+        <v>135</v>
+      </c>
+      <c r="F7" s="2" t="s">
+        <v>135</v>
+      </c>
+      <c r="G7" s="2" t="s">
+        <v>63</v>
+      </c>
+      <c r="H7" s="14">
+        <v>0</v>
+      </c>
+      <c r="I7" s="2"/>
+    </row>
+    <row r="8" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="D8" s="93"/>
+      <c r="E8" s="94"/>
+    </row>
+    <row r="9" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="D9" s="93"/>
+    </row>
+    <row r="10" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="D10" s="93"/>
+    </row>
+    <row r="11" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="D11" s="93"/>
+    </row>
+    <row r="12" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="D12" s="93"/>
+    </row>
+    <row r="13" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="D13" s="93"/>
+    </row>
+    <row r="14" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="D14" s="93"/>
+    </row>
+    <row r="15" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="D15" s="93"/>
+    </row>
+    <row r="16" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="D16" s="93"/>
+    </row>
+    <row r="17" spans="4:9" x14ac:dyDescent="0.3">
+      <c r="D17" s="93"/>
+    </row>
+    <row r="18" spans="4:9" x14ac:dyDescent="0.3">
+      <c r="D18" s="93"/>
+    </row>
+    <row r="19" spans="4:9" x14ac:dyDescent="0.3">
+      <c r="D19" s="93"/>
+    </row>
+    <row r="20" spans="4:9" x14ac:dyDescent="0.3">
+      <c r="D20" s="93"/>
+      <c r="I20" s="91"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
feat: Power Query - consolidacion de ventas 3 sucursales con Append Queries
</commit_message>
<xml_diff>
--- a/EXCEL/Presupuesto Personal.xlsx
+++ b/EXCEL/Presupuesto Personal.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/1d86eecf8daf4f0d/Documents/SQL Server Management Studio 22/Tienda-sqlserver/EXCEL/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="4" documentId="8_{EE053816-48E3-4E91-A6AD-611A9303676C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{2933B2D6-B1F1-4430-BB71-35C809E9BCE4}"/>
+  <xr:revisionPtr revIDLastSave="5" documentId="8_{EE053816-48E3-4E91-A6AD-611A9303676C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{CEB52EFF-F485-4B5A-B956-FBB827413A8C}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="1" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-1620" yWindow="228" windowWidth="12336" windowHeight="12240" firstSheet="1" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Personal-Budget_2026" sheetId="2" r:id="rId1"/>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="321" uniqueCount="221">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="327" uniqueCount="228">
   <si>
     <t xml:space="preserve">Cantidad </t>
   </si>
@@ -702,20 +702,41 @@
     <t xml:space="preserve">Morgan Housel </t>
   </si>
   <si>
-    <t>04/15/2026</t>
-  </si>
-  <si>
     <t xml:space="preserve">Done </t>
   </si>
   <si>
     <t>Leyendo</t>
+  </si>
+  <si>
+    <t>Utiles de Oficina</t>
+  </si>
+  <si>
+    <t>JUN 18, 2026</t>
+  </si>
+  <si>
+    <t>Suministro</t>
+  </si>
+  <si>
+    <t>JUN 18, 2027</t>
+  </si>
+  <si>
+    <t>Barber-Shop</t>
+  </si>
+  <si>
+    <t>Corte</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Utiles de Oficina </t>
+  </si>
+  <si>
+    <t>Total Dias Leyendo</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="8">
+  <numFmts count="9">
     <numFmt numFmtId="44" formatCode="_-&quot;XDR&quot;* #,##0.00_-;\-&quot;XDR&quot;* #,##0.00_-;_-&quot;XDR&quot;* &quot;-&quot;??_-;_-@_-"/>
     <numFmt numFmtId="43" formatCode="_-* #,##0.00_-;\-* #,##0.00_-;_-* &quot;-&quot;??_-;_-@_-"/>
     <numFmt numFmtId="164" formatCode="_-[$$-409]* #,##0.00_ ;_-[$$-409]* \-#,##0.00\ ;_-[$$-409]* &quot;-&quot;??_ ;_-@_ "/>
@@ -723,7 +744,8 @@
     <numFmt numFmtId="166" formatCode="_-* #,##0.0_-;\-* #,##0.0_-;_-* &quot;-&quot;??_-;_-@_-"/>
     <numFmt numFmtId="167" formatCode="_-[$$-2C0A]\ * #,##0.00_-;\-[$$-2C0A]\ * #,##0.00_-;_-[$$-2C0A]\ * &quot;-&quot;??_-;_-@_-"/>
     <numFmt numFmtId="168" formatCode="dd/mm/yyyy;@"/>
-    <numFmt numFmtId="170" formatCode="mm/dd/yyyy;@"/>
+    <numFmt numFmtId="169" formatCode="mm/dd/yyyy;@"/>
+    <numFmt numFmtId="170" formatCode="#,##0_ ;\-#,##0\ "/>
   </numFmts>
   <fonts count="20" x14ac:knownFonts="1">
     <font>
@@ -1037,7 +1059,7 @@
     <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="44" fontId="14" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="107">
+  <cellXfs count="110">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -1254,8 +1276,95 @@
     <xf numFmtId="167" fontId="15" fillId="14" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="167" fontId="16" fillId="14" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="1">
       <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="169" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="168" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="169" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="168" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="169" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="169" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="18" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="19" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="19" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="169" fontId="18" fillId="19" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="14" fontId="18" fillId="19" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="10" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="12" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="15" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
@@ -1263,101 +1372,23 @@
     <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="167" fontId="15" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="10" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="12" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="1">
+    <xf numFmtId="170" fontId="0" fillId="0" borderId="1" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1">
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="1" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="170" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="168" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="170" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="168" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="170" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="170" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="14" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="18" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="19" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="19" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="170" fontId="18" fillId="19" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="14" fontId="18" fillId="19" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="4">
@@ -1366,7 +1397,14 @@
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
     <cellStyle name="Percent" xfId="1" builtinId="5"/>
   </cellStyles>
-  <dxfs count="16">
+  <dxfs count="17">
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF00B050"/>
+        </patternFill>
+      </fill>
+    </dxf>
     <dxf>
       <font>
         <color rgb="FF9C0006"/>
@@ -3311,26 +3349,26 @@
       </c>
     </row>
     <row r="6" spans="1:18" ht="31.2" x14ac:dyDescent="0.3">
-      <c r="A6" s="77" t="s">
+      <c r="A6" s="90" t="s">
         <v>46</v>
       </c>
-      <c r="B6" s="77"/>
-      <c r="C6" s="77"/>
-      <c r="D6" s="77"/>
-      <c r="E6" s="77"/>
-      <c r="F6" s="77"/>
-      <c r="G6" s="77"/>
-      <c r="H6" s="77"/>
-      <c r="I6" s="77"/>
-      <c r="J6" s="77"/>
-      <c r="K6" s="77"/>
-      <c r="L6" s="77"/>
-      <c r="M6" s="77"/>
-      <c r="N6" s="77"/>
-      <c r="O6" s="77"/>
-      <c r="P6" s="77"/>
-      <c r="Q6" s="77"/>
-      <c r="R6" s="77"/>
+      <c r="B6" s="90"/>
+      <c r="C6" s="90"/>
+      <c r="D6" s="90"/>
+      <c r="E6" s="90"/>
+      <c r="F6" s="90"/>
+      <c r="G6" s="90"/>
+      <c r="H6" s="90"/>
+      <c r="I6" s="90"/>
+      <c r="J6" s="90"/>
+      <c r="K6" s="90"/>
+      <c r="L6" s="90"/>
+      <c r="M6" s="90"/>
+      <c r="N6" s="90"/>
+      <c r="O6" s="90"/>
+      <c r="P6" s="90"/>
+      <c r="Q6" s="90"/>
+      <c r="R6" s="90"/>
     </row>
     <row r="8" spans="1:18" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A8" s="34" t="s">
@@ -3567,20 +3605,20 @@
       </c>
     </row>
     <row r="20" spans="1:14" ht="31.2" x14ac:dyDescent="0.3">
-      <c r="A20" s="78" t="s">
+      <c r="A20" s="91" t="s">
         <v>79</v>
       </c>
-      <c r="B20" s="78"/>
-      <c r="C20" s="78"/>
-      <c r="D20" s="78"/>
-      <c r="E20" s="78"/>
-      <c r="F20" s="78"/>
-      <c r="G20" s="78"/>
-      <c r="H20" s="78"/>
-      <c r="I20" s="78"/>
-      <c r="J20" s="78"/>
-      <c r="K20" s="78"/>
-      <c r="L20" s="78"/>
+      <c r="B20" s="91"/>
+      <c r="C20" s="91"/>
+      <c r="D20" s="91"/>
+      <c r="E20" s="91"/>
+      <c r="F20" s="91"/>
+      <c r="G20" s="91"/>
+      <c r="H20" s="91"/>
+      <c r="I20" s="91"/>
+      <c r="J20" s="91"/>
+      <c r="K20" s="91"/>
+      <c r="L20" s="91"/>
       <c r="N20" s="16" t="s">
         <v>90</v>
       </c>
@@ -3747,20 +3785,20 @@
       </c>
     </row>
     <row r="33" spans="1:12" ht="31.2" x14ac:dyDescent="0.3">
-      <c r="A33" s="79" t="s">
+      <c r="A33" s="92" t="s">
         <v>107</v>
       </c>
-      <c r="B33" s="79"/>
-      <c r="C33" s="79"/>
-      <c r="D33" s="79"/>
-      <c r="E33" s="79"/>
-      <c r="F33" s="79"/>
-      <c r="G33" s="79"/>
-      <c r="H33" s="79"/>
-      <c r="I33" s="79"/>
-      <c r="J33" s="79"/>
-      <c r="K33" s="79"/>
-      <c r="L33" s="79"/>
+      <c r="B33" s="92"/>
+      <c r="C33" s="92"/>
+      <c r="D33" s="92"/>
+      <c r="E33" s="92"/>
+      <c r="F33" s="92"/>
+      <c r="G33" s="92"/>
+      <c r="H33" s="92"/>
+      <c r="I33" s="92"/>
+      <c r="J33" s="92"/>
+      <c r="K33" s="92"/>
+      <c r="L33" s="92"/>
     </row>
     <row r="35" spans="1:12" ht="23.4" x14ac:dyDescent="0.3">
       <c r="A35" s="16" t="s">
@@ -3768,20 +3806,20 @@
       </c>
     </row>
     <row r="37" spans="1:12" ht="31.2" x14ac:dyDescent="0.3">
-      <c r="A37" s="80" t="s">
+      <c r="A37" s="93" t="s">
         <v>98</v>
       </c>
-      <c r="B37" s="80"/>
-      <c r="C37" s="80"/>
-      <c r="D37" s="80"/>
-      <c r="E37" s="80"/>
-      <c r="F37" s="80"/>
-      <c r="G37" s="80"/>
-      <c r="H37" s="80"/>
-      <c r="I37" s="80"/>
-      <c r="J37" s="80"/>
-      <c r="K37" s="80"/>
-      <c r="L37" s="80"/>
+      <c r="B37" s="93"/>
+      <c r="C37" s="93"/>
+      <c r="D37" s="93"/>
+      <c r="E37" s="93"/>
+      <c r="F37" s="93"/>
+      <c r="G37" s="93"/>
+      <c r="H37" s="93"/>
+      <c r="I37" s="93"/>
+      <c r="J37" s="93"/>
+      <c r="K37" s="93"/>
+      <c r="L37" s="93"/>
     </row>
     <row r="39" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A39" s="35" t="s">
@@ -3898,16 +3936,16 @@
       </c>
     </row>
     <row r="51" spans="1:9" ht="31.2" x14ac:dyDescent="0.3">
-      <c r="A51" s="81" t="s">
+      <c r="A51" s="94" t="s">
         <v>109</v>
       </c>
-      <c r="B51" s="81"/>
-      <c r="C51" s="81"/>
-      <c r="D51" s="81"/>
-      <c r="E51" s="81"/>
-      <c r="F51" s="81"/>
-      <c r="G51" s="81"/>
-      <c r="H51" s="81"/>
+      <c r="B51" s="94"/>
+      <c r="C51" s="94"/>
+      <c r="D51" s="94"/>
+      <c r="E51" s="94"/>
+      <c r="F51" s="94"/>
+      <c r="G51" s="94"/>
+      <c r="H51" s="94"/>
       <c r="I51" s="40"/>
     </row>
     <row r="53" spans="1:9" ht="28.8" x14ac:dyDescent="0.3">
@@ -3974,18 +4012,18 @@
       </c>
     </row>
     <row r="66" spans="1:10" ht="31.2" x14ac:dyDescent="0.3">
-      <c r="A66" s="76" t="s">
+      <c r="A66" s="89" t="s">
         <v>117</v>
       </c>
-      <c r="B66" s="76"/>
-      <c r="C66" s="76"/>
-      <c r="D66" s="76"/>
-      <c r="E66" s="76"/>
-      <c r="F66" s="76"/>
-      <c r="G66" s="76"/>
-      <c r="H66" s="76"/>
-      <c r="I66" s="76"/>
-      <c r="J66" s="76"/>
+      <c r="B66" s="89"/>
+      <c r="C66" s="89"/>
+      <c r="D66" s="89"/>
+      <c r="E66" s="89"/>
+      <c r="F66" s="89"/>
+      <c r="G66" s="89"/>
+      <c r="H66" s="89"/>
+      <c r="I66" s="89"/>
+      <c r="J66" s="89"/>
     </row>
     <row r="68" spans="1:10" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A68" s="23" t="s">
@@ -4168,11 +4206,11 @@
       </c>
     </row>
     <row r="77" spans="1:10" ht="18" x14ac:dyDescent="0.3">
-      <c r="A77" s="75" t="s">
+      <c r="A77" s="88" t="s">
         <v>165</v>
       </c>
-      <c r="B77" s="75"/>
-      <c r="C77" s="75"/>
+      <c r="B77" s="88"/>
+      <c r="C77" s="88"/>
       <c r="D77" s="46"/>
       <c r="E77" s="46"/>
     </row>
@@ -4332,11 +4370,11 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:4" ht="18" x14ac:dyDescent="0.3">
-      <c r="A1" s="84" t="s">
+      <c r="A1" s="97" t="s">
         <v>4</v>
       </c>
-      <c r="B1" s="85"/>
-      <c r="C1" s="85"/>
+      <c r="B1" s="98"/>
+      <c r="C1" s="98"/>
     </row>
     <row r="2" spans="1:4" ht="15" x14ac:dyDescent="0.3">
       <c r="B2" s="1"/>
@@ -4477,11 +4515,11 @@
       <c r="C16" s="8"/>
     </row>
     <row r="17" spans="1:4" ht="21" x14ac:dyDescent="0.3">
-      <c r="A17" s="86" t="s">
+      <c r="A17" s="99" t="s">
         <v>13</v>
       </c>
-      <c r="B17" s="86"/>
-      <c r="C17" s="86"/>
+      <c r="B17" s="99"/>
+      <c r="C17" s="99"/>
     </row>
     <row r="19" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A19" s="12" t="s">
@@ -4633,11 +4671,11 @@
       </c>
     </row>
     <row r="31" spans="1:4" ht="21" x14ac:dyDescent="0.3">
-      <c r="A31" s="86" t="s">
+      <c r="A31" s="99" t="s">
         <v>13</v>
       </c>
-      <c r="B31" s="86"/>
-      <c r="C31" s="86"/>
+      <c r="B31" s="99"/>
+      <c r="C31" s="99"/>
     </row>
     <row r="33" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A33" s="12" t="s">
@@ -4789,26 +4827,26 @@
       </c>
     </row>
     <row r="46" spans="1:7" ht="25.8" x14ac:dyDescent="0.3">
-      <c r="A46" s="87" t="s">
+      <c r="A46" s="100" t="s">
         <v>27</v>
       </c>
-      <c r="B46" s="87"/>
-      <c r="C46" s="87"/>
-      <c r="D46" s="87"/>
-      <c r="E46" s="87"/>
-      <c r="F46" s="87"/>
-      <c r="G46" s="87"/>
+      <c r="B46" s="100"/>
+      <c r="C46" s="100"/>
+      <c r="D46" s="100"/>
+      <c r="E46" s="100"/>
+      <c r="F46" s="100"/>
+      <c r="G46" s="100"/>
     </row>
     <row r="48" spans="1:7" ht="18" x14ac:dyDescent="0.3">
-      <c r="A48" s="88" t="s">
+      <c r="A48" s="101" t="s">
         <v>28</v>
       </c>
-      <c r="B48" s="88"/>
-      <c r="C48" s="88"/>
-      <c r="D48" s="88"/>
-      <c r="E48" s="88"/>
-      <c r="F48" s="88"/>
-      <c r="G48" s="88"/>
+      <c r="B48" s="101"/>
+      <c r="C48" s="101"/>
+      <c r="D48" s="101"/>
+      <c r="E48" s="101"/>
+      <c r="F48" s="101"/>
+      <c r="G48" s="101"/>
     </row>
     <row r="50" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A50" s="13" t="s">
@@ -4985,11 +5023,11 @@
       <c r="D81" s="60">
         <v>1083</v>
       </c>
-      <c r="E81" s="82" t="s">
+      <c r="E81" s="95" t="s">
         <v>189</v>
       </c>
-      <c r="F81" s="83"/>
-      <c r="G81" s="83"/>
+      <c r="F81" s="96"/>
+      <c r="G81" s="96"/>
     </row>
     <row r="82" spans="1:7" ht="18" x14ac:dyDescent="0.3">
       <c r="A82" s="59" t="s">
@@ -5134,28 +5172,28 @@
   </mergeCells>
   <phoneticPr fontId="11" type="noConversion"/>
   <conditionalFormatting sqref="D80:D85">
-    <cfRule type="cellIs" dxfId="15" priority="11" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="16" priority="11" operator="greaterThan">
       <formula>1050</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="14" priority="12" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="15" priority="12" operator="greaterThan">
       <formula>500</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="13" priority="13" operator="lessThan">
+    <cfRule type="cellIs" dxfId="14" priority="13" operator="lessThan">
       <formula>500</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="12" priority="14" operator="lessThan">
+    <cfRule type="cellIs" dxfId="13" priority="14" operator="lessThan">
       <formula>500</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="11" priority="15" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="12" priority="15" operator="greaterThan">
       <formula>1050</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="10" priority="16" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="11" priority="16" operator="greaterThan">
       <formula>500</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="9" priority="17" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="10" priority="17" operator="greaterThan">
       <formula>1000</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="8" priority="18" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="9" priority="18" operator="greaterThan">
       <formula>" $ 1,100.00"</formula>
     </cfRule>
     <cfRule type="colorScale" priority="19">
@@ -5178,7 +5216,7 @@
   <sheetPr>
     <tabColor rgb="FFFF0000"/>
   </sheetPr>
-  <dimension ref="A2:G20"/>
+  <dimension ref="A2:G25"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="17.77734375" bestFit="1" customWidth="1"/>
@@ -5248,11 +5286,11 @@
       <c r="D5" s="62">
         <v>1083</v>
       </c>
-      <c r="E5" s="73" t="s">
+      <c r="E5" s="102" t="s">
         <v>189</v>
       </c>
-      <c r="F5" s="74"/>
-      <c r="G5" s="74"/>
+      <c r="F5" s="103"/>
+      <c r="G5" s="103"/>
     </row>
     <row r="6" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A6" s="63" t="s">
@@ -5325,82 +5363,83 @@
       <c r="G9" s="55"/>
     </row>
     <row r="10" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A10" s="55"/>
-      <c r="B10" s="55"/>
-      <c r="C10" s="55"/>
-      <c r="D10" s="55"/>
+      <c r="A10" s="63" t="s">
+        <v>221</v>
+      </c>
+      <c r="B10" s="63" t="s">
+        <v>220</v>
+      </c>
+      <c r="C10" s="63" t="s">
+        <v>222</v>
+      </c>
+      <c r="D10" s="105">
+        <v>510</v>
+      </c>
       <c r="E10" s="55"/>
       <c r="F10" s="55"/>
       <c r="G10" s="55"/>
     </row>
     <row r="11" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A11" s="55"/>
-      <c r="B11" s="55"/>
-      <c r="C11" s="55"/>
-      <c r="D11" s="55"/>
+      <c r="A11" s="63" t="s">
+        <v>223</v>
+      </c>
+      <c r="B11" s="63" t="s">
+        <v>224</v>
+      </c>
+      <c r="C11" s="63" t="s">
+        <v>225</v>
+      </c>
+      <c r="D11" s="105">
+        <v>400</v>
+      </c>
       <c r="E11" s="55"/>
       <c r="F11" s="55"/>
       <c r="G11" s="55"/>
     </row>
     <row r="12" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A12" s="55" t="s">
-        <v>200</v>
-      </c>
-      <c r="B12" s="55"/>
-      <c r="C12" s="69"/>
-      <c r="D12" s="55"/>
+      <c r="A12" s="104"/>
+      <c r="B12" s="104"/>
+      <c r="C12" s="104"/>
+      <c r="D12" s="104"/>
       <c r="E12" s="55"/>
       <c r="F12" s="55"/>
       <c r="G12" s="55"/>
     </row>
     <row r="13" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A13" s="67" t="s">
-        <v>153</v>
-      </c>
-      <c r="B13" s="67" t="s">
-        <v>190</v>
-      </c>
-      <c r="C13" s="55"/>
-      <c r="D13" s="55"/>
+      <c r="A13" s="104"/>
+      <c r="B13" s="104"/>
+      <c r="C13" s="104"/>
+      <c r="D13" s="104"/>
       <c r="E13" s="55"/>
       <c r="F13" s="55"/>
       <c r="G13" s="55"/>
     </row>
     <row r="14" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A14" s="70" t="s">
-        <v>181</v>
-      </c>
-      <c r="B14" s="71">
-        <f ca="1">SUMIF($B$4:$B$9, A14, $D$4:$D$8)</f>
-        <v>1083</v>
-      </c>
-      <c r="C14" s="55"/>
-      <c r="D14" s="55"/>
+      <c r="A14" s="104"/>
+      <c r="B14" s="104"/>
+      <c r="C14" s="104"/>
+      <c r="D14" s="104"/>
       <c r="E14" s="55"/>
       <c r="F14" s="55"/>
       <c r="G14" s="55"/>
     </row>
     <row r="15" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A15" s="70" t="s">
-        <v>191</v>
-      </c>
-      <c r="B15" s="71">
-        <f t="shared" ref="B15:B18" ca="1" si="0">SUMIF($B$4:$B$9, A15, $D$4:$D$8)</f>
-        <v>0</v>
-      </c>
-      <c r="C15" s="55"/>
+      <c r="A15" s="55" t="s">
+        <v>200</v>
+      </c>
+      <c r="B15" s="55"/>
+      <c r="C15" s="69"/>
       <c r="D15" s="55"/>
       <c r="E15" s="55"/>
       <c r="F15" s="55"/>
       <c r="G15" s="55"/>
     </row>
     <row r="16" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A16" s="70" t="s">
-        <v>192</v>
-      </c>
-      <c r="B16" s="71">
-        <f t="shared" ca="1" si="0"/>
-        <v>0</v>
+      <c r="A16" s="67" t="s">
+        <v>153</v>
+      </c>
+      <c r="B16" s="67" t="s">
+        <v>190</v>
       </c>
       <c r="C16" s="55"/>
       <c r="D16" s="55"/>
@@ -5410,11 +5449,11 @@
     </row>
     <row r="17" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A17" s="70" t="s">
-        <v>178</v>
+        <v>181</v>
       </c>
       <c r="B17" s="71">
-        <f t="shared" ca="1" si="0"/>
-        <v>4800</v>
+        <f>SUMIF($B$4:$B$11,A17,$D$4:$D$11)</f>
+        <v>1083</v>
       </c>
       <c r="C17" s="55"/>
       <c r="D17" s="55"/>
@@ -5424,10 +5463,10 @@
     </row>
     <row r="18" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A18" s="70" t="s">
-        <v>186</v>
+        <v>191</v>
       </c>
       <c r="B18" s="71">
-        <f t="shared" ca="1" si="0"/>
+        <f t="shared" ref="B18:B24" si="0">SUMIF($B$4:$B$11,A18,$D$4:$D$11)</f>
         <v>0</v>
       </c>
       <c r="C18" s="55"/>
@@ -5438,11 +5477,11 @@
     </row>
     <row r="19" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A19" s="70" t="s">
-        <v>193</v>
-      </c>
-      <c r="B19" s="72">
-        <f ca="1">+SUM(B14:B18)</f>
-        <v>5883</v>
+        <v>192</v>
+      </c>
+      <c r="B19" s="71">
+        <f t="shared" si="0"/>
+        <v>0</v>
       </c>
       <c r="C19" s="55"/>
       <c r="D19" s="55"/>
@@ -5451,44 +5490,115 @@
       <c r="G19" s="55"/>
     </row>
     <row r="20" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A20" s="55"/>
-      <c r="B20" s="55"/>
+      <c r="A20" s="70" t="s">
+        <v>178</v>
+      </c>
+      <c r="B20" s="71">
+        <f t="shared" si="0"/>
+        <v>4800</v>
+      </c>
       <c r="C20" s="55"/>
       <c r="D20" s="55"/>
       <c r="E20" s="55"/>
       <c r="F20" s="55"/>
       <c r="G20" s="55"/>
     </row>
+    <row r="21" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A21" s="70" t="s">
+        <v>186</v>
+      </c>
+      <c r="B21" s="71">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="C21" s="55"/>
+      <c r="D21" s="55"/>
+      <c r="E21" s="55"/>
+      <c r="F21" s="55"/>
+      <c r="G21" s="55"/>
+    </row>
+    <row r="22" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A22" s="70" t="s">
+        <v>226</v>
+      </c>
+      <c r="B22" s="71">
+        <f>SUMIF(B4:B11, "Utiles de Oficina",D4:D11)</f>
+        <v>510</v>
+      </c>
+      <c r="C22" s="55"/>
+      <c r="D22" s="55"/>
+      <c r="E22" s="55"/>
+      <c r="F22" s="55"/>
+      <c r="G22" s="55"/>
+    </row>
+    <row r="23" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A23" s="70" t="s">
+        <v>224</v>
+      </c>
+      <c r="B23" s="71">
+        <f t="shared" si="0"/>
+        <v>400</v>
+      </c>
+      <c r="C23" s="55"/>
+      <c r="D23" s="55"/>
+      <c r="E23" s="55"/>
+      <c r="F23" s="55"/>
+      <c r="G23" s="55"/>
+    </row>
+    <row r="24" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A24" s="70" t="s">
+        <v>193</v>
+      </c>
+      <c r="B24" s="71">
+        <f>SUM(B17:B23)</f>
+        <v>6793</v>
+      </c>
+      <c r="C24" s="55"/>
+      <c r="D24" s="55"/>
+      <c r="E24" s="55"/>
+      <c r="F24" s="55"/>
+      <c r="G24" s="55"/>
+    </row>
+    <row r="25" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A25" s="55"/>
+      <c r="B25" s="55"/>
+      <c r="C25" s="55"/>
+      <c r="D25" s="55"/>
+      <c r="E25" s="55"/>
+      <c r="F25" s="55"/>
+      <c r="G25" s="55"/>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="E5:G5"/>
   </mergeCells>
+  <phoneticPr fontId="11" type="noConversion"/>
   <conditionalFormatting sqref="D4:D9">
-    <cfRule type="cellIs" dxfId="7" priority="1" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="8" priority="2" operator="greaterThan">
       <formula>1050</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="6" priority="2" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="7" priority="3" operator="greaterThan">
       <formula>500</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="5" priority="3" operator="lessThan">
+    <cfRule type="cellIs" dxfId="6" priority="4" operator="lessThan">
       <formula>500</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="4" priority="4" operator="lessThan">
+    <cfRule type="cellIs" dxfId="5" priority="5" operator="lessThan">
       <formula>500</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="3" priority="5" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="4" priority="6" operator="greaterThan">
       <formula>1050</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="2" priority="6" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="3" priority="7" operator="greaterThan">
       <formula>500</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="1" priority="7" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="2" priority="8" operator="greaterThan">
       <formula>1000</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="0" priority="8" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="1" priority="9" operator="greaterThan">
       <formula>" $ 1,100.00"</formula>
     </cfRule>
-    <cfRule type="colorScale" priority="9">
+    <cfRule type="colorScale" priority="10">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="max"/>
@@ -5497,7 +5607,15 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
+  <conditionalFormatting sqref="D10:D11">
+    <cfRule type="cellIs" dxfId="0" priority="1" operator="lessThan">
+      <formula>1000</formula>
+    </cfRule>
+  </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <ignoredErrors>
+    <ignoredError sqref="B22" formula="1"/>
+  </ignoredErrors>
 </worksheet>
 </file>
 
@@ -5506,68 +5624,73 @@
   <sheetPr>
     <tabColor rgb="FF002060"/>
   </sheetPr>
-  <dimension ref="A1:I20"/>
+  <dimension ref="A1:J20"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="2.109375" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="27.77734375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="13.6640625" style="89" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="10.5546875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="10.5546875" style="92" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="13.109375" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="9.109375" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="10.44140625" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="14.6640625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="2.44140625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="22.33203125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="14.5546875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="11.6640625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="11.6640625" style="74" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="14.21875" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="9.77734375" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="14.21875" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="14.21875" customWidth="1"/>
+    <col min="10" max="10" width="15.5546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" ht="18" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:10" ht="18" x14ac:dyDescent="0.3">
       <c r="B1" s="57" t="s">
         <v>201</v>
       </c>
-      <c r="D1" s="93"/>
-    </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A2" s="98"/>
-      <c r="B2" s="98"/>
-      <c r="C2" s="99"/>
-      <c r="D2" s="100"/>
-      <c r="E2" s="101"/>
-      <c r="F2" s="98"/>
-      <c r="G2" s="98"/>
-      <c r="H2" s="98"/>
-      <c r="I2" s="98"/>
-    </row>
-    <row r="3" spans="1:9" s="90" customFormat="1" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A3" s="102" t="s">
+      <c r="D1" s="75"/>
+    </row>
+    <row r="2" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A2" s="80"/>
+      <c r="B2" s="80"/>
+      <c r="C2" s="80"/>
+      <c r="D2" s="81"/>
+      <c r="E2" s="82"/>
+      <c r="F2" s="80"/>
+      <c r="G2" s="80"/>
+      <c r="H2" s="80"/>
+      <c r="I2" s="80"/>
+      <c r="J2" s="80"/>
+    </row>
+    <row r="3" spans="1:10" s="72" customFormat="1" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A3" s="83" t="s">
         <v>209</v>
       </c>
-      <c r="B3" s="103" t="s">
+      <c r="B3" s="84" t="s">
         <v>202</v>
       </c>
-      <c r="C3" s="104" t="s">
+      <c r="C3" s="85" t="s">
         <v>203</v>
       </c>
-      <c r="D3" s="105" t="s">
+      <c r="D3" s="86" t="s">
         <v>204</v>
       </c>
-      <c r="E3" s="106" t="s">
+      <c r="E3" s="87" t="s">
         <v>205</v>
       </c>
-      <c r="F3" s="103" t="s">
+      <c r="F3" s="84" t="s">
         <v>206</v>
       </c>
-      <c r="G3" s="103" t="s">
+      <c r="G3" s="84" t="s">
         <v>56</v>
       </c>
-      <c r="H3" s="103" t="s">
+      <c r="H3" s="84" t="s">
         <v>208</v>
       </c>
-      <c r="I3" s="103" t="s">
+      <c r="I3" s="84" t="s">
+        <v>227</v>
+      </c>
+      <c r="J3" s="84" t="s">
         <v>207</v>
       </c>
     </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A4" s="42">
+    <row r="4" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A4" s="106">
         <v>1</v>
       </c>
       <c r="B4" s="2" t="s">
@@ -5576,23 +5699,30 @@
       <c r="C4" s="18" t="s">
         <v>214</v>
       </c>
-      <c r="D4" s="48" t="s">
-        <v>218</v>
+      <c r="D4" s="48">
+        <v>46127</v>
       </c>
       <c r="E4" s="48">
         <v>46154</v>
       </c>
-      <c r="F4" s="2"/>
+      <c r="F4" s="2">
+        <f>E4-D4</f>
+        <v>27</v>
+      </c>
       <c r="G4" s="2" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
       <c r="H4" s="14">
         <v>4</v>
       </c>
-      <c r="I4" s="2"/>
-    </row>
-    <row r="5" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A5" s="42">
+      <c r="I4" s="108">
+        <f ca="1">SUM(F4:F6)</f>
+        <v>90</v>
+      </c>
+      <c r="J4" s="2"/>
+    </row>
+    <row r="5" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A5" s="106">
         <v>2</v>
       </c>
       <c r="B5" s="2" t="s">
@@ -5601,25 +5731,30 @@
       <c r="C5" s="18" t="s">
         <v>215</v>
       </c>
-      <c r="D5" s="95">
+      <c r="D5" s="77">
         <v>46157</v>
       </c>
       <c r="E5" s="48">
         <v>46203</v>
       </c>
-      <c r="F5" s="2" t="s">
-        <v>135</v>
+      <c r="F5" s="2">
+        <f>E5-D5</f>
+        <v>46</v>
       </c>
       <c r="G5" s="2" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
       <c r="H5" s="14">
         <v>5</v>
       </c>
-      <c r="I5" s="2"/>
-    </row>
-    <row r="6" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A6" s="42">
+      <c r="I5" s="109">
+        <f ca="1">AVERAGE(F4:F6)</f>
+        <v>30</v>
+      </c>
+      <c r="J5" s="2"/>
+    </row>
+    <row r="6" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A6" s="106">
         <v>3</v>
       </c>
       <c r="B6" s="2" t="s">
@@ -5628,25 +5763,27 @@
       <c r="C6" s="18" t="s">
         <v>216</v>
       </c>
-      <c r="D6" s="95">
+      <c r="D6" s="77">
         <v>46174</v>
       </c>
-      <c r="E6" s="96" t="s">
+      <c r="E6" s="78" t="s">
         <v>135</v>
       </c>
-      <c r="F6" s="2" t="s">
-        <v>135</v>
+      <c r="F6" s="107">
+        <f ca="1">TODAY()-D6</f>
+        <v>17</v>
       </c>
       <c r="G6" s="2" t="s">
-        <v>220</v>
+        <v>219</v>
       </c>
       <c r="H6" s="14">
         <v>5</v>
       </c>
-      <c r="I6" s="2"/>
-    </row>
-    <row r="7" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A7" s="42">
+      <c r="I6" s="14"/>
+      <c r="J6" s="2"/>
+    </row>
+    <row r="7" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A7" s="106">
         <v>4</v>
       </c>
       <c r="B7" s="2" t="s">
@@ -5655,10 +5792,10 @@
       <c r="C7" s="18" t="s">
         <v>217</v>
       </c>
-      <c r="D7" s="97" t="s">
+      <c r="D7" s="79" t="s">
         <v>135</v>
       </c>
-      <c r="E7" s="96" t="s">
+      <c r="E7" s="78" t="s">
         <v>135</v>
       </c>
       <c r="F7" s="2" t="s">
@@ -5670,48 +5807,49 @@
       <c r="H7" s="14">
         <v>0</v>
       </c>
-      <c r="I7" s="2"/>
-    </row>
-    <row r="8" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="D8" s="93"/>
-      <c r="E8" s="94"/>
-    </row>
-    <row r="9" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="D9" s="93"/>
-    </row>
-    <row r="10" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="D10" s="93"/>
-    </row>
-    <row r="11" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="D11" s="93"/>
-    </row>
-    <row r="12" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="D12" s="93"/>
-    </row>
-    <row r="13" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="D13" s="93"/>
-    </row>
-    <row r="14" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="D14" s="93"/>
-    </row>
-    <row r="15" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="D15" s="93"/>
-    </row>
-    <row r="16" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="D16" s="93"/>
-    </row>
-    <row r="17" spans="4:9" x14ac:dyDescent="0.3">
-      <c r="D17" s="93"/>
-    </row>
-    <row r="18" spans="4:9" x14ac:dyDescent="0.3">
-      <c r="D18" s="93"/>
-    </row>
-    <row r="19" spans="4:9" x14ac:dyDescent="0.3">
-      <c r="D19" s="93"/>
-    </row>
-    <row r="20" spans="4:9" x14ac:dyDescent="0.3">
-      <c r="D20" s="93"/>
-      <c r="I20" s="91"/>
+      <c r="I7" s="14"/>
+      <c r="J7" s="2"/>
+    </row>
+    <row r="8" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="D8" s="75"/>
+      <c r="E8" s="76"/>
+    </row>
+    <row r="9" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="D9" s="75"/>
+    </row>
+    <row r="10" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="D10" s="75"/>
+    </row>
+    <row r="11" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="D11" s="75"/>
+    </row>
+    <row r="12" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="D12" s="75"/>
+    </row>
+    <row r="13" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="D13" s="75"/>
+    </row>
+    <row r="14" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="D14" s="75"/>
+    </row>
+    <row r="15" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="D15" s="75"/>
+    </row>
+    <row r="16" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="D16" s="75"/>
+    </row>
+    <row r="17" spans="4:10" x14ac:dyDescent="0.3">
+      <c r="D17" s="75"/>
+    </row>
+    <row r="18" spans="4:10" x14ac:dyDescent="0.3">
+      <c r="D18" s="75"/>
+    </row>
+    <row r="19" spans="4:10" x14ac:dyDescent="0.3">
+      <c r="D19" s="75"/>
+    </row>
+    <row r="20" spans="4:10" x14ac:dyDescent="0.3">
+      <c r="D20" s="75"/>
+      <c r="J20" s="73"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
feat: Tablas Dinamicas Avanzadas - PivotTable, Slicers, PivotChart, Timeline y Campo Calculado
</commit_message>
<xml_diff>
--- a/EXCEL/Presupuesto Personal.xlsx
+++ b/EXCEL/Presupuesto Personal.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/1d86eecf8daf4f0d/Documents/SQL Server Management Studio 22/Tienda-sqlserver/EXCEL/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="5" documentId="8_{EE053816-48E3-4E91-A6AD-611A9303676C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{CEB52EFF-F485-4B5A-B956-FBB827413A8C}"/>
+  <xr:revisionPtr revIDLastSave="6" documentId="8_{EE053816-48E3-4E91-A6AD-611A9303676C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{58A4560E-BAA5-4759-B562-A6CBA4876ED6}"/>
   <bookViews>
-    <workbookView xWindow="-1620" yWindow="228" windowWidth="12336" windowHeight="12240" firstSheet="1" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="12336" windowHeight="12240" firstSheet="1" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Personal-Budget_2026" sheetId="2" r:id="rId1"/>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="327" uniqueCount="228">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="328" uniqueCount="230">
   <si>
     <t xml:space="preserve">Cantidad </t>
   </si>
@@ -730,6 +730,12 @@
   </si>
   <si>
     <t>Total Dias Leyendo</t>
+  </si>
+  <si>
+    <t>JUN 20, 2026</t>
+  </si>
+  <si>
+    <t>Mini Market</t>
   </si>
 </sst>
 </file>
@@ -1059,7 +1065,7 @@
     <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="44" fontId="14" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="110">
+  <cellXfs count="109">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -1324,6 +1330,21 @@
     <xf numFmtId="14" fontId="18" fillId="19" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="167" fontId="15" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="170" fontId="0" fillId="0" borderId="1" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="1" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
@@ -1371,24 +1392,6 @@
     </xf>
     <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="167" fontId="15" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="1" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="170" fontId="0" fillId="0" borderId="1" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="1" fontId="0" fillId="0" borderId="1" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="4">
@@ -1398,13 +1401,6 @@
     <cellStyle name="Percent" xfId="1" builtinId="5"/>
   </cellStyles>
   <dxfs count="17">
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FF00B050"/>
-        </patternFill>
-      </fill>
-    </dxf>
     <dxf>
       <font>
         <color rgb="FF9C0006"/>
@@ -1461,6 +1457,13 @@
       <fill>
         <patternFill>
           <bgColor rgb="FFFF0000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF00B050"/>
         </patternFill>
       </fill>
     </dxf>
@@ -3349,26 +3352,26 @@
       </c>
     </row>
     <row r="6" spans="1:18" ht="31.2" x14ac:dyDescent="0.3">
-      <c r="A6" s="90" t="s">
+      <c r="A6" s="95" t="s">
         <v>46</v>
       </c>
-      <c r="B6" s="90"/>
-      <c r="C6" s="90"/>
-      <c r="D6" s="90"/>
-      <c r="E6" s="90"/>
-      <c r="F6" s="90"/>
-      <c r="G6" s="90"/>
-      <c r="H6" s="90"/>
-      <c r="I6" s="90"/>
-      <c r="J6" s="90"/>
-      <c r="K6" s="90"/>
-      <c r="L6" s="90"/>
-      <c r="M6" s="90"/>
-      <c r="N6" s="90"/>
-      <c r="O6" s="90"/>
-      <c r="P6" s="90"/>
-      <c r="Q6" s="90"/>
-      <c r="R6" s="90"/>
+      <c r="B6" s="95"/>
+      <c r="C6" s="95"/>
+      <c r="D6" s="95"/>
+      <c r="E6" s="95"/>
+      <c r="F6" s="95"/>
+      <c r="G6" s="95"/>
+      <c r="H6" s="95"/>
+      <c r="I6" s="95"/>
+      <c r="J6" s="95"/>
+      <c r="K6" s="95"/>
+      <c r="L6" s="95"/>
+      <c r="M6" s="95"/>
+      <c r="N6" s="95"/>
+      <c r="O6" s="95"/>
+      <c r="P6" s="95"/>
+      <c r="Q6" s="95"/>
+      <c r="R6" s="95"/>
     </row>
     <row r="8" spans="1:18" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A8" s="34" t="s">
@@ -3605,20 +3608,20 @@
       </c>
     </row>
     <row r="20" spans="1:14" ht="31.2" x14ac:dyDescent="0.3">
-      <c r="A20" s="91" t="s">
+      <c r="A20" s="96" t="s">
         <v>79</v>
       </c>
-      <c r="B20" s="91"/>
-      <c r="C20" s="91"/>
-      <c r="D20" s="91"/>
-      <c r="E20" s="91"/>
-      <c r="F20" s="91"/>
-      <c r="G20" s="91"/>
-      <c r="H20" s="91"/>
-      <c r="I20" s="91"/>
-      <c r="J20" s="91"/>
-      <c r="K20" s="91"/>
-      <c r="L20" s="91"/>
+      <c r="B20" s="96"/>
+      <c r="C20" s="96"/>
+      <c r="D20" s="96"/>
+      <c r="E20" s="96"/>
+      <c r="F20" s="96"/>
+      <c r="G20" s="96"/>
+      <c r="H20" s="96"/>
+      <c r="I20" s="96"/>
+      <c r="J20" s="96"/>
+      <c r="K20" s="96"/>
+      <c r="L20" s="96"/>
       <c r="N20" s="16" t="s">
         <v>90</v>
       </c>
@@ -3785,20 +3788,20 @@
       </c>
     </row>
     <row r="33" spans="1:12" ht="31.2" x14ac:dyDescent="0.3">
-      <c r="A33" s="92" t="s">
+      <c r="A33" s="97" t="s">
         <v>107</v>
       </c>
-      <c r="B33" s="92"/>
-      <c r="C33" s="92"/>
-      <c r="D33" s="92"/>
-      <c r="E33" s="92"/>
-      <c r="F33" s="92"/>
-      <c r="G33" s="92"/>
-      <c r="H33" s="92"/>
-      <c r="I33" s="92"/>
-      <c r="J33" s="92"/>
-      <c r="K33" s="92"/>
-      <c r="L33" s="92"/>
+      <c r="B33" s="97"/>
+      <c r="C33" s="97"/>
+      <c r="D33" s="97"/>
+      <c r="E33" s="97"/>
+      <c r="F33" s="97"/>
+      <c r="G33" s="97"/>
+      <c r="H33" s="97"/>
+      <c r="I33" s="97"/>
+      <c r="J33" s="97"/>
+      <c r="K33" s="97"/>
+      <c r="L33" s="97"/>
     </row>
     <row r="35" spans="1:12" ht="23.4" x14ac:dyDescent="0.3">
       <c r="A35" s="16" t="s">
@@ -3806,20 +3809,20 @@
       </c>
     </row>
     <row r="37" spans="1:12" ht="31.2" x14ac:dyDescent="0.3">
-      <c r="A37" s="93" t="s">
+      <c r="A37" s="98" t="s">
         <v>98</v>
       </c>
-      <c r="B37" s="93"/>
-      <c r="C37" s="93"/>
-      <c r="D37" s="93"/>
-      <c r="E37" s="93"/>
-      <c r="F37" s="93"/>
-      <c r="G37" s="93"/>
-      <c r="H37" s="93"/>
-      <c r="I37" s="93"/>
-      <c r="J37" s="93"/>
-      <c r="K37" s="93"/>
-      <c r="L37" s="93"/>
+      <c r="B37" s="98"/>
+      <c r="C37" s="98"/>
+      <c r="D37" s="98"/>
+      <c r="E37" s="98"/>
+      <c r="F37" s="98"/>
+      <c r="G37" s="98"/>
+      <c r="H37" s="98"/>
+      <c r="I37" s="98"/>
+      <c r="J37" s="98"/>
+      <c r="K37" s="98"/>
+      <c r="L37" s="98"/>
     </row>
     <row r="39" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A39" s="35" t="s">
@@ -3936,16 +3939,16 @@
       </c>
     </row>
     <row r="51" spans="1:9" ht="31.2" x14ac:dyDescent="0.3">
-      <c r="A51" s="94" t="s">
+      <c r="A51" s="99" t="s">
         <v>109</v>
       </c>
-      <c r="B51" s="94"/>
-      <c r="C51" s="94"/>
-      <c r="D51" s="94"/>
-      <c r="E51" s="94"/>
-      <c r="F51" s="94"/>
-      <c r="G51" s="94"/>
-      <c r="H51" s="94"/>
+      <c r="B51" s="99"/>
+      <c r="C51" s="99"/>
+      <c r="D51" s="99"/>
+      <c r="E51" s="99"/>
+      <c r="F51" s="99"/>
+      <c r="G51" s="99"/>
+      <c r="H51" s="99"/>
       <c r="I51" s="40"/>
     </row>
     <row r="53" spans="1:9" ht="28.8" x14ac:dyDescent="0.3">
@@ -4012,18 +4015,18 @@
       </c>
     </row>
     <row r="66" spans="1:10" ht="31.2" x14ac:dyDescent="0.3">
-      <c r="A66" s="89" t="s">
+      <c r="A66" s="94" t="s">
         <v>117</v>
       </c>
-      <c r="B66" s="89"/>
-      <c r="C66" s="89"/>
-      <c r="D66" s="89"/>
-      <c r="E66" s="89"/>
-      <c r="F66" s="89"/>
-      <c r="G66" s="89"/>
-      <c r="H66" s="89"/>
-      <c r="I66" s="89"/>
-      <c r="J66" s="89"/>
+      <c r="B66" s="94"/>
+      <c r="C66" s="94"/>
+      <c r="D66" s="94"/>
+      <c r="E66" s="94"/>
+      <c r="F66" s="94"/>
+      <c r="G66" s="94"/>
+      <c r="H66" s="94"/>
+      <c r="I66" s="94"/>
+      <c r="J66" s="94"/>
     </row>
     <row r="68" spans="1:10" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A68" s="23" t="s">
@@ -4206,11 +4209,11 @@
       </c>
     </row>
     <row r="77" spans="1:10" ht="18" x14ac:dyDescent="0.3">
-      <c r="A77" s="88" t="s">
+      <c r="A77" s="93" t="s">
         <v>165</v>
       </c>
-      <c r="B77" s="88"/>
-      <c r="C77" s="88"/>
+      <c r="B77" s="93"/>
+      <c r="C77" s="93"/>
       <c r="D77" s="46"/>
       <c r="E77" s="46"/>
     </row>
@@ -4370,11 +4373,11 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:4" ht="18" x14ac:dyDescent="0.3">
-      <c r="A1" s="97" t="s">
+      <c r="A1" s="102" t="s">
         <v>4</v>
       </c>
-      <c r="B1" s="98"/>
-      <c r="C1" s="98"/>
+      <c r="B1" s="103"/>
+      <c r="C1" s="103"/>
     </row>
     <row r="2" spans="1:4" ht="15" x14ac:dyDescent="0.3">
       <c r="B2" s="1"/>
@@ -4515,11 +4518,11 @@
       <c r="C16" s="8"/>
     </row>
     <row r="17" spans="1:4" ht="21" x14ac:dyDescent="0.3">
-      <c r="A17" s="99" t="s">
+      <c r="A17" s="104" t="s">
         <v>13</v>
       </c>
-      <c r="B17" s="99"/>
-      <c r="C17" s="99"/>
+      <c r="B17" s="104"/>
+      <c r="C17" s="104"/>
     </row>
     <row r="19" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A19" s="12" t="s">
@@ -4671,11 +4674,11 @@
       </c>
     </row>
     <row r="31" spans="1:4" ht="21" x14ac:dyDescent="0.3">
-      <c r="A31" s="99" t="s">
+      <c r="A31" s="104" t="s">
         <v>13</v>
       </c>
-      <c r="B31" s="99"/>
-      <c r="C31" s="99"/>
+      <c r="B31" s="104"/>
+      <c r="C31" s="104"/>
     </row>
     <row r="33" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A33" s="12" t="s">
@@ -4827,26 +4830,26 @@
       </c>
     </row>
     <row r="46" spans="1:7" ht="25.8" x14ac:dyDescent="0.3">
-      <c r="A46" s="100" t="s">
+      <c r="A46" s="105" t="s">
         <v>27</v>
       </c>
-      <c r="B46" s="100"/>
-      <c r="C46" s="100"/>
-      <c r="D46" s="100"/>
-      <c r="E46" s="100"/>
-      <c r="F46" s="100"/>
-      <c r="G46" s="100"/>
+      <c r="B46" s="105"/>
+      <c r="C46" s="105"/>
+      <c r="D46" s="105"/>
+      <c r="E46" s="105"/>
+      <c r="F46" s="105"/>
+      <c r="G46" s="105"/>
     </row>
     <row r="48" spans="1:7" ht="18" x14ac:dyDescent="0.3">
-      <c r="A48" s="101" t="s">
+      <c r="A48" s="106" t="s">
         <v>28</v>
       </c>
-      <c r="B48" s="101"/>
-      <c r="C48" s="101"/>
-      <c r="D48" s="101"/>
-      <c r="E48" s="101"/>
-      <c r="F48" s="101"/>
-      <c r="G48" s="101"/>
+      <c r="B48" s="106"/>
+      <c r="C48" s="106"/>
+      <c r="D48" s="106"/>
+      <c r="E48" s="106"/>
+      <c r="F48" s="106"/>
+      <c r="G48" s="106"/>
     </row>
     <row r="50" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A50" s="13" t="s">
@@ -5023,11 +5026,11 @@
       <c r="D81" s="60">
         <v>1083</v>
       </c>
-      <c r="E81" s="95" t="s">
+      <c r="E81" s="100" t="s">
         <v>189</v>
       </c>
-      <c r="F81" s="96"/>
-      <c r="G81" s="96"/>
+      <c r="F81" s="101"/>
+      <c r="G81" s="101"/>
     </row>
     <row r="82" spans="1:7" ht="18" x14ac:dyDescent="0.3">
       <c r="A82" s="59" t="s">
@@ -5216,7 +5219,7 @@
   <sheetPr>
     <tabColor rgb="FFFF0000"/>
   </sheetPr>
-  <dimension ref="A2:G25"/>
+  <dimension ref="A2:G26"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="17.77734375" bestFit="1" customWidth="1"/>
@@ -5286,60 +5289,60 @@
       <c r="D5" s="62">
         <v>1083</v>
       </c>
-      <c r="E5" s="102" t="s">
+      <c r="E5" s="107" t="s">
         <v>189</v>
       </c>
-      <c r="F5" s="103"/>
-      <c r="G5" s="103"/>
+      <c r="F5" s="108"/>
+      <c r="G5" s="108"/>
     </row>
     <row r="6" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A6" s="63" t="s">
         <v>184</v>
       </c>
       <c r="B6" s="63" t="s">
-        <v>182</v>
+        <v>195</v>
       </c>
       <c r="C6" s="63" t="s">
-        <v>183</v>
+        <v>197</v>
       </c>
       <c r="D6" s="62">
         <v>0</v>
       </c>
-      <c r="E6" s="68" t="s">
-        <v>188</v>
-      </c>
+      <c r="E6" s="55"/>
       <c r="F6" s="55"/>
       <c r="G6" s="55"/>
     </row>
     <row r="7" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A7" s="63" t="s">
-        <v>184</v>
+        <v>198</v>
       </c>
       <c r="B7" s="63" t="s">
-        <v>195</v>
+        <v>178</v>
       </c>
       <c r="C7" s="63" t="s">
-        <v>197</v>
+        <v>199</v>
       </c>
       <c r="D7" s="62">
-        <v>0</v>
-      </c>
-      <c r="E7" s="55"/>
+        <v>3800</v>
+      </c>
+      <c r="E7" s="68" t="s">
+        <v>188</v>
+      </c>
       <c r="F7" s="55"/>
       <c r="G7" s="55"/>
     </row>
     <row r="8" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A8" s="63" t="s">
-        <v>198</v>
+        <v>184</v>
       </c>
       <c r="B8" s="63" t="s">
-        <v>178</v>
+        <v>185</v>
       </c>
       <c r="C8" s="63" t="s">
-        <v>199</v>
+        <v>196</v>
       </c>
       <c r="D8" s="62">
-        <v>3800</v>
+        <v>0</v>
       </c>
       <c r="E8" s="55"/>
       <c r="F8" s="55"/>
@@ -5347,16 +5350,16 @@
     </row>
     <row r="9" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A9" s="63" t="s">
-        <v>184</v>
+        <v>221</v>
       </c>
       <c r="B9" s="63" t="s">
-        <v>185</v>
+        <v>220</v>
       </c>
       <c r="C9" s="63" t="s">
-        <v>196</v>
-      </c>
-      <c r="D9" s="62">
-        <v>0</v>
+        <v>222</v>
+      </c>
+      <c r="D9" s="88">
+        <v>510</v>
       </c>
       <c r="E9" s="55"/>
       <c r="F9" s="55"/>
@@ -5364,16 +5367,16 @@
     </row>
     <row r="10" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A10" s="63" t="s">
-        <v>221</v>
+        <v>228</v>
       </c>
       <c r="B10" s="63" t="s">
-        <v>220</v>
+        <v>229</v>
       </c>
       <c r="C10" s="63" t="s">
-        <v>222</v>
-      </c>
-      <c r="D10" s="105">
-        <v>510</v>
+        <v>183</v>
+      </c>
+      <c r="D10" s="88">
+        <v>15</v>
       </c>
       <c r="E10" s="55"/>
       <c r="F10" s="55"/>
@@ -5389,7 +5392,7 @@
       <c r="C11" s="63" t="s">
         <v>225</v>
       </c>
-      <c r="D11" s="105">
+      <c r="D11" s="88">
         <v>400</v>
       </c>
       <c r="E11" s="55"/>
@@ -5397,28 +5400,28 @@
       <c r="G11" s="55"/>
     </row>
     <row r="12" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A12" s="104"/>
-      <c r="B12" s="104"/>
-      <c r="C12" s="104"/>
-      <c r="D12" s="104"/>
+      <c r="A12" s="55"/>
+      <c r="B12" s="55"/>
+      <c r="C12" s="55"/>
+      <c r="D12" s="55"/>
       <c r="E12" s="55"/>
       <c r="F12" s="55"/>
       <c r="G12" s="55"/>
     </row>
     <row r="13" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A13" s="104"/>
-      <c r="B13" s="104"/>
-      <c r="C13" s="104"/>
-      <c r="D13" s="104"/>
+      <c r="A13" s="55"/>
+      <c r="B13" s="55"/>
+      <c r="C13" s="55"/>
+      <c r="D13" s="55"/>
       <c r="E13" s="55"/>
       <c r="F13" s="55"/>
       <c r="G13" s="55"/>
     </row>
     <row r="14" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A14" s="104"/>
-      <c r="B14" s="104"/>
-      <c r="C14" s="104"/>
-      <c r="D14" s="104"/>
+      <c r="A14" s="55"/>
+      <c r="B14" s="55"/>
+      <c r="C14" s="55"/>
+      <c r="D14" s="55"/>
       <c r="E14" s="55"/>
       <c r="F14" s="55"/>
       <c r="G14" s="55"/>
@@ -5463,10 +5466,10 @@
     </row>
     <row r="18" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A18" s="70" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="B18" s="71">
-        <f t="shared" ref="B18:B24" si="0">SUMIF($B$4:$B$11,A18,$D$4:$D$11)</f>
+        <f t="shared" ref="B18:B25" si="0">SUMIF($B$4:$B$11,A18,$D$4:$D$11)</f>
         <v>0</v>
       </c>
       <c r="C18" s="55"/>
@@ -5477,11 +5480,11 @@
     </row>
     <row r="19" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A19" s="70" t="s">
-        <v>192</v>
+        <v>178</v>
       </c>
       <c r="B19" s="71">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>4800</v>
       </c>
       <c r="C19" s="55"/>
       <c r="D19" s="55"/>
@@ -5491,11 +5494,11 @@
     </row>
     <row r="20" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A20" s="70" t="s">
-        <v>178</v>
+        <v>186</v>
       </c>
       <c r="B20" s="71">
         <f t="shared" si="0"/>
-        <v>4800</v>
+        <v>0</v>
       </c>
       <c r="C20" s="55"/>
       <c r="D20" s="55"/>
@@ -5505,7 +5508,7 @@
     </row>
     <row r="21" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A21" s="70" t="s">
-        <v>186</v>
+        <v>226</v>
       </c>
       <c r="B21" s="71">
         <f t="shared" si="0"/>
@@ -5519,11 +5522,11 @@
     </row>
     <row r="22" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A22" s="70" t="s">
-        <v>226</v>
+        <v>191</v>
       </c>
       <c r="B22" s="71">
-        <f>SUMIF(B4:B11, "Utiles de Oficina",D4:D11)</f>
-        <v>510</v>
+        <f t="shared" si="0"/>
+        <v>0</v>
       </c>
       <c r="C22" s="55"/>
       <c r="D22" s="55"/>
@@ -5533,11 +5536,11 @@
     </row>
     <row r="23" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A23" s="70" t="s">
-        <v>224</v>
+        <v>229</v>
       </c>
       <c r="B23" s="71">
         <f t="shared" si="0"/>
-        <v>400</v>
+        <v>15</v>
       </c>
       <c r="C23" s="55"/>
       <c r="D23" s="55"/>
@@ -5547,11 +5550,11 @@
     </row>
     <row r="24" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A24" s="70" t="s">
-        <v>193</v>
+        <v>224</v>
       </c>
       <c r="B24" s="71">
-        <f>SUM(B17:B23)</f>
-        <v>6793</v>
+        <f t="shared" si="0"/>
+        <v>400</v>
       </c>
       <c r="C24" s="55"/>
       <c r="D24" s="55"/>
@@ -5560,45 +5563,64 @@
       <c r="G24" s="55"/>
     </row>
     <row r="25" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A25" s="55"/>
-      <c r="B25" s="55"/>
+      <c r="A25" s="70" t="s">
+        <v>193</v>
+      </c>
+      <c r="B25" s="71">
+        <f>+SUM(B17:B24)</f>
+        <v>6298</v>
+      </c>
       <c r="C25" s="55"/>
       <c r="D25" s="55"/>
       <c r="E25" s="55"/>
       <c r="F25" s="55"/>
       <c r="G25" s="55"/>
     </row>
+    <row r="26" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A26" s="55"/>
+      <c r="B26" s="55"/>
+      <c r="C26" s="55"/>
+      <c r="D26" s="55"/>
+      <c r="E26" s="55"/>
+      <c r="F26" s="55"/>
+      <c r="G26" s="55"/>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="E5:G5"/>
   </mergeCells>
   <phoneticPr fontId="11" type="noConversion"/>
-  <conditionalFormatting sqref="D4:D9">
-    <cfRule type="cellIs" dxfId="8" priority="2" operator="greaterThan">
+  <conditionalFormatting sqref="D9:D11">
+    <cfRule type="cellIs" dxfId="8" priority="1" operator="lessThan">
+      <formula>1000</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="D4:D8">
+    <cfRule type="cellIs" dxfId="7" priority="20" operator="greaterThan">
       <formula>1050</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="7" priority="3" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="6" priority="21" operator="greaterThan">
       <formula>500</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="6" priority="4" operator="lessThan">
+    <cfRule type="cellIs" dxfId="5" priority="22" operator="lessThan">
       <formula>500</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="5" priority="5" operator="lessThan">
+    <cfRule type="cellIs" dxfId="4" priority="23" operator="lessThan">
       <formula>500</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="4" priority="6" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="3" priority="24" operator="greaterThan">
       <formula>1050</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="3" priority="7" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="2" priority="25" operator="greaterThan">
       <formula>500</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="2" priority="8" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="1" priority="26" operator="greaterThan">
       <formula>1000</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="1" priority="9" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="0" priority="27" operator="greaterThan">
       <formula>" $ 1,100.00"</formula>
     </cfRule>
-    <cfRule type="colorScale" priority="10">
+    <cfRule type="colorScale" priority="28">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="max"/>
@@ -5607,15 +5629,8 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="D10:D11">
-    <cfRule type="cellIs" dxfId="0" priority="1" operator="lessThan">
-      <formula>1000</formula>
-    </cfRule>
-  </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <ignoredErrors>
-    <ignoredError sqref="B22" formula="1"/>
-  </ignoredErrors>
+  <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -5690,7 +5705,7 @@
       </c>
     </row>
     <row r="4" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A4" s="106">
+      <c r="A4" s="89">
         <v>1</v>
       </c>
       <c r="B4" s="2" t="s">
@@ -5715,14 +5730,14 @@
       <c r="H4" s="14">
         <v>4</v>
       </c>
-      <c r="I4" s="108">
+      <c r="I4" s="91">
         <f ca="1">SUM(F4:F6)</f>
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="J4" s="2"/>
     </row>
     <row r="5" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A5" s="106">
+      <c r="A5" s="89">
         <v>2</v>
       </c>
       <c r="B5" s="2" t="s">
@@ -5747,14 +5762,14 @@
       <c r="H5" s="14">
         <v>5</v>
       </c>
-      <c r="I5" s="109">
+      <c r="I5" s="92">
         <f ca="1">AVERAGE(F4:F6)</f>
-        <v>30</v>
+        <v>30.666666666666668</v>
       </c>
       <c r="J5" s="2"/>
     </row>
     <row r="6" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A6" s="106">
+      <c r="A6" s="89">
         <v>3</v>
       </c>
       <c r="B6" s="2" t="s">
@@ -5769,9 +5784,9 @@
       <c r="E6" s="78" t="s">
         <v>135</v>
       </c>
-      <c r="F6" s="107">
+      <c r="F6" s="90">
         <f ca="1">TODAY()-D6</f>
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="G6" s="2" t="s">
         <v>219</v>
@@ -5783,7 +5798,7 @@
       <c r="J6" s="2"/>
     </row>
     <row r="7" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A7" s="106">
+      <c r="A7" s="89">
         <v>4</v>
       </c>
       <c r="B7" s="2" t="s">

</xml_diff>

<commit_message>
feat: Formulas de Fecha - DATEDIF, NETWORKDAYS, EDATE, WEEKDAY, TODAY y Formato Condicional
</commit_message>
<xml_diff>
--- a/EXCEL/Presupuesto Personal.xlsx
+++ b/EXCEL/Presupuesto Personal.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/1d86eecf8daf4f0d/Documents/SQL Server Management Studio 22/Tienda-sqlserver/EXCEL/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="6" documentId="8_{EE053816-48E3-4E91-A6AD-611A9303676C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{58A4560E-BAA5-4759-B562-A6CBA4876ED6}"/>
+  <xr:revisionPtr revIDLastSave="7" documentId="8_{EE053816-48E3-4E91-A6AD-611A9303676C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{AACE90FA-FE84-4743-AB65-8F6BB954B883}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="12336" windowHeight="12240" firstSheet="1" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="1" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Personal-Budget_2026" sheetId="2" r:id="rId1"/>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="328" uniqueCount="230">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="332" uniqueCount="233">
   <si>
     <t xml:space="preserve">Cantidad </t>
   </si>
@@ -736,6 +736,15 @@
   </si>
   <si>
     <t>Mini Market</t>
+  </si>
+  <si>
+    <t>JUN 25,2026</t>
+  </si>
+  <si>
+    <t>Farmacia</t>
+  </si>
+  <si>
+    <t>Recarga</t>
   </si>
 </sst>
 </file>
@@ -1065,7 +1074,7 @@
     <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="44" fontId="14" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="109">
+  <cellXfs count="110">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -1345,6 +1354,12 @@
     <xf numFmtId="1" fontId="0" fillId="0" borderId="1" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
@@ -1387,11 +1402,8 @@
     <xf numFmtId="0" fontId="8" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
+    <xf numFmtId="0" fontId="16" fillId="17" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1">
+      <alignment vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="4">
@@ -1400,7 +1412,21 @@
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
     <cellStyle name="Percent" xfId="1" builtinId="5"/>
   </cellStyles>
-  <dxfs count="17">
+  <dxfs count="18">
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF00B050"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF00B050"/>
+        </patternFill>
+      </fill>
+    </dxf>
     <dxf>
       <font>
         <color rgb="FF9C0006"/>
@@ -1457,13 +1483,6 @@
       <fill>
         <patternFill>
           <bgColor rgb="FFFF0000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FF00B050"/>
         </patternFill>
       </fill>
     </dxf>
@@ -3352,26 +3371,26 @@
       </c>
     </row>
     <row r="6" spans="1:18" ht="31.2" x14ac:dyDescent="0.3">
-      <c r="A6" s="95" t="s">
+      <c r="A6" s="97" t="s">
         <v>46</v>
       </c>
-      <c r="B6" s="95"/>
-      <c r="C6" s="95"/>
-      <c r="D6" s="95"/>
-      <c r="E6" s="95"/>
-      <c r="F6" s="95"/>
-      <c r="G6" s="95"/>
-      <c r="H6" s="95"/>
-      <c r="I6" s="95"/>
-      <c r="J6" s="95"/>
-      <c r="K6" s="95"/>
-      <c r="L6" s="95"/>
-      <c r="M6" s="95"/>
-      <c r="N6" s="95"/>
-      <c r="O6" s="95"/>
-      <c r="P6" s="95"/>
-      <c r="Q6" s="95"/>
-      <c r="R6" s="95"/>
+      <c r="B6" s="97"/>
+      <c r="C6" s="97"/>
+      <c r="D6" s="97"/>
+      <c r="E6" s="97"/>
+      <c r="F6" s="97"/>
+      <c r="G6" s="97"/>
+      <c r="H6" s="97"/>
+      <c r="I6" s="97"/>
+      <c r="J6" s="97"/>
+      <c r="K6" s="97"/>
+      <c r="L6" s="97"/>
+      <c r="M6" s="97"/>
+      <c r="N6" s="97"/>
+      <c r="O6" s="97"/>
+      <c r="P6" s="97"/>
+      <c r="Q6" s="97"/>
+      <c r="R6" s="97"/>
     </row>
     <row r="8" spans="1:18" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A8" s="34" t="s">
@@ -3608,20 +3627,20 @@
       </c>
     </row>
     <row r="20" spans="1:14" ht="31.2" x14ac:dyDescent="0.3">
-      <c r="A20" s="96" t="s">
+      <c r="A20" s="98" t="s">
         <v>79</v>
       </c>
-      <c r="B20" s="96"/>
-      <c r="C20" s="96"/>
-      <c r="D20" s="96"/>
-      <c r="E20" s="96"/>
-      <c r="F20" s="96"/>
-      <c r="G20" s="96"/>
-      <c r="H20" s="96"/>
-      <c r="I20" s="96"/>
-      <c r="J20" s="96"/>
-      <c r="K20" s="96"/>
-      <c r="L20" s="96"/>
+      <c r="B20" s="98"/>
+      <c r="C20" s="98"/>
+      <c r="D20" s="98"/>
+      <c r="E20" s="98"/>
+      <c r="F20" s="98"/>
+      <c r="G20" s="98"/>
+      <c r="H20" s="98"/>
+      <c r="I20" s="98"/>
+      <c r="J20" s="98"/>
+      <c r="K20" s="98"/>
+      <c r="L20" s="98"/>
       <c r="N20" s="16" t="s">
         <v>90</v>
       </c>
@@ -3788,20 +3807,20 @@
       </c>
     </row>
     <row r="33" spans="1:12" ht="31.2" x14ac:dyDescent="0.3">
-      <c r="A33" s="97" t="s">
+      <c r="A33" s="99" t="s">
         <v>107</v>
       </c>
-      <c r="B33" s="97"/>
-      <c r="C33" s="97"/>
-      <c r="D33" s="97"/>
-      <c r="E33" s="97"/>
-      <c r="F33" s="97"/>
-      <c r="G33" s="97"/>
-      <c r="H33" s="97"/>
-      <c r="I33" s="97"/>
-      <c r="J33" s="97"/>
-      <c r="K33" s="97"/>
-      <c r="L33" s="97"/>
+      <c r="B33" s="99"/>
+      <c r="C33" s="99"/>
+      <c r="D33" s="99"/>
+      <c r="E33" s="99"/>
+      <c r="F33" s="99"/>
+      <c r="G33" s="99"/>
+      <c r="H33" s="99"/>
+      <c r="I33" s="99"/>
+      <c r="J33" s="99"/>
+      <c r="K33" s="99"/>
+      <c r="L33" s="99"/>
     </row>
     <row r="35" spans="1:12" ht="23.4" x14ac:dyDescent="0.3">
       <c r="A35" s="16" t="s">
@@ -3809,20 +3828,20 @@
       </c>
     </row>
     <row r="37" spans="1:12" ht="31.2" x14ac:dyDescent="0.3">
-      <c r="A37" s="98" t="s">
+      <c r="A37" s="100" t="s">
         <v>98</v>
       </c>
-      <c r="B37" s="98"/>
-      <c r="C37" s="98"/>
-      <c r="D37" s="98"/>
-      <c r="E37" s="98"/>
-      <c r="F37" s="98"/>
-      <c r="G37" s="98"/>
-      <c r="H37" s="98"/>
-      <c r="I37" s="98"/>
-      <c r="J37" s="98"/>
-      <c r="K37" s="98"/>
-      <c r="L37" s="98"/>
+      <c r="B37" s="100"/>
+      <c r="C37" s="100"/>
+      <c r="D37" s="100"/>
+      <c r="E37" s="100"/>
+      <c r="F37" s="100"/>
+      <c r="G37" s="100"/>
+      <c r="H37" s="100"/>
+      <c r="I37" s="100"/>
+      <c r="J37" s="100"/>
+      <c r="K37" s="100"/>
+      <c r="L37" s="100"/>
     </row>
     <row r="39" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A39" s="35" t="s">
@@ -3939,16 +3958,16 @@
       </c>
     </row>
     <row r="51" spans="1:9" ht="31.2" x14ac:dyDescent="0.3">
-      <c r="A51" s="99" t="s">
+      <c r="A51" s="101" t="s">
         <v>109</v>
       </c>
-      <c r="B51" s="99"/>
-      <c r="C51" s="99"/>
-      <c r="D51" s="99"/>
-      <c r="E51" s="99"/>
-      <c r="F51" s="99"/>
-      <c r="G51" s="99"/>
-      <c r="H51" s="99"/>
+      <c r="B51" s="101"/>
+      <c r="C51" s="101"/>
+      <c r="D51" s="101"/>
+      <c r="E51" s="101"/>
+      <c r="F51" s="101"/>
+      <c r="G51" s="101"/>
+      <c r="H51" s="101"/>
       <c r="I51" s="40"/>
     </row>
     <row r="53" spans="1:9" ht="28.8" x14ac:dyDescent="0.3">
@@ -4015,18 +4034,18 @@
       </c>
     </row>
     <row r="66" spans="1:10" ht="31.2" x14ac:dyDescent="0.3">
-      <c r="A66" s="94" t="s">
+      <c r="A66" s="96" t="s">
         <v>117</v>
       </c>
-      <c r="B66" s="94"/>
-      <c r="C66" s="94"/>
-      <c r="D66" s="94"/>
-      <c r="E66" s="94"/>
-      <c r="F66" s="94"/>
-      <c r="G66" s="94"/>
-      <c r="H66" s="94"/>
-      <c r="I66" s="94"/>
-      <c r="J66" s="94"/>
+      <c r="B66" s="96"/>
+      <c r="C66" s="96"/>
+      <c r="D66" s="96"/>
+      <c r="E66" s="96"/>
+      <c r="F66" s="96"/>
+      <c r="G66" s="96"/>
+      <c r="H66" s="96"/>
+      <c r="I66" s="96"/>
+      <c r="J66" s="96"/>
     </row>
     <row r="68" spans="1:10" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A68" s="23" t="s">
@@ -4209,11 +4228,11 @@
       </c>
     </row>
     <row r="77" spans="1:10" ht="18" x14ac:dyDescent="0.3">
-      <c r="A77" s="93" t="s">
+      <c r="A77" s="95" t="s">
         <v>165</v>
       </c>
-      <c r="B77" s="93"/>
-      <c r="C77" s="93"/>
+      <c r="B77" s="95"/>
+      <c r="C77" s="95"/>
       <c r="D77" s="46"/>
       <c r="E77" s="46"/>
     </row>
@@ -4373,11 +4392,11 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:4" ht="18" x14ac:dyDescent="0.3">
-      <c r="A1" s="102" t="s">
+      <c r="A1" s="104" t="s">
         <v>4</v>
       </c>
-      <c r="B1" s="103"/>
-      <c r="C1" s="103"/>
+      <c r="B1" s="105"/>
+      <c r="C1" s="105"/>
     </row>
     <row r="2" spans="1:4" ht="15" x14ac:dyDescent="0.3">
       <c r="B2" s="1"/>
@@ -4518,11 +4537,11 @@
       <c r="C16" s="8"/>
     </row>
     <row r="17" spans="1:4" ht="21" x14ac:dyDescent="0.3">
-      <c r="A17" s="104" t="s">
+      <c r="A17" s="106" t="s">
         <v>13</v>
       </c>
-      <c r="B17" s="104"/>
-      <c r="C17" s="104"/>
+      <c r="B17" s="106"/>
+      <c r="C17" s="106"/>
     </row>
     <row r="19" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A19" s="12" t="s">
@@ -4674,11 +4693,11 @@
       </c>
     </row>
     <row r="31" spans="1:4" ht="21" x14ac:dyDescent="0.3">
-      <c r="A31" s="104" t="s">
+      <c r="A31" s="106" t="s">
         <v>13</v>
       </c>
-      <c r="B31" s="104"/>
-      <c r="C31" s="104"/>
+      <c r="B31" s="106"/>
+      <c r="C31" s="106"/>
     </row>
     <row r="33" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A33" s="12" t="s">
@@ -4830,26 +4849,26 @@
       </c>
     </row>
     <row r="46" spans="1:7" ht="25.8" x14ac:dyDescent="0.3">
-      <c r="A46" s="105" t="s">
+      <c r="A46" s="107" t="s">
         <v>27</v>
       </c>
-      <c r="B46" s="105"/>
-      <c r="C46" s="105"/>
-      <c r="D46" s="105"/>
-      <c r="E46" s="105"/>
-      <c r="F46" s="105"/>
-      <c r="G46" s="105"/>
+      <c r="B46" s="107"/>
+      <c r="C46" s="107"/>
+      <c r="D46" s="107"/>
+      <c r="E46" s="107"/>
+      <c r="F46" s="107"/>
+      <c r="G46" s="107"/>
     </row>
     <row r="48" spans="1:7" ht="18" x14ac:dyDescent="0.3">
-      <c r="A48" s="106" t="s">
+      <c r="A48" s="108" t="s">
         <v>28</v>
       </c>
-      <c r="B48" s="106"/>
-      <c r="C48" s="106"/>
-      <c r="D48" s="106"/>
-      <c r="E48" s="106"/>
-      <c r="F48" s="106"/>
-      <c r="G48" s="106"/>
+      <c r="B48" s="108"/>
+      <c r="C48" s="108"/>
+      <c r="D48" s="108"/>
+      <c r="E48" s="108"/>
+      <c r="F48" s="108"/>
+      <c r="G48" s="108"/>
     </row>
     <row r="50" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A50" s="13" t="s">
@@ -5026,11 +5045,11 @@
       <c r="D81" s="60">
         <v>1083</v>
       </c>
-      <c r="E81" s="100" t="s">
+      <c r="E81" s="102" t="s">
         <v>189</v>
       </c>
-      <c r="F81" s="101"/>
-      <c r="G81" s="101"/>
+      <c r="F81" s="103"/>
+      <c r="G81" s="103"/>
     </row>
     <row r="82" spans="1:7" ht="18" x14ac:dyDescent="0.3">
       <c r="A82" s="59" t="s">
@@ -5175,28 +5194,28 @@
   </mergeCells>
   <phoneticPr fontId="11" type="noConversion"/>
   <conditionalFormatting sqref="D80:D85">
-    <cfRule type="cellIs" dxfId="16" priority="11" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="17" priority="11" operator="greaterThan">
       <formula>1050</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="15" priority="12" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="16" priority="12" operator="greaterThan">
       <formula>500</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="14" priority="13" operator="lessThan">
+    <cfRule type="cellIs" dxfId="15" priority="13" operator="lessThan">
       <formula>500</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="13" priority="14" operator="lessThan">
+    <cfRule type="cellIs" dxfId="14" priority="14" operator="lessThan">
       <formula>500</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="12" priority="15" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="13" priority="15" operator="greaterThan">
       <formula>1050</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="11" priority="16" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="12" priority="16" operator="greaterThan">
       <formula>500</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="10" priority="17" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="11" priority="17" operator="greaterThan">
       <formula>1000</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="9" priority="18" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="10" priority="18" operator="greaterThan">
       <formula>" $ 1,100.00"</formula>
     </cfRule>
     <cfRule type="colorScale" priority="19">
@@ -5219,7 +5238,7 @@
   <sheetPr>
     <tabColor rgb="FFFF0000"/>
   </sheetPr>
-  <dimension ref="A2:G26"/>
+  <dimension ref="A2:G27"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="17.77734375" bestFit="1" customWidth="1"/>
@@ -5289,11 +5308,11 @@
       <c r="D5" s="62">
         <v>1083</v>
       </c>
-      <c r="E5" s="107" t="s">
+      <c r="E5" s="93" t="s">
         <v>189</v>
       </c>
-      <c r="F5" s="108"/>
-      <c r="G5" s="108"/>
+      <c r="F5" s="94"/>
+      <c r="G5" s="94"/>
     </row>
     <row r="6" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A6" s="63" t="s">
@@ -5393,17 +5412,25 @@
         <v>225</v>
       </c>
       <c r="D11" s="88">
-        <v>400</v>
+        <v>900</v>
       </c>
       <c r="E11" s="55"/>
       <c r="F11" s="55"/>
       <c r="G11" s="55"/>
     </row>
     <row r="12" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A12" s="55"/>
-      <c r="B12" s="55"/>
-      <c r="C12" s="55"/>
-      <c r="D12" s="55"/>
+      <c r="A12" s="63" t="s">
+        <v>230</v>
+      </c>
+      <c r="B12" s="63" t="s">
+        <v>231</v>
+      </c>
+      <c r="C12" s="63" t="s">
+        <v>232</v>
+      </c>
+      <c r="D12" s="88">
+        <v>230</v>
+      </c>
       <c r="E12" s="55"/>
       <c r="F12" s="55"/>
       <c r="G12" s="55"/>
@@ -5554,7 +5581,7 @@
       </c>
       <c r="B24" s="71">
         <f t="shared" si="0"/>
-        <v>400</v>
+        <v>900</v>
       </c>
       <c r="C24" s="55"/>
       <c r="D24" s="55"/>
@@ -5564,11 +5591,11 @@
     </row>
     <row r="25" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A25" s="70" t="s">
-        <v>193</v>
+        <v>231</v>
       </c>
       <c r="B25" s="71">
-        <f>+SUM(B17:B24)</f>
-        <v>6298</v>
+        <f>SUMIF($B$4:$B$12,A25,$D$4:$D$12)</f>
+        <v>230</v>
       </c>
       <c r="C25" s="55"/>
       <c r="D25" s="55"/>
@@ -5577,56 +5604,75 @@
       <c r="G25" s="55"/>
     </row>
     <row r="26" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A26" s="55"/>
-      <c r="B26" s="55"/>
+      <c r="A26" s="109" t="s">
+        <v>193</v>
+      </c>
+      <c r="B26" s="71">
+        <f>+SUM(B17:B25)</f>
+        <v>7028</v>
+      </c>
       <c r="C26" s="55"/>
       <c r="D26" s="55"/>
       <c r="E26" s="55"/>
       <c r="F26" s="55"/>
       <c r="G26" s="55"/>
     </row>
+    <row r="27" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A27" s="55"/>
+      <c r="B27" s="55"/>
+      <c r="C27" s="55"/>
+      <c r="D27" s="55"/>
+      <c r="E27" s="55"/>
+      <c r="F27" s="55"/>
+      <c r="G27" s="55"/>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="E5:G5"/>
   </mergeCells>
   <phoneticPr fontId="11" type="noConversion"/>
-  <conditionalFormatting sqref="D9:D11">
-    <cfRule type="cellIs" dxfId="8" priority="1" operator="lessThan">
+  <conditionalFormatting sqref="D4:D8">
+    <cfRule type="cellIs" dxfId="9" priority="21" operator="greaterThan">
+      <formula>1050</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="8" priority="22" operator="greaterThan">
+      <formula>500</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="7" priority="23" operator="lessThan">
+      <formula>500</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="6" priority="24" operator="lessThan">
+      <formula>500</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="5" priority="25" operator="greaterThan">
+      <formula>1050</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="4" priority="26" operator="greaterThan">
+      <formula>500</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="3" priority="27" operator="greaterThan">
       <formula>1000</formula>
     </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="D4:D8">
-    <cfRule type="cellIs" dxfId="7" priority="20" operator="greaterThan">
-      <formula>1050</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="6" priority="21" operator="greaterThan">
-      <formula>500</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="5" priority="22" operator="lessThan">
-      <formula>500</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="4" priority="23" operator="lessThan">
-      <formula>500</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="3" priority="24" operator="greaterThan">
-      <formula>1050</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="2" priority="25" operator="greaterThan">
-      <formula>500</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="1" priority="26" operator="greaterThan">
-      <formula>1000</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="0" priority="27" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="2" priority="28" operator="greaterThan">
       <formula>" $ 1,100.00"</formula>
     </cfRule>
-    <cfRule type="colorScale" priority="28">
+    <cfRule type="colorScale" priority="29">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="max"/>
         <color rgb="FFFF7128"/>
         <color rgb="FFFFEF9C"/>
       </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="D9:D11">
+    <cfRule type="cellIs" dxfId="1" priority="2" operator="lessThan">
+      <formula>1000</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="D12">
+    <cfRule type="cellIs" dxfId="0" priority="1" operator="lessThan">
+      <formula>1000</formula>
     </cfRule>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -5732,7 +5778,7 @@
       </c>
       <c r="I4" s="91">
         <f ca="1">SUM(F4:F6)</f>
-        <v>92</v>
+        <v>97</v>
       </c>
       <c r="J4" s="2"/>
     </row>
@@ -5764,7 +5810,7 @@
       </c>
       <c r="I5" s="92">
         <f ca="1">AVERAGE(F4:F6)</f>
-        <v>30.666666666666668</v>
+        <v>32.333333333333336</v>
       </c>
       <c r="J5" s="2"/>
     </row>
@@ -5786,7 +5832,7 @@
       </c>
       <c r="F6" s="90">
         <f ca="1">TODAY()-D6</f>
-        <v>19</v>
+        <v>24</v>
       </c>
       <c r="G6" s="2" t="s">
         <v>219</v>

</xml_diff>

<commit_message>
feat: Porcentajes y Divisiones - Basico, Intermedio y Avanzado con % acumulado
</commit_message>
<xml_diff>
--- a/EXCEL/Presupuesto Personal.xlsx
+++ b/EXCEL/Presupuesto Personal.xlsx
@@ -8,15 +8,16 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/1d86eecf8daf4f0d/Documents/SQL Server Management Studio 22/Tienda-sqlserver/EXCEL/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="10" documentId="8_{EE053816-48E3-4E91-A6AD-611A9303676C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{80D3040D-699B-464B-8F05-187A883198B0}"/>
+  <xr:revisionPtr revIDLastSave="11" documentId="8_{EE053816-48E3-4E91-A6AD-611A9303676C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{B25F7DDF-792B-4102-8524-9E402BBE1367}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="1" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Personal-Budget_2026" sheetId="2" r:id="rId1"/>
     <sheet name="Junio-2026" sheetId="1" r:id="rId2"/>
-    <sheet name="Resumen" sheetId="3" r:id="rId3"/>
-    <sheet name="Libros " sheetId="4" r:id="rId4"/>
+    <sheet name="Junio-30-2026" sheetId="3" r:id="rId3"/>
+    <sheet name="Julio-31-2026" sheetId="5" r:id="rId4"/>
+    <sheet name="Libros " sheetId="4" r:id="rId5"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -34,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="338" uniqueCount="239">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="371" uniqueCount="245">
   <si>
     <t xml:space="preserve">Cantidad </t>
   </si>
@@ -763,6 +764,24 @@
   </si>
   <si>
     <t>Disciplina, Constancia,Persevrancia,Orden</t>
+  </si>
+  <si>
+    <t>Compras</t>
+  </si>
+  <si>
+    <t>Categoria</t>
+  </si>
+  <si>
+    <t>Total RD $</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Total Gastos </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Gatos </t>
+  </si>
+  <si>
+    <t>Mayor Alto Gasto</t>
   </si>
 </sst>
 </file>
@@ -780,7 +799,7 @@
     <numFmt numFmtId="169" formatCode="mm/dd/yyyy;@"/>
     <numFmt numFmtId="170" formatCode="#,##0_ ;\-#,##0\ "/>
   </numFmts>
-  <fonts count="23" x14ac:knownFonts="1">
+  <fonts count="26" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -942,8 +961,28 @@
       <name val="Times New Roman"/>
       <family val="1"/>
     </font>
+    <font>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="Times New Roman"/>
+      <family val="1"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="Times New Roman"/>
+      <family val="1"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="12"/>
+      <color theme="0"/>
+      <name val="Times New Roman"/>
+      <family val="1"/>
+    </font>
   </fonts>
-  <fills count="20">
+  <fills count="22">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -1058,6 +1097,18 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF7CEB99"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFC6C6"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="5">
     <border>
@@ -1120,7 +1171,7 @@
     <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="44" fontId="14" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="119">
+  <cellXfs count="130">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -1355,127 +1406,160 @@
     <xf numFmtId="0" fontId="15" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="169" fontId="18" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="18" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="0" applyFont="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="169" fontId="20" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="20" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="18" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="19" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="19" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="169" fontId="21" fillId="19" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="14" fontId="21" fillId="19" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="19" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="168" fontId="18" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="18" fillId="0" borderId="1" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="170" fontId="18" fillId="0" borderId="1" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="169" fontId="18" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="18" fillId="0" borderId="1" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="168" fontId="18" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="18" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="169" fontId="18" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="168" fontId="18" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="10" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="12" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="10" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="12" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="169" fontId="18" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="14" fontId="18" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="0" applyFont="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="169" fontId="20" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="14" fontId="20" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="18" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="19" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="19" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="169" fontId="21" fillId="19" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="14" fontId="21" fillId="19" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="19" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="168" fontId="18" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="166" fontId="18" fillId="0" borderId="1" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="170" fontId="18" fillId="0" borderId="1" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="169" fontId="18" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="1" fontId="18" fillId="0" borderId="1" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="168" fontId="18" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="1" fontId="18" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="169" fontId="18" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="168" fontId="18" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1">
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="0" xfId="0" applyFont="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="168" fontId="23" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="167" fontId="23" fillId="0" borderId="1" xfId="3" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="167" fontId="23" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="0" xfId="0" applyFont="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="17" fontId="23" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="20" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="21" borderId="0" xfId="0" applyFont="1" applyFill="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="21" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="17" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1">
       <alignment vertical="center"/>
     </xf>
   </cellXfs>
@@ -1485,7 +1569,28 @@
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
     <cellStyle name="Percent" xfId="1" builtinId="5"/>
   </cellStyles>
-  <dxfs count="11">
+  <dxfs count="17">
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF0000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF00B050"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFFF00"/>
+        </patternFill>
+      </fill>
+    </dxf>
     <dxf>
       <fill>
         <patternFill>
@@ -1563,6 +1668,27 @@
       <fill>
         <patternFill>
           <bgColor rgb="FFFF0000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF0000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF00B050"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFFF00"/>
         </patternFill>
       </fill>
     </dxf>
@@ -3392,26 +3518,26 @@
       </c>
     </row>
     <row r="6" spans="1:18" ht="31.2" x14ac:dyDescent="0.3">
-      <c r="A6" s="81" t="s">
+      <c r="A6" s="106" t="s">
         <v>46</v>
       </c>
-      <c r="B6" s="81"/>
-      <c r="C6" s="81"/>
-      <c r="D6" s="81"/>
-      <c r="E6" s="81"/>
-      <c r="F6" s="81"/>
-      <c r="G6" s="81"/>
-      <c r="H6" s="81"/>
-      <c r="I6" s="81"/>
-      <c r="J6" s="81"/>
-      <c r="K6" s="81"/>
-      <c r="L6" s="81"/>
-      <c r="M6" s="81"/>
-      <c r="N6" s="81"/>
-      <c r="O6" s="81"/>
-      <c r="P6" s="81"/>
-      <c r="Q6" s="81"/>
-      <c r="R6" s="81"/>
+      <c r="B6" s="106"/>
+      <c r="C6" s="106"/>
+      <c r="D6" s="106"/>
+      <c r="E6" s="106"/>
+      <c r="F6" s="106"/>
+      <c r="G6" s="106"/>
+      <c r="H6" s="106"/>
+      <c r="I6" s="106"/>
+      <c r="J6" s="106"/>
+      <c r="K6" s="106"/>
+      <c r="L6" s="106"/>
+      <c r="M6" s="106"/>
+      <c r="N6" s="106"/>
+      <c r="O6" s="106"/>
+      <c r="P6" s="106"/>
+      <c r="Q6" s="106"/>
+      <c r="R6" s="106"/>
     </row>
     <row r="8" spans="1:18" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A8" s="34" t="s">
@@ -3648,20 +3774,20 @@
       </c>
     </row>
     <row r="20" spans="1:14" ht="31.2" x14ac:dyDescent="0.3">
-      <c r="A20" s="82" t="s">
+      <c r="A20" s="107" t="s">
         <v>79</v>
       </c>
-      <c r="B20" s="82"/>
-      <c r="C20" s="82"/>
-      <c r="D20" s="82"/>
-      <c r="E20" s="82"/>
-      <c r="F20" s="82"/>
-      <c r="G20" s="82"/>
-      <c r="H20" s="82"/>
-      <c r="I20" s="82"/>
-      <c r="J20" s="82"/>
-      <c r="K20" s="82"/>
-      <c r="L20" s="82"/>
+      <c r="B20" s="107"/>
+      <c r="C20" s="107"/>
+      <c r="D20" s="107"/>
+      <c r="E20" s="107"/>
+      <c r="F20" s="107"/>
+      <c r="G20" s="107"/>
+      <c r="H20" s="107"/>
+      <c r="I20" s="107"/>
+      <c r="J20" s="107"/>
+      <c r="K20" s="107"/>
+      <c r="L20" s="107"/>
       <c r="N20" s="16" t="s">
         <v>90</v>
       </c>
@@ -3828,20 +3954,20 @@
       </c>
     </row>
     <row r="33" spans="1:12" ht="31.2" x14ac:dyDescent="0.3">
-      <c r="A33" s="83" t="s">
+      <c r="A33" s="108" t="s">
         <v>107</v>
       </c>
-      <c r="B33" s="83"/>
-      <c r="C33" s="83"/>
-      <c r="D33" s="83"/>
-      <c r="E33" s="83"/>
-      <c r="F33" s="83"/>
-      <c r="G33" s="83"/>
-      <c r="H33" s="83"/>
-      <c r="I33" s="83"/>
-      <c r="J33" s="83"/>
-      <c r="K33" s="83"/>
-      <c r="L33" s="83"/>
+      <c r="B33" s="108"/>
+      <c r="C33" s="108"/>
+      <c r="D33" s="108"/>
+      <c r="E33" s="108"/>
+      <c r="F33" s="108"/>
+      <c r="G33" s="108"/>
+      <c r="H33" s="108"/>
+      <c r="I33" s="108"/>
+      <c r="J33" s="108"/>
+      <c r="K33" s="108"/>
+      <c r="L33" s="108"/>
     </row>
     <row r="35" spans="1:12" ht="23.4" x14ac:dyDescent="0.3">
       <c r="A35" s="16" t="s">
@@ -3849,20 +3975,20 @@
       </c>
     </row>
     <row r="37" spans="1:12" ht="31.2" x14ac:dyDescent="0.3">
-      <c r="A37" s="84" t="s">
+      <c r="A37" s="109" t="s">
         <v>98</v>
       </c>
-      <c r="B37" s="84"/>
-      <c r="C37" s="84"/>
-      <c r="D37" s="84"/>
-      <c r="E37" s="84"/>
-      <c r="F37" s="84"/>
-      <c r="G37" s="84"/>
-      <c r="H37" s="84"/>
-      <c r="I37" s="84"/>
-      <c r="J37" s="84"/>
-      <c r="K37" s="84"/>
-      <c r="L37" s="84"/>
+      <c r="B37" s="109"/>
+      <c r="C37" s="109"/>
+      <c r="D37" s="109"/>
+      <c r="E37" s="109"/>
+      <c r="F37" s="109"/>
+      <c r="G37" s="109"/>
+      <c r="H37" s="109"/>
+      <c r="I37" s="109"/>
+      <c r="J37" s="109"/>
+      <c r="K37" s="109"/>
+      <c r="L37" s="109"/>
     </row>
     <row r="39" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A39" s="35" t="s">
@@ -3979,16 +4105,16 @@
       </c>
     </row>
     <row r="51" spans="1:9" ht="31.2" x14ac:dyDescent="0.3">
-      <c r="A51" s="85" t="s">
+      <c r="A51" s="110" t="s">
         <v>109</v>
       </c>
-      <c r="B51" s="85"/>
-      <c r="C51" s="85"/>
-      <c r="D51" s="85"/>
-      <c r="E51" s="85"/>
-      <c r="F51" s="85"/>
-      <c r="G51" s="85"/>
-      <c r="H51" s="85"/>
+      <c r="B51" s="110"/>
+      <c r="C51" s="110"/>
+      <c r="D51" s="110"/>
+      <c r="E51" s="110"/>
+      <c r="F51" s="110"/>
+      <c r="G51" s="110"/>
+      <c r="H51" s="110"/>
       <c r="I51" s="40"/>
     </row>
     <row r="53" spans="1:9" ht="28.8" x14ac:dyDescent="0.3">
@@ -4055,18 +4181,18 @@
       </c>
     </row>
     <row r="66" spans="1:10" ht="31.2" x14ac:dyDescent="0.3">
-      <c r="A66" s="80" t="s">
+      <c r="A66" s="105" t="s">
         <v>117</v>
       </c>
-      <c r="B66" s="80"/>
-      <c r="C66" s="80"/>
-      <c r="D66" s="80"/>
-      <c r="E66" s="80"/>
-      <c r="F66" s="80"/>
-      <c r="G66" s="80"/>
-      <c r="H66" s="80"/>
-      <c r="I66" s="80"/>
-      <c r="J66" s="80"/>
+      <c r="B66" s="105"/>
+      <c r="C66" s="105"/>
+      <c r="D66" s="105"/>
+      <c r="E66" s="105"/>
+      <c r="F66" s="105"/>
+      <c r="G66" s="105"/>
+      <c r="H66" s="105"/>
+      <c r="I66" s="105"/>
+      <c r="J66" s="105"/>
     </row>
     <row r="68" spans="1:10" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A68" s="23" t="s">
@@ -4249,11 +4375,11 @@
       </c>
     </row>
     <row r="77" spans="1:10" ht="18" x14ac:dyDescent="0.3">
-      <c r="A77" s="79" t="s">
+      <c r="A77" s="104" t="s">
         <v>165</v>
       </c>
-      <c r="B77" s="79"/>
-      <c r="C77" s="79"/>
+      <c r="B77" s="104"/>
+      <c r="C77" s="104"/>
       <c r="D77" s="46"/>
       <c r="E77" s="46"/>
     </row>
@@ -4413,11 +4539,11 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:4" ht="18" x14ac:dyDescent="0.3">
-      <c r="A1" s="88" t="s">
+      <c r="A1" s="113" t="s">
         <v>4</v>
       </c>
-      <c r="B1" s="89"/>
-      <c r="C1" s="89"/>
+      <c r="B1" s="114"/>
+      <c r="C1" s="114"/>
     </row>
     <row r="2" spans="1:4" ht="15" x14ac:dyDescent="0.3">
       <c r="B2" s="1"/>
@@ -4558,11 +4684,11 @@
       <c r="C16" s="8"/>
     </row>
     <row r="17" spans="1:4" ht="21" x14ac:dyDescent="0.3">
-      <c r="A17" s="90" t="s">
+      <c r="A17" s="115" t="s">
         <v>13</v>
       </c>
-      <c r="B17" s="90"/>
-      <c r="C17" s="90"/>
+      <c r="B17" s="115"/>
+      <c r="C17" s="115"/>
     </row>
     <row r="19" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A19" s="12" t="s">
@@ -4714,11 +4840,11 @@
       </c>
     </row>
     <row r="31" spans="1:4" ht="21" x14ac:dyDescent="0.3">
-      <c r="A31" s="90" t="s">
+      <c r="A31" s="115" t="s">
         <v>13</v>
       </c>
-      <c r="B31" s="90"/>
-      <c r="C31" s="90"/>
+      <c r="B31" s="115"/>
+      <c r="C31" s="115"/>
     </row>
     <row r="33" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A33" s="12" t="s">
@@ -4870,26 +4996,26 @@
       </c>
     </row>
     <row r="46" spans="1:7" ht="25.8" x14ac:dyDescent="0.3">
-      <c r="A46" s="91" t="s">
+      <c r="A46" s="116" t="s">
         <v>27</v>
       </c>
-      <c r="B46" s="91"/>
-      <c r="C46" s="91"/>
-      <c r="D46" s="91"/>
-      <c r="E46" s="91"/>
-      <c r="F46" s="91"/>
-      <c r="G46" s="91"/>
+      <c r="B46" s="116"/>
+      <c r="C46" s="116"/>
+      <c r="D46" s="116"/>
+      <c r="E46" s="116"/>
+      <c r="F46" s="116"/>
+      <c r="G46" s="116"/>
     </row>
     <row r="48" spans="1:7" ht="18" x14ac:dyDescent="0.3">
-      <c r="A48" s="92" t="s">
+      <c r="A48" s="117" t="s">
         <v>28</v>
       </c>
-      <c r="B48" s="92"/>
-      <c r="C48" s="92"/>
-      <c r="D48" s="92"/>
-      <c r="E48" s="92"/>
-      <c r="F48" s="92"/>
-      <c r="G48" s="92"/>
+      <c r="B48" s="117"/>
+      <c r="C48" s="117"/>
+      <c r="D48" s="117"/>
+      <c r="E48" s="117"/>
+      <c r="F48" s="117"/>
+      <c r="G48" s="117"/>
     </row>
     <row r="50" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A50" s="13" t="s">
@@ -5066,11 +5192,11 @@
       <c r="D81" s="60">
         <v>1083</v>
       </c>
-      <c r="E81" s="86" t="s">
+      <c r="E81" s="111" t="s">
         <v>189</v>
       </c>
-      <c r="F81" s="87"/>
-      <c r="G81" s="87"/>
+      <c r="F81" s="112"/>
+      <c r="G81" s="112"/>
     </row>
     <row r="82" spans="1:7" ht="18" x14ac:dyDescent="0.3">
       <c r="A82" s="59" t="s">
@@ -5215,28 +5341,28 @@
   </mergeCells>
   <phoneticPr fontId="11" type="noConversion"/>
   <conditionalFormatting sqref="D80:D85">
-    <cfRule type="cellIs" dxfId="10" priority="11" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="13" priority="11" operator="greaterThan">
       <formula>1050</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="9" priority="12" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="12" priority="12" operator="greaterThan">
       <formula>500</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="8" priority="13" operator="lessThan">
+    <cfRule type="cellIs" dxfId="11" priority="13" operator="lessThan">
       <formula>500</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="7" priority="14" operator="lessThan">
+    <cfRule type="cellIs" dxfId="10" priority="14" operator="lessThan">
       <formula>500</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="6" priority="15" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="9" priority="15" operator="greaterThan">
       <formula>1050</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="5" priority="16" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="8" priority="16" operator="greaterThan">
       <formula>500</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="4" priority="17" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="7" priority="17" operator="greaterThan">
       <formula>1000</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="3" priority="18" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="6" priority="18" operator="greaterThan">
       <formula>" $ 1,100.00"</formula>
     </cfRule>
     <cfRule type="colorScale" priority="19">
@@ -5259,7 +5385,7 @@
   <sheetPr>
     <tabColor rgb="FFFF0000"/>
   </sheetPr>
-  <dimension ref="A2:G29"/>
+  <dimension ref="A2:G30"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="17.77734375" bestFit="1" customWidth="1"/>
@@ -5329,11 +5455,11 @@
       <c r="D5" s="62">
         <v>1083</v>
       </c>
-      <c r="E5" s="78" t="s">
+      <c r="E5" s="118" t="s">
         <v>189</v>
       </c>
-      <c r="F5" s="78"/>
-      <c r="G5" s="78"/>
+      <c r="F5" s="118"/>
+      <c r="G5" s="118"/>
     </row>
     <row r="6" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A6" s="63" t="s">
@@ -5469,9 +5595,7 @@
       <c r="D13" s="75">
         <v>1000</v>
       </c>
-      <c r="E13" s="55">
-        <v>650</v>
-      </c>
+      <c r="E13" s="55"/>
       <c r="F13" s="55"/>
       <c r="G13" s="55"/>
     </row>
@@ -5480,9 +5604,7 @@
       <c r="B14" s="55"/>
       <c r="C14" s="55"/>
       <c r="D14" s="55"/>
-      <c r="E14" s="55">
-        <v>59.11</v>
-      </c>
+      <c r="E14" s="55"/>
       <c r="F14" s="55"/>
       <c r="G14" s="55"/>
     </row>
@@ -5491,9 +5613,7 @@
       <c r="B15" s="55"/>
       <c r="C15" s="55"/>
       <c r="D15" s="55"/>
-      <c r="E15" s="55">
-        <v>132.22</v>
-      </c>
+      <c r="E15" s="55"/>
       <c r="F15" s="55"/>
       <c r="G15" s="55"/>
     </row>
@@ -5504,9 +5624,7 @@
       <c r="B16" s="55"/>
       <c r="C16" s="68"/>
       <c r="D16" s="55"/>
-      <c r="E16" s="55">
-        <v>800</v>
-      </c>
+      <c r="E16" s="55"/>
       <c r="F16" s="55"/>
       <c r="G16" s="55"/>
     </row>
@@ -5519,10 +5637,6 @@
       </c>
       <c r="C17" s="55"/>
       <c r="D17" s="55"/>
-      <c r="E17">
-        <f>SUM(E13:E16)</f>
-        <v>1641.33</v>
-      </c>
       <c r="F17" s="55"/>
       <c r="G17" s="55"/>
     </row>
@@ -5681,7 +5795,9 @@
       <c r="G28" s="55"/>
     </row>
     <row r="29" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A29" s="55"/>
+      <c r="A29" s="55" t="s">
+        <v>243</v>
+      </c>
       <c r="B29" s="55"/>
       <c r="C29" s="55"/>
       <c r="D29" s="55"/>
@@ -5689,21 +5805,38 @@
       <c r="F29" s="55"/>
       <c r="G29" s="55"/>
     </row>
+    <row r="30" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A30" s="129" t="s">
+        <v>244</v>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="E5:G5"/>
   </mergeCells>
   <phoneticPr fontId="11" type="noConversion"/>
   <conditionalFormatting sqref="D4:D13">
-    <cfRule type="cellIs" dxfId="2" priority="1" operator="lessThan">
+    <cfRule type="cellIs" dxfId="5" priority="2" operator="lessThan">
       <formula>500</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="1" priority="2" operator="between">
+    <cfRule type="cellIs" dxfId="4" priority="3" operator="between">
       <formula>1000</formula>
       <formula>501</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="0" priority="4" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="3" priority="5" operator="greaterThan">
       <formula>1000</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B18:B28">
+    <cfRule type="colorScale" priority="1">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FF63BE7B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FFF8696B"/>
+      </colorScale>
     </cfRule>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -5712,6 +5845,431 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6E615C9F-0186-4EF2-A8A9-8EDEC3DDF483}">
+  <dimension ref="A1:I29"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="2" width="14.33203125" customWidth="1"/>
+    <col min="3" max="3" width="16.33203125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="12.33203125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="11.77734375" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A1" s="119"/>
+      <c r="B1" s="119"/>
+      <c r="C1" s="119"/>
+      <c r="D1" s="119"/>
+      <c r="E1" s="119"/>
+      <c r="F1" s="119"/>
+      <c r="G1" s="119"/>
+      <c r="H1" s="119"/>
+      <c r="I1" s="55"/>
+    </row>
+    <row r="2" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A2" s="124" t="s">
+        <v>172</v>
+      </c>
+      <c r="B2" s="124"/>
+      <c r="C2" s="125">
+        <v>46204</v>
+      </c>
+      <c r="D2" s="119"/>
+      <c r="E2" s="119"/>
+      <c r="F2" s="119"/>
+      <c r="G2" s="119"/>
+      <c r="H2" s="119"/>
+      <c r="I2" s="55"/>
+    </row>
+    <row r="3" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A3" s="119"/>
+      <c r="B3" s="119"/>
+      <c r="C3" s="119"/>
+      <c r="D3" s="119"/>
+      <c r="E3" s="119"/>
+      <c r="F3" s="119"/>
+      <c r="G3" s="119"/>
+      <c r="H3" s="119"/>
+      <c r="I3" s="55"/>
+    </row>
+    <row r="4" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A4" s="126" t="s">
+        <v>173</v>
+      </c>
+      <c r="B4" s="126" t="s">
+        <v>47</v>
+      </c>
+      <c r="C4" s="126" t="s">
+        <v>153</v>
+      </c>
+      <c r="D4" s="126" t="s">
+        <v>174</v>
+      </c>
+      <c r="E4" s="126" t="s">
+        <v>175</v>
+      </c>
+      <c r="F4" s="119"/>
+      <c r="G4" s="119"/>
+      <c r="H4" s="119"/>
+      <c r="I4" s="55"/>
+    </row>
+    <row r="5" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A5" s="120"/>
+      <c r="B5" s="120"/>
+      <c r="C5" s="121" t="s">
+        <v>178</v>
+      </c>
+      <c r="D5" s="121" t="s">
+        <v>180</v>
+      </c>
+      <c r="E5" s="122"/>
+      <c r="F5" s="119"/>
+      <c r="G5" s="119"/>
+      <c r="H5" s="119"/>
+      <c r="I5" s="55"/>
+    </row>
+    <row r="6" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A6" s="120"/>
+      <c r="B6" s="120"/>
+      <c r="C6" s="121" t="s">
+        <v>181</v>
+      </c>
+      <c r="D6" s="121" t="s">
+        <v>179</v>
+      </c>
+      <c r="E6" s="122"/>
+      <c r="F6" s="119"/>
+      <c r="G6" s="119"/>
+      <c r="H6" s="119"/>
+      <c r="I6" s="55"/>
+    </row>
+    <row r="7" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A7" s="120"/>
+      <c r="B7" s="120"/>
+      <c r="C7" s="121" t="s">
+        <v>195</v>
+      </c>
+      <c r="D7" s="121" t="s">
+        <v>197</v>
+      </c>
+      <c r="E7" s="122"/>
+      <c r="F7" s="119"/>
+      <c r="G7" s="119"/>
+      <c r="H7" s="119"/>
+      <c r="I7" s="55"/>
+    </row>
+    <row r="8" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A8" s="120"/>
+      <c r="B8" s="120"/>
+      <c r="C8" s="121" t="s">
+        <v>178</v>
+      </c>
+      <c r="D8" s="121" t="s">
+        <v>199</v>
+      </c>
+      <c r="E8" s="122"/>
+      <c r="F8" s="119"/>
+      <c r="G8" s="119"/>
+      <c r="H8" s="119"/>
+      <c r="I8" s="55"/>
+    </row>
+    <row r="9" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A9" s="120"/>
+      <c r="B9" s="120"/>
+      <c r="C9" s="121" t="s">
+        <v>185</v>
+      </c>
+      <c r="D9" s="121" t="s">
+        <v>196</v>
+      </c>
+      <c r="E9" s="122"/>
+      <c r="F9" s="119"/>
+      <c r="G9" s="119"/>
+      <c r="H9" s="119"/>
+      <c r="I9" s="55"/>
+    </row>
+    <row r="10" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A10" s="120"/>
+      <c r="B10" s="120"/>
+      <c r="C10" s="121" t="s">
+        <v>220</v>
+      </c>
+      <c r="D10" s="121" t="s">
+        <v>222</v>
+      </c>
+      <c r="E10" s="123"/>
+      <c r="F10" s="119"/>
+      <c r="G10" s="119"/>
+      <c r="H10" s="119"/>
+      <c r="I10" s="55"/>
+    </row>
+    <row r="11" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A11" s="120">
+        <v>46204</v>
+      </c>
+      <c r="B11" s="120"/>
+      <c r="C11" s="121" t="s">
+        <v>229</v>
+      </c>
+      <c r="D11" s="121" t="s">
+        <v>239</v>
+      </c>
+      <c r="E11" s="123">
+        <v>170</v>
+      </c>
+      <c r="F11" s="119"/>
+      <c r="G11" s="119"/>
+      <c r="H11" s="119"/>
+      <c r="I11" s="55"/>
+    </row>
+    <row r="12" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A12" s="120"/>
+      <c r="B12" s="120"/>
+      <c r="C12" s="121" t="s">
+        <v>224</v>
+      </c>
+      <c r="D12" s="121" t="s">
+        <v>225</v>
+      </c>
+      <c r="E12" s="123"/>
+      <c r="F12" s="119"/>
+      <c r="G12" s="119"/>
+      <c r="H12" s="119"/>
+      <c r="I12" s="55"/>
+    </row>
+    <row r="13" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A13" s="120"/>
+      <c r="B13" s="120"/>
+      <c r="C13" s="121" t="s">
+        <v>231</v>
+      </c>
+      <c r="D13" s="121" t="s">
+        <v>232</v>
+      </c>
+      <c r="E13" s="123"/>
+      <c r="F13" s="119"/>
+      <c r="G13" s="119"/>
+      <c r="H13" s="119"/>
+      <c r="I13" s="55"/>
+    </row>
+    <row r="14" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A14" s="120"/>
+      <c r="B14" s="120"/>
+      <c r="C14" s="121" t="s">
+        <v>235</v>
+      </c>
+      <c r="D14" s="121" t="s">
+        <v>236</v>
+      </c>
+      <c r="E14" s="123"/>
+      <c r="F14" s="119"/>
+      <c r="G14" s="119"/>
+      <c r="H14" s="119"/>
+      <c r="I14" s="55">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="15" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A15" s="119"/>
+      <c r="B15" s="119"/>
+      <c r="C15" s="119"/>
+      <c r="D15" s="119"/>
+      <c r="E15" s="119"/>
+      <c r="F15" s="119"/>
+      <c r="G15" s="119"/>
+      <c r="H15" s="119"/>
+      <c r="I15" s="55">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="16" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A16" s="127" t="s">
+        <v>240</v>
+      </c>
+      <c r="B16" s="127"/>
+      <c r="C16" s="128" t="s">
+        <v>241</v>
+      </c>
+      <c r="D16" s="119"/>
+      <c r="E16" s="119"/>
+      <c r="F16" s="119"/>
+      <c r="G16" s="119"/>
+      <c r="H16" s="119"/>
+      <c r="I16" s="55">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="17" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A17" s="124" t="s">
+        <v>229</v>
+      </c>
+      <c r="B17" s="124"/>
+      <c r="C17" s="119">
+        <f>SUMIF($C$5:$C$14,$A$17,$E$5:$E$14)</f>
+        <v>170</v>
+      </c>
+      <c r="D17" s="119"/>
+      <c r="E17" s="119"/>
+      <c r="F17" s="119"/>
+      <c r="G17" s="119"/>
+      <c r="H17" s="119"/>
+      <c r="I17" s="55">
+        <f>SUM(I14:I16)</f>
+        <v>85</v>
+      </c>
+    </row>
+    <row r="18" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A18" s="124" t="s">
+        <v>193</v>
+      </c>
+      <c r="B18" s="124"/>
+      <c r="C18" s="119"/>
+      <c r="D18" s="119"/>
+      <c r="E18" s="119"/>
+      <c r="F18" s="119"/>
+      <c r="G18" s="119"/>
+      <c r="H18" s="119"/>
+      <c r="I18" s="55">
+        <f>+SUM(I14:I17)</f>
+        <v>170</v>
+      </c>
+    </row>
+    <row r="19" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A19" s="124" t="s">
+        <v>242</v>
+      </c>
+      <c r="B19" s="124"/>
+      <c r="C19" s="119">
+        <f>SUM(C17:C18)</f>
+        <v>170</v>
+      </c>
+      <c r="D19" s="119"/>
+      <c r="E19" s="119"/>
+      <c r="F19" s="119"/>
+      <c r="G19" s="119"/>
+      <c r="H19" s="119"/>
+      <c r="I19" s="55"/>
+    </row>
+    <row r="20" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A20" s="119"/>
+      <c r="B20" s="119"/>
+      <c r="C20" s="119"/>
+      <c r="D20" s="119"/>
+      <c r="E20" s="119"/>
+      <c r="F20" s="119"/>
+      <c r="G20" s="119"/>
+      <c r="H20" s="119"/>
+      <c r="I20" s="55"/>
+    </row>
+    <row r="21" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A21" s="119"/>
+      <c r="B21" s="119"/>
+      <c r="C21" s="119"/>
+      <c r="D21" s="119"/>
+      <c r="E21" s="119"/>
+      <c r="F21" s="119"/>
+      <c r="G21" s="119"/>
+      <c r="H21" s="119"/>
+      <c r="I21" s="55"/>
+    </row>
+    <row r="22" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A22" s="78"/>
+      <c r="B22" s="78"/>
+      <c r="C22" s="78"/>
+      <c r="D22" s="78"/>
+      <c r="E22" s="78"/>
+      <c r="F22" s="78"/>
+      <c r="G22" s="78"/>
+      <c r="H22" s="78"/>
+    </row>
+    <row r="23" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A23" s="78"/>
+      <c r="B23" s="78"/>
+      <c r="C23" s="78"/>
+      <c r="D23" s="78"/>
+      <c r="E23" s="78"/>
+      <c r="F23" s="78"/>
+      <c r="G23" s="78"/>
+      <c r="H23" s="78"/>
+    </row>
+    <row r="24" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A24" s="78"/>
+      <c r="B24" s="78"/>
+      <c r="C24" s="78"/>
+      <c r="D24" s="78"/>
+      <c r="E24" s="78"/>
+      <c r="F24" s="78"/>
+      <c r="G24" s="78"/>
+      <c r="H24" s="78"/>
+    </row>
+    <row r="25" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A25" s="78"/>
+      <c r="B25" s="78"/>
+      <c r="C25" s="78"/>
+      <c r="D25" s="78"/>
+      <c r="E25" s="78"/>
+      <c r="F25" s="78"/>
+      <c r="G25" s="78"/>
+      <c r="H25" s="78"/>
+    </row>
+    <row r="26" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A26" s="78"/>
+      <c r="B26" s="78"/>
+      <c r="C26" s="78"/>
+      <c r="D26" s="78"/>
+      <c r="E26" s="78"/>
+      <c r="F26" s="78"/>
+      <c r="G26" s="78"/>
+      <c r="H26" s="78"/>
+    </row>
+    <row r="27" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A27" s="78"/>
+      <c r="B27" s="78"/>
+      <c r="C27" s="78"/>
+      <c r="D27" s="78"/>
+      <c r="E27" s="78"/>
+      <c r="F27" s="78"/>
+      <c r="G27" s="78"/>
+      <c r="H27" s="78"/>
+    </row>
+    <row r="28" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A28" s="78"/>
+      <c r="B28" s="78"/>
+      <c r="C28" s="78"/>
+      <c r="D28" s="78"/>
+      <c r="E28" s="78"/>
+      <c r="F28" s="78"/>
+      <c r="G28" s="78"/>
+      <c r="H28" s="78"/>
+    </row>
+    <row r="29" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A29" s="78"/>
+      <c r="B29" s="78"/>
+      <c r="C29" s="78"/>
+      <c r="D29" s="78"/>
+      <c r="E29" s="78"/>
+      <c r="F29" s="78"/>
+      <c r="G29" s="78"/>
+      <c r="H29" s="78"/>
+    </row>
+  </sheetData>
+  <conditionalFormatting sqref="E5:E14">
+    <cfRule type="cellIs" dxfId="2" priority="1" operator="lessThan">
+      <formula>500</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="1" priority="2" operator="between">
+      <formula>1000</formula>
+      <formula>501</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="0" priority="3" operator="greaterThan">
+      <formula>1000</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CFFFD5F3-00B0-4AD2-8853-B354DEE4CC20}">
   <sheetPr>
     <tabColor rgb="FF002060"/>
@@ -5732,246 +6290,246 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:11" ht="17.399999999999999" x14ac:dyDescent="0.3">
-      <c r="A1" s="93"/>
-      <c r="B1" s="94" t="s">
+      <c r="A1" s="78"/>
+      <c r="B1" s="79" t="s">
         <v>201</v>
       </c>
-      <c r="C1" s="93"/>
-      <c r="D1" s="95"/>
-      <c r="E1" s="96"/>
-      <c r="F1" s="93"/>
-      <c r="G1" s="93"/>
-      <c r="H1" s="93"/>
-      <c r="I1" s="93"/>
-      <c r="J1" s="93"/>
-      <c r="K1" s="93"/>
+      <c r="C1" s="78"/>
+      <c r="D1" s="80"/>
+      <c r="E1" s="81"/>
+      <c r="F1" s="78"/>
+      <c r="G1" s="78"/>
+      <c r="H1" s="78"/>
+      <c r="I1" s="78"/>
+      <c r="J1" s="78"/>
+      <c r="K1" s="78"/>
     </row>
     <row r="2" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A2" s="97"/>
-      <c r="B2" s="97"/>
-      <c r="C2" s="97"/>
-      <c r="D2" s="98"/>
-      <c r="E2" s="99"/>
-      <c r="F2" s="97"/>
-      <c r="G2" s="97"/>
-      <c r="H2" s="97"/>
-      <c r="I2" s="97"/>
-      <c r="J2" s="97"/>
-      <c r="K2" s="93"/>
-    </row>
-    <row r="3" spans="1:11" s="71" customFormat="1" ht="27.6" x14ac:dyDescent="0.3">
-      <c r="A3" s="100" t="s">
+      <c r="A2" s="82"/>
+      <c r="B2" s="82"/>
+      <c r="C2" s="82"/>
+      <c r="D2" s="83"/>
+      <c r="E2" s="84"/>
+      <c r="F2" s="82"/>
+      <c r="G2" s="82"/>
+      <c r="H2" s="82"/>
+      <c r="I2" s="82"/>
+      <c r="J2" s="82"/>
+      <c r="K2" s="78"/>
+    </row>
+    <row r="3" spans="1:11" s="71" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A3" s="85" t="s">
         <v>209</v>
       </c>
-      <c r="B3" s="101" t="s">
+      <c r="B3" s="86" t="s">
         <v>202</v>
       </c>
-      <c r="C3" s="102" t="s">
+      <c r="C3" s="87" t="s">
         <v>203</v>
       </c>
-      <c r="D3" s="103" t="s">
+      <c r="D3" s="88" t="s">
         <v>204</v>
       </c>
-      <c r="E3" s="104" t="s">
+      <c r="E3" s="89" t="s">
         <v>205</v>
       </c>
-      <c r="F3" s="101" t="s">
+      <c r="F3" s="86" t="s">
         <v>206</v>
       </c>
-      <c r="G3" s="101" t="s">
+      <c r="G3" s="86" t="s">
         <v>56</v>
       </c>
-      <c r="H3" s="101" t="s">
+      <c r="H3" s="86" t="s">
         <v>208</v>
       </c>
-      <c r="I3" s="101" t="s">
+      <c r="I3" s="86" t="s">
         <v>227</v>
       </c>
-      <c r="J3" s="101" t="s">
+      <c r="J3" s="86" t="s">
         <v>207</v>
       </c>
-      <c r="K3" s="105"/>
+      <c r="K3" s="90"/>
     </row>
     <row r="4" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A4" s="106">
+      <c r="A4" s="91">
         <v>1</v>
       </c>
-      <c r="B4" s="107" t="s">
+      <c r="B4" s="92" t="s">
         <v>210</v>
       </c>
-      <c r="C4" s="108" t="s">
+      <c r="C4" s="93" t="s">
         <v>214</v>
       </c>
-      <c r="D4" s="109">
+      <c r="D4" s="94">
         <v>46127</v>
       </c>
-      <c r="E4" s="109">
+      <c r="E4" s="94">
         <v>46154</v>
       </c>
-      <c r="F4" s="110">
+      <c r="F4" s="95">
         <f>E4-D4</f>
         <v>27</v>
       </c>
-      <c r="G4" s="110" t="s">
+      <c r="G4" s="95" t="s">
         <v>218</v>
       </c>
-      <c r="H4" s="111">
+      <c r="H4" s="96">
         <v>4</v>
       </c>
-      <c r="I4" s="112">
+      <c r="I4" s="97">
         <f ca="1">SUM(F4:F6)</f>
-        <v>103</v>
-      </c>
-      <c r="J4" s="110"/>
-      <c r="K4" s="93"/>
+        <v>104</v>
+      </c>
+      <c r="J4" s="95"/>
+      <c r="K4" s="78"/>
     </row>
     <row r="5" spans="1:11" ht="41.4" x14ac:dyDescent="0.3">
-      <c r="A5" s="106">
+      <c r="A5" s="91">
         <v>2</v>
       </c>
-      <c r="B5" s="107" t="s">
+      <c r="B5" s="92" t="s">
         <v>211</v>
       </c>
-      <c r="C5" s="108" t="s">
+      <c r="C5" s="93" t="s">
         <v>215</v>
       </c>
-      <c r="D5" s="113">
+      <c r="D5" s="98">
         <v>46157</v>
       </c>
-      <c r="E5" s="109">
+      <c r="E5" s="94">
         <v>46203</v>
       </c>
-      <c r="F5" s="110">
+      <c r="F5" s="95">
         <f>E5-D5</f>
         <v>46</v>
       </c>
-      <c r="G5" s="110" t="s">
+      <c r="G5" s="95" t="s">
         <v>218</v>
       </c>
-      <c r="H5" s="111">
+      <c r="H5" s="96">
         <v>5</v>
       </c>
-      <c r="I5" s="114">
+      <c r="I5" s="99">
         <f ca="1">AVERAGE(F4:F6)</f>
-        <v>34.333333333333336</v>
-      </c>
-      <c r="J5" s="108" t="s">
+        <v>34.666666666666664</v>
+      </c>
+      <c r="J5" s="93" t="s">
         <v>238</v>
       </c>
-      <c r="K5" s="93"/>
+      <c r="K5" s="78"/>
     </row>
     <row r="6" spans="1:11" ht="41.4" x14ac:dyDescent="0.3">
-      <c r="A6" s="106">
+      <c r="A6" s="91">
         <v>3</v>
       </c>
-      <c r="B6" s="107" t="s">
+      <c r="B6" s="92" t="s">
         <v>212</v>
       </c>
-      <c r="C6" s="108" t="s">
+      <c r="C6" s="93" t="s">
         <v>216</v>
       </c>
-      <c r="D6" s="113">
+      <c r="D6" s="98">
         <v>46174</v>
       </c>
-      <c r="E6" s="115" t="s">
+      <c r="E6" s="100" t="s">
         <v>135</v>
       </c>
-      <c r="F6" s="116">
+      <c r="F6" s="101">
         <f ca="1">TODAY()-D6</f>
-        <v>30</v>
-      </c>
-      <c r="G6" s="110" t="s">
+        <v>31</v>
+      </c>
+      <c r="G6" s="95" t="s">
         <v>219</v>
       </c>
-      <c r="H6" s="111">
+      <c r="H6" s="96">
         <v>5</v>
       </c>
-      <c r="I6" s="111"/>
-      <c r="J6" s="108" t="s">
+      <c r="I6" s="96"/>
+      <c r="J6" s="93" t="s">
         <v>237</v>
       </c>
-      <c r="K6" s="93"/>
+      <c r="K6" s="78"/>
     </row>
     <row r="7" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A7" s="106">
+      <c r="A7" s="91">
         <v>4</v>
       </c>
-      <c r="B7" s="107" t="s">
+      <c r="B7" s="92" t="s">
         <v>213</v>
       </c>
-      <c r="C7" s="108" t="s">
+      <c r="C7" s="93" t="s">
         <v>217</v>
       </c>
-      <c r="D7" s="117" t="s">
+      <c r="D7" s="102" t="s">
         <v>135</v>
       </c>
-      <c r="E7" s="115" t="s">
+      <c r="E7" s="100" t="s">
         <v>135</v>
       </c>
-      <c r="F7" s="110" t="s">
+      <c r="F7" s="95" t="s">
         <v>135</v>
       </c>
-      <c r="G7" s="110" t="s">
+      <c r="G7" s="95" t="s">
         <v>63</v>
       </c>
-      <c r="H7" s="111">
+      <c r="H7" s="96">
         <v>0</v>
       </c>
-      <c r="I7" s="111"/>
-      <c r="J7" s="110"/>
-      <c r="K7" s="93"/>
+      <c r="I7" s="96"/>
+      <c r="J7" s="95"/>
+      <c r="K7" s="78"/>
     </row>
     <row r="8" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A8" s="93"/>
-      <c r="B8" s="93"/>
-      <c r="C8" s="93"/>
-      <c r="D8" s="95"/>
-      <c r="E8" s="118"/>
-      <c r="F8" s="93"/>
-      <c r="G8" s="93"/>
-      <c r="H8" s="93"/>
-      <c r="I8" s="93"/>
-      <c r="J8" s="93"/>
-      <c r="K8" s="93"/>
+      <c r="A8" s="78"/>
+      <c r="B8" s="78"/>
+      <c r="C8" s="78"/>
+      <c r="D8" s="80"/>
+      <c r="E8" s="103"/>
+      <c r="F8" s="78"/>
+      <c r="G8" s="78"/>
+      <c r="H8" s="78"/>
+      <c r="I8" s="78"/>
+      <c r="J8" s="78"/>
+      <c r="K8" s="78"/>
     </row>
     <row r="9" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A9" s="93"/>
-      <c r="B9" s="93"/>
-      <c r="C9" s="93"/>
-      <c r="D9" s="95"/>
-      <c r="E9" s="96"/>
-      <c r="F9" s="93"/>
-      <c r="G9" s="93"/>
-      <c r="H9" s="93"/>
-      <c r="I9" s="93"/>
-      <c r="J9" s="93"/>
-      <c r="K9" s="93"/>
+      <c r="A9" s="78"/>
+      <c r="B9" s="78"/>
+      <c r="C9" s="78"/>
+      <c r="D9" s="80"/>
+      <c r="E9" s="81"/>
+      <c r="F9" s="78"/>
+      <c r="G9" s="78"/>
+      <c r="H9" s="78"/>
+      <c r="I9" s="78"/>
+      <c r="J9" s="78"/>
+      <c r="K9" s="78"/>
     </row>
     <row r="10" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A10" s="93"/>
-      <c r="B10" s="93"/>
-      <c r="C10" s="93"/>
-      <c r="D10" s="95"/>
-      <c r="E10" s="96"/>
-      <c r="F10" s="93"/>
-      <c r="G10" s="93"/>
-      <c r="H10" s="93"/>
-      <c r="I10" s="93"/>
-      <c r="J10" s="93"/>
-      <c r="K10" s="93"/>
+      <c r="A10" s="78"/>
+      <c r="B10" s="78"/>
+      <c r="C10" s="78"/>
+      <c r="D10" s="80"/>
+      <c r="E10" s="81"/>
+      <c r="F10" s="78"/>
+      <c r="G10" s="78"/>
+      <c r="H10" s="78"/>
+      <c r="I10" s="78"/>
+      <c r="J10" s="78"/>
+      <c r="K10" s="78"/>
     </row>
     <row r="11" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A11" s="93"/>
-      <c r="B11" s="93"/>
-      <c r="C11" s="93"/>
-      <c r="D11" s="95"/>
-      <c r="E11" s="96"/>
-      <c r="F11" s="93"/>
-      <c r="G11" s="93"/>
-      <c r="H11" s="93"/>
-      <c r="I11" s="93"/>
-      <c r="J11" s="93"/>
-      <c r="K11" s="93"/>
+      <c r="A11" s="78"/>
+      <c r="B11" s="78"/>
+      <c r="C11" s="78"/>
+      <c r="D11" s="80"/>
+      <c r="E11" s="81"/>
+      <c r="F11" s="78"/>
+      <c r="G11" s="78"/>
+      <c r="H11" s="78"/>
+      <c r="I11" s="78"/>
+      <c r="J11" s="78"/>
+      <c r="K11" s="78"/>
     </row>
     <row r="12" spans="1:11" x14ac:dyDescent="0.3">
       <c r="D12" s="74"/>

</xml_diff>

<commit_message>
feat: Pestanas Excel completas - Inicio, Insertar y Trazo a fondo con graficos, mapas y simbolos
</commit_message>
<xml_diff>
--- a/EXCEL/Presupuesto Personal.xlsx
+++ b/EXCEL/Presupuesto Personal.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/1d86eecf8daf4f0d/Documents/SQL Server Management Studio 22/Tienda-sqlserver/EXCEL/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="11" documentId="8_{EE053816-48E3-4E91-A6AD-611A9303676C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{B25F7DDF-792B-4102-8524-9E402BBE1367}"/>
+  <xr:revisionPtr revIDLastSave="20" documentId="8_{EE053816-48E3-4E91-A6AD-611A9303676C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{4A3C341F-FFCD-42C0-8A6E-6C0A04255D82}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Personal-Budget_2026" sheetId="2" r:id="rId1"/>
@@ -1171,7 +1171,7 @@
     <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="44" fontId="14" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="130">
+  <cellXfs count="129">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -1484,6 +1484,36 @@
     <xf numFmtId="168" fontId="18" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="0" xfId="0" applyFont="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="168" fontId="23" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="167" fontId="23" fillId="0" borderId="1" xfId="3" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="167" fontId="23" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="0" xfId="0" applyFont="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="17" fontId="23" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="20" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="21" borderId="0" xfId="0" applyFont="1" applyFill="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="17" borderId="0" xfId="0" applyFont="1" applyFill="1">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
@@ -1529,47 +1559,14 @@
     <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="23" fillId="0" borderId="0" xfId="0" applyFont="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="168" fontId="23" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="167" fontId="23" fillId="0" borderId="1" xfId="3" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="167" fontId="23" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="0" xfId="0" applyFont="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="17" fontId="23" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="20" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="21" borderId="0" xfId="0" applyFont="1" applyFill="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="21" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="17" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1">
-      <alignment vertical="center"/>
-    </xf>
   </cellXfs>
   <cellStyles count="4">
-    <cellStyle name="Comma" xfId="2" builtinId="3"/>
-    <cellStyle name="Currency" xfId="3" builtinId="4"/>
+    <cellStyle name="Millares" xfId="2" builtinId="3"/>
+    <cellStyle name="Moneda" xfId="3" builtinId="4"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
-    <cellStyle name="Percent" xfId="1" builtinId="5"/>
+    <cellStyle name="Porcentaje" xfId="1" builtinId="5"/>
   </cellStyles>
-  <dxfs count="17">
+  <dxfs count="14">
     <dxf>
       <fill>
         <patternFill>
@@ -1671,27 +1668,6 @@
         </patternFill>
       </fill>
     </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFF0000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FF00B050"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFFF00"/>
-        </patternFill>
-      </fill>
-    </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
@@ -1708,7 +1684,7 @@
 <file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
 <c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
   <c:date1904 val="0"/>
-  <c:lang val="en-US"/>
+  <c:lang val="es-MX"/>
   <c:roundedCorners val="0"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
@@ -3488,7 +3464,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E523AC75-1258-4F5B-8926-C1F345A2AD27}">
   <dimension ref="A2:R81"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="11.109375" customWidth="1"/>
     <col min="2" max="2" width="14.5546875" customWidth="1"/>
@@ -3518,26 +3494,26 @@
       </c>
     </row>
     <row r="6" spans="1:18" ht="31.2" x14ac:dyDescent="0.3">
-      <c r="A6" s="106" t="s">
+      <c r="A6" s="116" t="s">
         <v>46</v>
       </c>
-      <c r="B6" s="106"/>
-      <c r="C6" s="106"/>
-      <c r="D6" s="106"/>
-      <c r="E6" s="106"/>
-      <c r="F6" s="106"/>
-      <c r="G6" s="106"/>
-      <c r="H6" s="106"/>
-      <c r="I6" s="106"/>
-      <c r="J6" s="106"/>
-      <c r="K6" s="106"/>
-      <c r="L6" s="106"/>
-      <c r="M6" s="106"/>
-      <c r="N6" s="106"/>
-      <c r="O6" s="106"/>
-      <c r="P6" s="106"/>
-      <c r="Q6" s="106"/>
-      <c r="R6" s="106"/>
+      <c r="B6" s="116"/>
+      <c r="C6" s="116"/>
+      <c r="D6" s="116"/>
+      <c r="E6" s="116"/>
+      <c r="F6" s="116"/>
+      <c r="G6" s="116"/>
+      <c r="H6" s="116"/>
+      <c r="I6" s="116"/>
+      <c r="J6" s="116"/>
+      <c r="K6" s="116"/>
+      <c r="L6" s="116"/>
+      <c r="M6" s="116"/>
+      <c r="N6" s="116"/>
+      <c r="O6" s="116"/>
+      <c r="P6" s="116"/>
+      <c r="Q6" s="116"/>
+      <c r="R6" s="116"/>
     </row>
     <row r="8" spans="1:18" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A8" s="34" t="s">
@@ -3774,20 +3750,20 @@
       </c>
     </row>
     <row r="20" spans="1:14" ht="31.2" x14ac:dyDescent="0.3">
-      <c r="A20" s="107" t="s">
+      <c r="A20" s="117" t="s">
         <v>79</v>
       </c>
-      <c r="B20" s="107"/>
-      <c r="C20" s="107"/>
-      <c r="D20" s="107"/>
-      <c r="E20" s="107"/>
-      <c r="F20" s="107"/>
-      <c r="G20" s="107"/>
-      <c r="H20" s="107"/>
-      <c r="I20" s="107"/>
-      <c r="J20" s="107"/>
-      <c r="K20" s="107"/>
-      <c r="L20" s="107"/>
+      <c r="B20" s="117"/>
+      <c r="C20" s="117"/>
+      <c r="D20" s="117"/>
+      <c r="E20" s="117"/>
+      <c r="F20" s="117"/>
+      <c r="G20" s="117"/>
+      <c r="H20" s="117"/>
+      <c r="I20" s="117"/>
+      <c r="J20" s="117"/>
+      <c r="K20" s="117"/>
+      <c r="L20" s="117"/>
       <c r="N20" s="16" t="s">
         <v>90</v>
       </c>
@@ -3954,20 +3930,20 @@
       </c>
     </row>
     <row r="33" spans="1:12" ht="31.2" x14ac:dyDescent="0.3">
-      <c r="A33" s="108" t="s">
+      <c r="A33" s="118" t="s">
         <v>107</v>
       </c>
-      <c r="B33" s="108"/>
-      <c r="C33" s="108"/>
-      <c r="D33" s="108"/>
-      <c r="E33" s="108"/>
-      <c r="F33" s="108"/>
-      <c r="G33" s="108"/>
-      <c r="H33" s="108"/>
-      <c r="I33" s="108"/>
-      <c r="J33" s="108"/>
-      <c r="K33" s="108"/>
-      <c r="L33" s="108"/>
+      <c r="B33" s="118"/>
+      <c r="C33" s="118"/>
+      <c r="D33" s="118"/>
+      <c r="E33" s="118"/>
+      <c r="F33" s="118"/>
+      <c r="G33" s="118"/>
+      <c r="H33" s="118"/>
+      <c r="I33" s="118"/>
+      <c r="J33" s="118"/>
+      <c r="K33" s="118"/>
+      <c r="L33" s="118"/>
     </row>
     <row r="35" spans="1:12" ht="23.4" x14ac:dyDescent="0.3">
       <c r="A35" s="16" t="s">
@@ -3975,20 +3951,20 @@
       </c>
     </row>
     <row r="37" spans="1:12" ht="31.2" x14ac:dyDescent="0.3">
-      <c r="A37" s="109" t="s">
+      <c r="A37" s="119" t="s">
         <v>98</v>
       </c>
-      <c r="B37" s="109"/>
-      <c r="C37" s="109"/>
-      <c r="D37" s="109"/>
-      <c r="E37" s="109"/>
-      <c r="F37" s="109"/>
-      <c r="G37" s="109"/>
-      <c r="H37" s="109"/>
-      <c r="I37" s="109"/>
-      <c r="J37" s="109"/>
-      <c r="K37" s="109"/>
-      <c r="L37" s="109"/>
+      <c r="B37" s="119"/>
+      <c r="C37" s="119"/>
+      <c r="D37" s="119"/>
+      <c r="E37" s="119"/>
+      <c r="F37" s="119"/>
+      <c r="G37" s="119"/>
+      <c r="H37" s="119"/>
+      <c r="I37" s="119"/>
+      <c r="J37" s="119"/>
+      <c r="K37" s="119"/>
+      <c r="L37" s="119"/>
     </row>
     <row r="39" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A39" s="35" t="s">
@@ -4105,16 +4081,16 @@
       </c>
     </row>
     <row r="51" spans="1:9" ht="31.2" x14ac:dyDescent="0.3">
-      <c r="A51" s="110" t="s">
+      <c r="A51" s="120" t="s">
         <v>109</v>
       </c>
-      <c r="B51" s="110"/>
-      <c r="C51" s="110"/>
-      <c r="D51" s="110"/>
-      <c r="E51" s="110"/>
-      <c r="F51" s="110"/>
-      <c r="G51" s="110"/>
-      <c r="H51" s="110"/>
+      <c r="B51" s="120"/>
+      <c r="C51" s="120"/>
+      <c r="D51" s="120"/>
+      <c r="E51" s="120"/>
+      <c r="F51" s="120"/>
+      <c r="G51" s="120"/>
+      <c r="H51" s="120"/>
       <c r="I51" s="40"/>
     </row>
     <row r="53" spans="1:9" ht="28.8" x14ac:dyDescent="0.3">
@@ -4181,18 +4157,18 @@
       </c>
     </row>
     <row r="66" spans="1:10" ht="31.2" x14ac:dyDescent="0.3">
-      <c r="A66" s="105" t="s">
+      <c r="A66" s="115" t="s">
         <v>117</v>
       </c>
-      <c r="B66" s="105"/>
-      <c r="C66" s="105"/>
-      <c r="D66" s="105"/>
-      <c r="E66" s="105"/>
-      <c r="F66" s="105"/>
-      <c r="G66" s="105"/>
-      <c r="H66" s="105"/>
-      <c r="I66" s="105"/>
-      <c r="J66" s="105"/>
+      <c r="B66" s="115"/>
+      <c r="C66" s="115"/>
+      <c r="D66" s="115"/>
+      <c r="E66" s="115"/>
+      <c r="F66" s="115"/>
+      <c r="G66" s="115"/>
+      <c r="H66" s="115"/>
+      <c r="I66" s="115"/>
+      <c r="J66" s="115"/>
     </row>
     <row r="68" spans="1:10" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A68" s="23" t="s">
@@ -4246,7 +4222,7 @@
         <v>130</v>
       </c>
     </row>
-    <row r="70" spans="1:10" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="70" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A70" s="18" t="s">
         <v>124</v>
       </c>
@@ -4375,11 +4351,11 @@
       </c>
     </row>
     <row r="77" spans="1:10" ht="18" x14ac:dyDescent="0.3">
-      <c r="A77" s="104" t="s">
+      <c r="A77" s="114" t="s">
         <v>165</v>
       </c>
-      <c r="B77" s="104"/>
-      <c r="C77" s="104"/>
+      <c r="B77" s="114"/>
+      <c r="C77" s="114"/>
       <c r="D77" s="46"/>
       <c r="E77" s="46"/>
     </row>
@@ -4528,7 +4504,7 @@
     <tabColor theme="1"/>
   </sheetPr>
   <dimension ref="A1:G96"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="17.33203125" customWidth="1"/>
     <col min="2" max="2" width="22.6640625" customWidth="1"/>
@@ -4539,11 +4515,11 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:4" ht="18" x14ac:dyDescent="0.3">
-      <c r="A1" s="113" t="s">
+      <c r="A1" s="123" t="s">
         <v>4</v>
       </c>
-      <c r="B1" s="114"/>
-      <c r="C1" s="114"/>
+      <c r="B1" s="124"/>
+      <c r="C1" s="124"/>
     </row>
     <row r="2" spans="1:4" ht="15" x14ac:dyDescent="0.3">
       <c r="B2" s="1"/>
@@ -4684,11 +4660,11 @@
       <c r="C16" s="8"/>
     </row>
     <row r="17" spans="1:4" ht="21" x14ac:dyDescent="0.3">
-      <c r="A17" s="115" t="s">
+      <c r="A17" s="125" t="s">
         <v>13</v>
       </c>
-      <c r="B17" s="115"/>
-      <c r="C17" s="115"/>
+      <c r="B17" s="125"/>
+      <c r="C17" s="125"/>
     </row>
     <row r="19" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A19" s="12" t="s">
@@ -4840,11 +4816,11 @@
       </c>
     </row>
     <row r="31" spans="1:4" ht="21" x14ac:dyDescent="0.3">
-      <c r="A31" s="115" t="s">
+      <c r="A31" s="125" t="s">
         <v>13</v>
       </c>
-      <c r="B31" s="115"/>
-      <c r="C31" s="115"/>
+      <c r="B31" s="125"/>
+      <c r="C31" s="125"/>
     </row>
     <row r="33" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A33" s="12" t="s">
@@ -4996,26 +4972,26 @@
       </c>
     </row>
     <row r="46" spans="1:7" ht="25.8" x14ac:dyDescent="0.3">
-      <c r="A46" s="116" t="s">
+      <c r="A46" s="126" t="s">
         <v>27</v>
       </c>
-      <c r="B46" s="116"/>
-      <c r="C46" s="116"/>
-      <c r="D46" s="116"/>
-      <c r="E46" s="116"/>
-      <c r="F46" s="116"/>
-      <c r="G46" s="116"/>
+      <c r="B46" s="126"/>
+      <c r="C46" s="126"/>
+      <c r="D46" s="126"/>
+      <c r="E46" s="126"/>
+      <c r="F46" s="126"/>
+      <c r="G46" s="126"/>
     </row>
     <row r="48" spans="1:7" ht="18" x14ac:dyDescent="0.3">
-      <c r="A48" s="117" t="s">
+      <c r="A48" s="127" t="s">
         <v>28</v>
       </c>
-      <c r="B48" s="117"/>
-      <c r="C48" s="117"/>
-      <c r="D48" s="117"/>
-      <c r="E48" s="117"/>
-      <c r="F48" s="117"/>
-      <c r="G48" s="117"/>
+      <c r="B48" s="127"/>
+      <c r="C48" s="127"/>
+      <c r="D48" s="127"/>
+      <c r="E48" s="127"/>
+      <c r="F48" s="127"/>
+      <c r="G48" s="127"/>
     </row>
     <row r="50" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A50" s="13" t="s">
@@ -5192,11 +5168,11 @@
       <c r="D81" s="60">
         <v>1083</v>
       </c>
-      <c r="E81" s="111" t="s">
+      <c r="E81" s="121" t="s">
         <v>189</v>
       </c>
-      <c r="F81" s="112"/>
-      <c r="G81" s="112"/>
+      <c r="F81" s="122"/>
+      <c r="G81" s="122"/>
     </row>
     <row r="82" spans="1:7" ht="18" x14ac:dyDescent="0.3">
       <c r="A82" s="59" t="s">
@@ -5386,7 +5362,7 @@
     <tabColor rgb="FFFF0000"/>
   </sheetPr>
   <dimension ref="A2:G30"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="17.77734375" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="17.88671875" bestFit="1" customWidth="1"/>
@@ -5455,11 +5431,11 @@
       <c r="D5" s="62">
         <v>1083</v>
       </c>
-      <c r="E5" s="118" t="s">
+      <c r="E5" s="128" t="s">
         <v>189</v>
       </c>
-      <c r="F5" s="118"/>
-      <c r="G5" s="118"/>
+      <c r="F5" s="128"/>
+      <c r="G5" s="128"/>
     </row>
     <row r="6" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A6" s="63" t="s">
@@ -5806,7 +5782,7 @@
       <c r="G29" s="55"/>
     </row>
     <row r="30" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A30" s="129" t="s">
+      <c r="A30" s="113" t="s">
         <v>244</v>
       </c>
     </row>
@@ -5815,6 +5791,18 @@
     <mergeCell ref="E5:G5"/>
   </mergeCells>
   <phoneticPr fontId="11" type="noConversion"/>
+  <conditionalFormatting sqref="B18:B28">
+    <cfRule type="colorScale" priority="1">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FF63BE7B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FFF8696B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
   <conditionalFormatting sqref="D4:D13">
     <cfRule type="cellIs" dxfId="5" priority="2" operator="lessThan">
       <formula>500</formula>
@@ -5827,18 +5815,6 @@
       <formula>1000</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B18:B28">
-    <cfRule type="colorScale" priority="1">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FF63BE7B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FFF8696B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
@@ -5847,7 +5823,7 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6E615C9F-0186-4EF2-A8A9-8EDEC3DDF483}">
   <dimension ref="A1:I29"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="2" width="14.33203125" customWidth="1"/>
     <col min="3" max="3" width="16.33203125" bestFit="1" customWidth="1"/>
@@ -5856,320 +5832,320 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A1" s="119"/>
-      <c r="B1" s="119"/>
-      <c r="C1" s="119"/>
-      <c r="D1" s="119"/>
-      <c r="E1" s="119"/>
-      <c r="F1" s="119"/>
-      <c r="G1" s="119"/>
-      <c r="H1" s="119"/>
+      <c r="A1" s="104"/>
+      <c r="B1" s="104"/>
+      <c r="C1" s="104"/>
+      <c r="D1" s="104"/>
+      <c r="E1" s="104"/>
+      <c r="F1" s="104"/>
+      <c r="G1" s="104"/>
+      <c r="H1" s="104"/>
       <c r="I1" s="55"/>
     </row>
     <row r="2" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A2" s="124" t="s">
+      <c r="A2" s="109" t="s">
         <v>172</v>
       </c>
-      <c r="B2" s="124"/>
-      <c r="C2" s="125">
+      <c r="B2" s="109"/>
+      <c r="C2" s="110">
         <v>46204</v>
       </c>
-      <c r="D2" s="119"/>
-      <c r="E2" s="119"/>
-      <c r="F2" s="119"/>
-      <c r="G2" s="119"/>
-      <c r="H2" s="119"/>
+      <c r="D2" s="104"/>
+      <c r="E2" s="104"/>
+      <c r="F2" s="104"/>
+      <c r="G2" s="104"/>
+      <c r="H2" s="104"/>
       <c r="I2" s="55"/>
     </row>
     <row r="3" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A3" s="119"/>
-      <c r="B3" s="119"/>
-      <c r="C3" s="119"/>
-      <c r="D3" s="119"/>
-      <c r="E3" s="119"/>
-      <c r="F3" s="119"/>
-      <c r="G3" s="119"/>
-      <c r="H3" s="119"/>
+      <c r="A3" s="104"/>
+      <c r="B3" s="104"/>
+      <c r="C3" s="104"/>
+      <c r="D3" s="104"/>
+      <c r="E3" s="104"/>
+      <c r="F3" s="104"/>
+      <c r="G3" s="104"/>
+      <c r="H3" s="104"/>
       <c r="I3" s="55"/>
     </row>
     <row r="4" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A4" s="126" t="s">
+      <c r="A4" s="111" t="s">
         <v>173</v>
       </c>
-      <c r="B4" s="126" t="s">
+      <c r="B4" s="111" t="s">
         <v>47</v>
       </c>
-      <c r="C4" s="126" t="s">
+      <c r="C4" s="111" t="s">
         <v>153</v>
       </c>
-      <c r="D4" s="126" t="s">
+      <c r="D4" s="111" t="s">
         <v>174</v>
       </c>
-      <c r="E4" s="126" t="s">
+      <c r="E4" s="111" t="s">
         <v>175</v>
       </c>
-      <c r="F4" s="119"/>
-      <c r="G4" s="119"/>
-      <c r="H4" s="119"/>
+      <c r="F4" s="104"/>
+      <c r="G4" s="104"/>
+      <c r="H4" s="104"/>
       <c r="I4" s="55"/>
     </row>
     <row r="5" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A5" s="120"/>
-      <c r="B5" s="120"/>
-      <c r="C5" s="121" t="s">
+      <c r="A5" s="105"/>
+      <c r="B5" s="105"/>
+      <c r="C5" s="106" t="s">
         <v>178</v>
       </c>
-      <c r="D5" s="121" t="s">
+      <c r="D5" s="106" t="s">
         <v>180</v>
       </c>
-      <c r="E5" s="122"/>
-      <c r="F5" s="119"/>
-      <c r="G5" s="119"/>
-      <c r="H5" s="119"/>
+      <c r="E5" s="107"/>
+      <c r="F5" s="104"/>
+      <c r="G5" s="104"/>
+      <c r="H5" s="104"/>
       <c r="I5" s="55"/>
     </row>
     <row r="6" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A6" s="120"/>
-      <c r="B6" s="120"/>
-      <c r="C6" s="121" t="s">
+      <c r="A6" s="105"/>
+      <c r="B6" s="105"/>
+      <c r="C6" s="106" t="s">
         <v>181</v>
       </c>
-      <c r="D6" s="121" t="s">
+      <c r="D6" s="106" t="s">
         <v>179</v>
       </c>
-      <c r="E6" s="122"/>
-      <c r="F6" s="119"/>
-      <c r="G6" s="119"/>
-      <c r="H6" s="119"/>
+      <c r="E6" s="107"/>
+      <c r="F6" s="104"/>
+      <c r="G6" s="104"/>
+      <c r="H6" s="104"/>
       <c r="I6" s="55"/>
     </row>
     <row r="7" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A7" s="120"/>
-      <c r="B7" s="120"/>
-      <c r="C7" s="121" t="s">
+      <c r="A7" s="105"/>
+      <c r="B7" s="105"/>
+      <c r="C7" s="106" t="s">
         <v>195</v>
       </c>
-      <c r="D7" s="121" t="s">
+      <c r="D7" s="106" t="s">
         <v>197</v>
       </c>
-      <c r="E7" s="122"/>
-      <c r="F7" s="119"/>
-      <c r="G7" s="119"/>
-      <c r="H7" s="119"/>
+      <c r="E7" s="107"/>
+      <c r="F7" s="104"/>
+      <c r="G7" s="104"/>
+      <c r="H7" s="104"/>
       <c r="I7" s="55"/>
     </row>
     <row r="8" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A8" s="120"/>
-      <c r="B8" s="120"/>
-      <c r="C8" s="121" t="s">
+      <c r="A8" s="105"/>
+      <c r="B8" s="105"/>
+      <c r="C8" s="106" t="s">
         <v>178</v>
       </c>
-      <c r="D8" s="121" t="s">
+      <c r="D8" s="106" t="s">
         <v>199</v>
       </c>
-      <c r="E8" s="122"/>
-      <c r="F8" s="119"/>
-      <c r="G8" s="119"/>
-      <c r="H8" s="119"/>
+      <c r="E8" s="107"/>
+      <c r="F8" s="104"/>
+      <c r="G8" s="104"/>
+      <c r="H8" s="104"/>
       <c r="I8" s="55"/>
     </row>
     <row r="9" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A9" s="120"/>
-      <c r="B9" s="120"/>
-      <c r="C9" s="121" t="s">
+      <c r="A9" s="105"/>
+      <c r="B9" s="105"/>
+      <c r="C9" s="106" t="s">
         <v>185</v>
       </c>
-      <c r="D9" s="121" t="s">
+      <c r="D9" s="106" t="s">
         <v>196</v>
       </c>
-      <c r="E9" s="122"/>
-      <c r="F9" s="119"/>
-      <c r="G9" s="119"/>
-      <c r="H9" s="119"/>
+      <c r="E9" s="107"/>
+      <c r="F9" s="104"/>
+      <c r="G9" s="104"/>
+      <c r="H9" s="104"/>
       <c r="I9" s="55"/>
     </row>
     <row r="10" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A10" s="120"/>
-      <c r="B10" s="120"/>
-      <c r="C10" s="121" t="s">
+      <c r="A10" s="105"/>
+      <c r="B10" s="105"/>
+      <c r="C10" s="106" t="s">
         <v>220</v>
       </c>
-      <c r="D10" s="121" t="s">
+      <c r="D10" s="106" t="s">
         <v>222</v>
       </c>
-      <c r="E10" s="123"/>
-      <c r="F10" s="119"/>
-      <c r="G10" s="119"/>
-      <c r="H10" s="119"/>
+      <c r="E10" s="108"/>
+      <c r="F10" s="104"/>
+      <c r="G10" s="104"/>
+      <c r="H10" s="104"/>
       <c r="I10" s="55"/>
     </row>
     <row r="11" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A11" s="120">
+      <c r="A11" s="105">
         <v>46204</v>
       </c>
-      <c r="B11" s="120"/>
-      <c r="C11" s="121" t="s">
+      <c r="B11" s="105"/>
+      <c r="C11" s="106" t="s">
         <v>229</v>
       </c>
-      <c r="D11" s="121" t="s">
+      <c r="D11" s="106" t="s">
         <v>239</v>
       </c>
-      <c r="E11" s="123">
-        <v>170</v>
-      </c>
-      <c r="F11" s="119"/>
-      <c r="G11" s="119"/>
-      <c r="H11" s="119"/>
+      <c r="E11" s="108">
+        <v>220</v>
+      </c>
+      <c r="F11" s="104"/>
+      <c r="G11" s="104"/>
+      <c r="H11" s="104"/>
       <c r="I11" s="55"/>
     </row>
     <row r="12" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A12" s="120"/>
-      <c r="B12" s="120"/>
-      <c r="C12" s="121" t="s">
+      <c r="A12" s="105"/>
+      <c r="B12" s="105"/>
+      <c r="C12" s="106" t="s">
         <v>224</v>
       </c>
-      <c r="D12" s="121" t="s">
+      <c r="D12" s="106" t="s">
         <v>225</v>
       </c>
-      <c r="E12" s="123"/>
-      <c r="F12" s="119"/>
-      <c r="G12" s="119"/>
-      <c r="H12" s="119"/>
+      <c r="E12" s="108"/>
+      <c r="F12" s="104"/>
+      <c r="G12" s="104"/>
+      <c r="H12" s="104"/>
       <c r="I12" s="55"/>
     </row>
     <row r="13" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A13" s="120"/>
-      <c r="B13" s="120"/>
-      <c r="C13" s="121" t="s">
+      <c r="A13" s="105"/>
+      <c r="B13" s="105"/>
+      <c r="C13" s="106" t="s">
         <v>231</v>
       </c>
-      <c r="D13" s="121" t="s">
+      <c r="D13" s="106" t="s">
         <v>232</v>
       </c>
-      <c r="E13" s="123"/>
-      <c r="F13" s="119"/>
-      <c r="G13" s="119"/>
-      <c r="H13" s="119"/>
+      <c r="E13" s="108"/>
+      <c r="F13" s="104"/>
+      <c r="G13" s="104"/>
+      <c r="H13" s="104"/>
       <c r="I13" s="55"/>
     </row>
     <row r="14" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A14" s="120"/>
-      <c r="B14" s="120"/>
-      <c r="C14" s="121" t="s">
+      <c r="A14" s="105"/>
+      <c r="B14" s="105"/>
+      <c r="C14" s="106" t="s">
         <v>235</v>
       </c>
-      <c r="D14" s="121" t="s">
+      <c r="D14" s="106" t="s">
         <v>236</v>
       </c>
-      <c r="E14" s="123"/>
-      <c r="F14" s="119"/>
-      <c r="G14" s="119"/>
-      <c r="H14" s="119"/>
+      <c r="E14" s="108"/>
+      <c r="F14" s="104"/>
+      <c r="G14" s="104"/>
+      <c r="H14" s="104"/>
       <c r="I14" s="55">
         <v>15</v>
       </c>
     </row>
     <row r="15" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A15" s="119"/>
-      <c r="B15" s="119"/>
-      <c r="C15" s="119"/>
-      <c r="D15" s="119"/>
-      <c r="E15" s="119"/>
-      <c r="F15" s="119"/>
-      <c r="G15" s="119"/>
-      <c r="H15" s="119"/>
+      <c r="A15" s="104"/>
+      <c r="B15" s="104"/>
+      <c r="C15" s="104"/>
+      <c r="D15" s="104"/>
+      <c r="E15" s="104"/>
+      <c r="F15" s="104"/>
+      <c r="G15" s="104"/>
+      <c r="H15" s="104"/>
       <c r="I15" s="55">
         <v>15</v>
       </c>
     </row>
     <row r="16" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A16" s="127" t="s">
+      <c r="A16" s="112" t="s">
         <v>240</v>
       </c>
-      <c r="B16" s="127"/>
-      <c r="C16" s="128" t="s">
+      <c r="B16" s="112"/>
+      <c r="C16" s="112" t="s">
         <v>241</v>
       </c>
-      <c r="D16" s="119"/>
-      <c r="E16" s="119"/>
-      <c r="F16" s="119"/>
-      <c r="G16" s="119"/>
-      <c r="H16" s="119"/>
+      <c r="D16" s="104"/>
+      <c r="E16" s="104"/>
+      <c r="F16" s="104"/>
+      <c r="G16" s="104"/>
+      <c r="H16" s="104"/>
       <c r="I16" s="55">
         <v>55</v>
       </c>
     </row>
     <row r="17" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A17" s="124" t="s">
+      <c r="A17" s="109" t="s">
         <v>229</v>
       </c>
-      <c r="B17" s="124"/>
-      <c r="C17" s="119">
+      <c r="B17" s="109"/>
+      <c r="C17" s="104">
         <f>SUMIF($C$5:$C$14,$A$17,$E$5:$E$14)</f>
-        <v>170</v>
-      </c>
-      <c r="D17" s="119"/>
-      <c r="E17" s="119"/>
-      <c r="F17" s="119"/>
-      <c r="G17" s="119"/>
-      <c r="H17" s="119"/>
+        <v>220</v>
+      </c>
+      <c r="D17" s="104"/>
+      <c r="E17" s="104"/>
+      <c r="F17" s="104"/>
+      <c r="G17" s="104"/>
+      <c r="H17" s="104"/>
       <c r="I17" s="55">
         <f>SUM(I14:I16)</f>
         <v>85</v>
       </c>
     </row>
     <row r="18" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A18" s="124" t="s">
+      <c r="A18" s="109" t="s">
         <v>193</v>
       </c>
-      <c r="B18" s="124"/>
-      <c r="C18" s="119"/>
-      <c r="D18" s="119"/>
-      <c r="E18" s="119"/>
-      <c r="F18" s="119"/>
-      <c r="G18" s="119"/>
-      <c r="H18" s="119"/>
+      <c r="B18" s="109"/>
+      <c r="C18" s="104"/>
+      <c r="D18" s="104"/>
+      <c r="E18" s="104"/>
+      <c r="F18" s="104"/>
+      <c r="G18" s="104"/>
+      <c r="H18" s="104"/>
       <c r="I18" s="55">
         <f>+SUM(I14:I17)</f>
         <v>170</v>
       </c>
     </row>
     <row r="19" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A19" s="124" t="s">
+      <c r="A19" s="109" t="s">
         <v>242</v>
       </c>
-      <c r="B19" s="124"/>
-      <c r="C19" s="119">
+      <c r="B19" s="109"/>
+      <c r="C19" s="104">
         <f>SUM(C17:C18)</f>
-        <v>170</v>
-      </c>
-      <c r="D19" s="119"/>
-      <c r="E19" s="119"/>
-      <c r="F19" s="119"/>
-      <c r="G19" s="119"/>
-      <c r="H19" s="119"/>
+        <v>220</v>
+      </c>
+      <c r="D19" s="104"/>
+      <c r="E19" s="104"/>
+      <c r="F19" s="104"/>
+      <c r="G19" s="104"/>
+      <c r="H19" s="104"/>
       <c r="I19" s="55"/>
     </row>
     <row r="20" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A20" s="119"/>
-      <c r="B20" s="119"/>
-      <c r="C20" s="119"/>
-      <c r="D20" s="119"/>
-      <c r="E20" s="119"/>
-      <c r="F20" s="119"/>
-      <c r="G20" s="119"/>
-      <c r="H20" s="119"/>
+      <c r="A20" s="104"/>
+      <c r="B20" s="104"/>
+      <c r="C20" s="104"/>
+      <c r="D20" s="104"/>
+      <c r="E20" s="104"/>
+      <c r="F20" s="104"/>
+      <c r="G20" s="104"/>
+      <c r="H20" s="104"/>
       <c r="I20" s="55"/>
     </row>
     <row r="21" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A21" s="119"/>
-      <c r="B21" s="119"/>
-      <c r="C21" s="119"/>
-      <c r="D21" s="119"/>
-      <c r="E21" s="119"/>
-      <c r="F21" s="119"/>
-      <c r="G21" s="119"/>
-      <c r="H21" s="119"/>
+      <c r="A21" s="104"/>
+      <c r="B21" s="104"/>
+      <c r="C21" s="104"/>
+      <c r="D21" s="104"/>
+      <c r="E21" s="104"/>
+      <c r="F21" s="104"/>
+      <c r="G21" s="104"/>
+      <c r="H21" s="104"/>
       <c r="I21" s="55"/>
     </row>
     <row r="22" spans="1:9" x14ac:dyDescent="0.3">
@@ -6275,7 +6251,7 @@
     <tabColor rgb="FF002060"/>
   </sheetPr>
   <dimension ref="A1:K20"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="2.21875" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="29.77734375" bestFit="1" customWidth="1"/>
@@ -6378,7 +6354,7 @@
       </c>
       <c r="I4" s="97">
         <f ca="1">SUM(F4:F6)</f>
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="J4" s="95"/>
       <c r="K4" s="78"/>
@@ -6411,7 +6387,7 @@
       </c>
       <c r="I5" s="99">
         <f ca="1">AVERAGE(F4:F6)</f>
-        <v>34.666666666666664</v>
+        <v>35.333333333333336</v>
       </c>
       <c r="J5" s="93" t="s">
         <v>238</v>
@@ -6436,7 +6412,7 @@
       </c>
       <c r="F6" s="101">
         <f ca="1">TODAY()-D6</f>
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="G6" s="95" t="s">
         <v>219</v>

</xml_diff>